<commit_message>
updated data set with WGI indicator changes
</commit_message>
<xml_diff>
--- a/index_bbg_rating_live.xlsx
+++ b/index_bbg_rating_live.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kaimin Khaw\Desktop\credit-rating-deploy\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kkhaw\Desktop\credit-rating-deploy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D46D2079-43DF-4FCB-AACE-5A9F1063036C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-72" windowWidth="23256" windowHeight="12456" xr2:uid="{2A12413E-A5EC-426E-A187-DE07F52921C3}"/>
+    <workbookView xWindow="22932" yWindow="-72" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
   <sheets>
     <sheet name="hard_code" sheetId="2" r:id="rId1"/>
@@ -38,7 +37,7 @@
     <definedName name="TreeMap">"TreeMap"</definedName>
     <definedName name="Waterfall">"Waterfall"</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -48,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="331">
   <si>
     <t>Turkey</t>
   </si>
@@ -1041,18 +1040,12 @@
   </si>
   <si>
     <t>3700Z US Equity</t>
-  </si>
-  <si>
-    <t>B- *-</t>
-  </si>
-  <si>
-    <t>CCC+ *</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1112,7 +1105,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{400A6006-A23C-4081-912F-5A311C167FBE}"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1132,1537 +1125,1537 @@
   <volType type="realTimeData">
     <main first="bofaddin.rtdserver">
       <tp t="s">
-        <v>#N/A Requesting Data...3725286179</v>
+        <v>#N/A Requesting Data...1495171584</v>
         <stp/>
         <stp>BDP|13719527809048657439</stp>
         <tr r="E3" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3682953405</v>
+        <v>#N/A Requesting Data...2816117322</v>
         <stp/>
         <stp>BDP|12363409739849183621</stp>
         <tr r="G98" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2712097647</v>
+        <v>#N/A Requesting Data...1589674933</v>
         <stp/>
         <stp>BDP|17606584297068117917</stp>
         <tr r="G105" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3457894443</v>
+        <v>#N/A Requesting Data...3948050665</v>
         <stp/>
         <stp>BDP|12825277506793769973</stp>
         <tr r="F22" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3068895775</v>
+        <v>#N/A Requesting Data...2115447891</v>
         <stp/>
         <stp>BDP|13615906068526188051</stp>
         <tr r="G101" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3413904074</v>
+        <v>#N/A Requesting Data...1231332740</v>
         <stp/>
         <stp>BDP|10912677687245148127</stp>
         <tr r="G106" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3955411311</v>
+        <v>#N/A Requesting Data...3964442118</v>
         <stp/>
         <stp>BDP|16221541486007837625</stp>
         <tr r="G58" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3356084695</v>
+        <v>#N/A Requesting Data...3388407610</v>
         <stp/>
         <stp>BDP|14989839765876665645</stp>
         <tr r="C81" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4171965425</v>
+        <v>#N/A Requesting Data...3824768112</v>
         <stp/>
         <stp>BDP|16792452589360294083</stp>
         <tr r="E11" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4230277971</v>
+        <v>#N/A Requesting Data...1763441809</v>
         <stp/>
         <stp>BDP|16409240184993364568</stp>
         <tr r="E54" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3819108035</v>
+        <v>#N/A Requesting Data...4148341142</v>
         <stp/>
         <stp>BDP|12376141866138693768</stp>
         <tr r="C88" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3652992439</v>
+        <v>#N/A Requesting Data...3311461251</v>
         <stp/>
         <stp>BDP|13146963289471890960</stp>
         <tr r="C18" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4288682520</v>
+        <v>#N/A Requesting Data...3394323663</v>
         <stp/>
         <stp>BDP|10167725043130019931</stp>
         <tr r="C110" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4156805597</v>
+        <v>#N/A Requesting Data...2947382196</v>
         <stp/>
         <stp>BDP|10589422899161895655</stp>
         <tr r="G76" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3744503109</v>
+        <v>#N/A Requesting Data...3258021052</v>
         <stp/>
         <stp>BDP|15228795190517586693</stp>
         <tr r="E84" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2832908597</v>
+        <v>#N/A Requesting Data...1609234337</v>
         <stp/>
         <stp>BDP|10096201946458505444</stp>
         <tr r="G97" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4118513039</v>
+        <v>#N/A Requesting Data...2187136403</v>
         <stp/>
         <stp>BDP|18253401034836307331</stp>
         <tr r="F99" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4258004245</v>
+        <v>#N/A Requesting Data...3965951927</v>
         <stp/>
         <stp>BDP|10867273920449518201</stp>
         <tr r="G71" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3427676950</v>
+        <v>#N/A Requesting Data...2420823896</v>
         <stp/>
         <stp>BDP|14811872563886412749</stp>
         <tr r="E114" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4158085797</v>
+        <v>#N/A Requesting Data...3792712175</v>
         <stp/>
         <stp>BDP|15237334583701669483</stp>
         <tr r="C112" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3338174033</v>
+        <v>#N/A Requesting Data...3339809001</v>
         <stp/>
         <stp>BDP|14006145231309322495</stp>
         <tr r="C65" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3481756758</v>
+        <v>#N/A Requesting Data...2866653552</v>
         <stp/>
         <stp>BDP|14761213634019822741</stp>
         <tr r="G2" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2838816535</v>
+        <v>#N/A Requesting Data...2593199478</v>
         <stp/>
         <stp>BDP|15399231330039360601</stp>
         <tr r="E42" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3433343946</v>
+        <v>#N/A Requesting Data...3615282683</v>
         <stp/>
         <stp>BDP|11120752607359953480</stp>
         <tr r="G61" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3404516086</v>
+        <v>#N/A Requesting Data...3497773119</v>
         <stp/>
         <stp>BDP|15939978441203902037</stp>
         <tr r="C26" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3179727328</v>
+        <v>#N/A Requesting Data...3795047610</v>
         <stp/>
         <stp>BDP|18066043829836356791</stp>
         <tr r="G78" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2991644879</v>
+        <v>#N/A Requesting Data...3176072306</v>
         <stp/>
         <stp>BDP|14168806967588813989</stp>
         <tr r="F77" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3848957305</v>
+        <v>#N/A Requesting Data...2180479652</v>
         <stp/>
         <stp>BDP|18397803367339867766</stp>
         <tr r="F101" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3162388050</v>
+        <v>#N/A Requesting Data...1231560785</v>
         <stp/>
         <stp>BDP|15895803206017416271</stp>
         <tr r="C33" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3509667565</v>
+        <v>#N/A Requesting Data...3268214886</v>
         <stp/>
         <stp>BDP|14908732543227691836</stp>
         <tr r="E94" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2932762296</v>
+        <v>#N/A Requesting Data...3973355893</v>
         <stp/>
         <stp>BDP|12957817799052931996</stp>
         <tr r="E120" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3562859702</v>
+        <v>#N/A Requesting Data...3902533854</v>
         <stp/>
         <stp>BDP|16275205432289392600</stp>
         <tr r="E101" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4229732340</v>
+        <v>#N/A Requesting Data...3844535882</v>
         <stp/>
         <stp>BDP|10407655300028223605</stp>
         <tr r="F47" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2846301103</v>
+        <v>#N/A Requesting Data...2963815830</v>
         <stp/>
         <stp>BDP|14031612538318230186</stp>
         <tr r="C136" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3599274546</v>
+        <v>#N/A Requesting Data...4007954854</v>
         <stp/>
         <stp>BDP|13840587393604095357</stp>
         <tr r="G3" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3530860175</v>
+        <v>#N/A Requesting Data...3158666686</v>
         <stp/>
         <stp>BDP|18397555740376217727</stp>
         <tr r="F17" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2921087364</v>
+        <v>#N/A Requesting Data...1607063208</v>
         <stp/>
         <stp>BDP|15886108592084595196</stp>
         <tr r="F19" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3048928160</v>
+        <v>#N/A Requesting Data...3133823169</v>
         <stp/>
         <stp>BDP|12574943311804341655</stp>
         <tr r="C58" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3026999114</v>
+        <v>#N/A Requesting Data...3560689914</v>
         <stp/>
         <stp>BDP|15276164033266227932</stp>
         <tr r="C121" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4180920902</v>
+        <v>#N/A Requesting Data...1389590046</v>
         <stp/>
         <stp>BDP|11413915902765857449</stp>
         <tr r="C135" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3193696555</v>
+        <v>#N/A Requesting Data...3258538480</v>
         <stp/>
         <stp>BDP|10888161880627674738</stp>
         <tr r="G74" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3132223004</v>
+        <v>#N/A Requesting Data...2057699158</v>
         <stp/>
         <stp>BDP|18252264749434830399</stp>
         <tr r="E91" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3052338807</v>
+        <v>#N/A Requesting Data...2477954752</v>
         <stp/>
         <stp>BDP|16230814927561165496</stp>
         <tr r="C25" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3456179868</v>
+        <v>#N/A Requesting Data...4250437320</v>
         <stp/>
         <stp>BDP|11669407615485914850</stp>
         <tr r="E28" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3385745019</v>
+        <v>#N/A Requesting Data...3809152726</v>
         <stp/>
         <stp>BDP|15385895124225473341</stp>
         <tr r="F89" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2955699802</v>
+        <v>#N/A Requesting Data...1277339091</v>
         <stp/>
         <stp>BDP|16215575297831427265</stp>
         <tr r="G19" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3557060868</v>
+        <v>#N/A Requesting Data...2536867880</v>
         <stp/>
         <stp>BDP|15664489079057139842</stp>
         <tr r="C50" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3008927927</v>
+        <v>#N/A Requesting Data...1921269186</v>
         <stp/>
         <stp>BDP|13556466380534139208</stp>
         <tr r="C63" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4131713775</v>
+        <v>#N/A Requesting Data...1820075382</v>
         <stp/>
         <stp>BDP|12426034393664290636</stp>
         <tr r="G70" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3733481827</v>
+        <v>#N/A Requesting Data...1616211561</v>
         <stp/>
         <stp>BDP|11206974657257798316</stp>
         <tr r="G5" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3965306526</v>
+        <v>#N/A Requesting Data...1696468943</v>
         <stp/>
         <stp>BDP|15687672872765725835</stp>
         <tr r="G133" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3821150659</v>
+        <v>#N/A Requesting Data...3592081734</v>
         <stp/>
         <stp>BDP|10646340980557108540</stp>
         <tr r="G83" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3168176976</v>
+        <v>#N/A Requesting Data...3762622912</v>
         <stp/>
         <stp>BDP|13932387258969800286</stp>
         <tr r="G30" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3524214830</v>
+        <v>#N/A Requesting Data...4164585596</v>
         <stp/>
         <stp>BDP|14685689793557045247</stp>
         <tr r="G11" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3846277668</v>
+        <v>#N/A Requesting Data...1870502319</v>
         <stp/>
         <stp>BDP|11792528289940283264</stp>
         <tr r="G39" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4137055508</v>
+        <v>#N/A Requesting Data...3164844209</v>
         <stp/>
         <stp>BDP|14038814629908297802</stp>
         <tr r="E14" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2840905499</v>
+        <v>#N/A Requesting Data...2549516750</v>
         <stp/>
         <stp>BDP|17960836852555549100</stp>
         <tr r="F79" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4045902897</v>
+        <v>#N/A Requesting Data...2217171053</v>
         <stp/>
         <stp>BDP|12258786923690042954</stp>
         <tr r="G82" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3194825029</v>
+        <v>#N/A Requesting Data...1492747077</v>
         <stp/>
         <stp>BDP|11831892951331348329</stp>
         <tr r="C35" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3675099196</v>
+        <v>#N/A Requesting Data...1987474935</v>
         <stp/>
         <stp>BDP|12634554786653062247</stp>
         <tr r="F34" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2749874834</v>
+        <v>#N/A Requesting Data...3211782278</v>
         <stp/>
         <stp>BDP|10304787173197381988</stp>
         <tr r="G53" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4228060172</v>
+        <v>#N/A Requesting Data...4136355566</v>
         <stp/>
         <stp>BDP|15772343051115104818</stp>
         <tr r="C127" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3401512065</v>
+        <v>#N/A Requesting Data...2727339208</v>
         <stp/>
         <stp>BDP|13619322587163510542</stp>
         <tr r="C45" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4229037868</v>
+        <v>#N/A Requesting Data...2408081287</v>
         <stp/>
         <stp>BDP|13709828003397613269</stp>
         <tr r="C54" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3213190128</v>
+        <v>#N/A Requesting Data...3949131276</v>
         <stp/>
         <stp>BDP|11596891797659679653</stp>
         <tr r="C89" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3747731837</v>
+        <v>#N/A Requesting Data...2342232692</v>
         <stp/>
         <stp>BDP|18339290641951108002</stp>
         <tr r="E17" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3199190008</v>
+        <v>#N/A Requesting Data...3357693919</v>
         <stp/>
         <stp>BDP|10418265688390464525</stp>
         <tr r="E18" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4166690228</v>
+        <v>#N/A Requesting Data...1655422539</v>
         <stp/>
         <stp>BDP|14859691791600738447</stp>
         <tr r="F45" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3198938341</v>
+        <v>#N/A Requesting Data...1525360372</v>
         <stp/>
         <stp>BDP|18255708956124343152</stp>
         <tr r="E26" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3847878904</v>
+        <v>#N/A Requesting Data...3909913868</v>
         <stp/>
         <stp>BDP|16855823919014233436</stp>
         <tr r="F30" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4055332729</v>
+        <v>#N/A Requesting Data...4078176081</v>
         <stp/>
         <stp>BDP|12821872971201299383</stp>
         <tr r="G124" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3996472694</v>
+        <v>#N/A Requesting Data...3903012952</v>
         <stp/>
         <stp>BDP|11466185903217969815</stp>
         <tr r="F33" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3998282562</v>
+        <v>#N/A Requesting Data...3186572290</v>
         <stp/>
         <stp>BDP|13711300257260836914</stp>
         <tr r="C102" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3104617039</v>
+        <v>#N/A Requesting Data...3019588603</v>
         <stp/>
         <stp>BDP|11622318103537999967</stp>
         <tr r="F15" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2949691889</v>
+        <v>#N/A Requesting Data...4114757111</v>
         <stp/>
         <stp>BDP|10597445640754361898</stp>
         <tr r="F50" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2908538226</v>
+        <v>#N/A Requesting Data...3762632851</v>
         <stp/>
         <stp>BDP|13987588094432951117</stp>
         <tr r="E127" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3373316217</v>
+        <v>#N/A Requesting Data...2556387781</v>
         <stp/>
         <stp>BDP|11655961067423868102</stp>
         <tr r="G104" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2923077671</v>
+        <v>#N/A Requesting Data...2675205110</v>
         <stp/>
         <stp>BDP|12468839190466923900</stp>
         <tr r="C20" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2878865788</v>
+        <v>#N/A Requesting Data...2355863096</v>
         <stp/>
         <stp>BDP|18411047804853597705</stp>
         <tr r="C67" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3507548304</v>
+        <v>#N/A Requesting Data...3196119112</v>
         <stp/>
         <stp>BDP|18331339124097518219</stp>
         <tr r="F66" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3070708489</v>
+        <v>#N/A Requesting Data...3383986848</v>
         <stp/>
         <stp>BDP|14983531083496973331</stp>
         <tr r="G132" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3841755370</v>
+        <v>#N/A Requesting Data...2779977571</v>
         <stp/>
         <stp>BDP|14115869171127460078</stp>
         <tr r="G37" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3773561698</v>
+        <v>#N/A Requesting Data...3526591944</v>
         <stp/>
         <stp>BDP|16963038037211063893</stp>
         <tr r="C13" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2921364539</v>
+        <v>#N/A Requesting Data...2300757572</v>
         <stp/>
         <stp>BDP|13900268704084418991</stp>
         <tr r="E37" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3781216602</v>
+        <v>#N/A Requesting Data...3608837704</v>
         <stp/>
         <stp>BDP|16311230542528118454</stp>
         <tr r="E9" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4022835905</v>
+        <v>#N/A Requesting Data...3498682125</v>
         <stp/>
         <stp>BDP|12403550728001134908</stp>
         <tr r="G38" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4095257665</v>
+        <v>#N/A Requesting Data...4189086861</v>
         <stp/>
         <stp>BDP|10528694388950747396</stp>
         <tr r="F80" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2911996083</v>
+        <v>#N/A Requesting Data...1575411060</v>
         <stp/>
         <stp>BDP|17962073596443790028</stp>
         <tr r="F23" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3177945602</v>
+        <v>#N/A Requesting Data...1489762608</v>
         <stp/>
         <stp>BDP|11322749828038387103</stp>
         <tr r="E122" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3004059595</v>
+        <v>#N/A Requesting Data...2138552600</v>
         <stp/>
         <stp>BDP|14872467854648029062</stp>
         <tr r="C75" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4008250047</v>
+        <v>#N/A Requesting Data...2858844170</v>
         <stp/>
         <stp>BDP|14951668809329151689</stp>
         <tr r="E56" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3950276684</v>
+        <v>#N/A Requesting Data...3894978481</v>
         <stp/>
         <stp>BDP|14211231849266296941</stp>
         <tr r="G103" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2846194956</v>
+        <v>#N/A Requesting Data...3921690586</v>
         <stp/>
         <stp>BDP|15282935006718574931</stp>
         <tr r="E92" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4031288455</v>
+        <v>#N/A Requesting Data...3129436206</v>
         <stp/>
         <stp>BDP|16389940868391785591</stp>
         <tr r="C120" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3681368272</v>
+        <v>#N/A Requesting Data...2380532310</v>
         <stp/>
         <stp>BDP|10830300668358540045</stp>
         <tr r="C115" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3601819854</v>
+        <v>#N/A Requesting Data...2260120275</v>
         <stp/>
         <stp>BDP|15417892931237679498</stp>
         <tr r="F8" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3655990393</v>
+        <v>#N/A Requesting Data...2490689595</v>
         <stp/>
         <stp>BDP|13776760394691002167</stp>
         <tr r="C4" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4228373890</v>
+        <v>#N/A Requesting Data...1761590865</v>
         <stp/>
         <stp>BDP|12950924085148446689</stp>
         <tr r="E121" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3622564565</v>
+        <v>#N/A Requesting Data...3469795525</v>
         <stp/>
         <stp>BDP|11202744698684518690</stp>
         <tr r="G111" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3263819649</v>
+        <v>#N/A Requesting Data...2509242644</v>
         <stp/>
         <stp>BDP|11005719894013994183</stp>
         <tr r="C3" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3401961555</v>
+        <v>#N/A Requesting Data...2767688116</v>
         <stp/>
         <stp>BDP|17061881470574956177</stp>
         <tr r="C69" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3638399677</v>
+        <v>#N/A Requesting Data...1513761494</v>
         <stp/>
         <stp>BDP|10195299258766033392</stp>
         <tr r="E90" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4211097164</v>
+        <v>#N/A Requesting Data...3450186891</v>
         <stp/>
         <stp>BDP|17559180385128709479</stp>
         <tr r="E15" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3143827041</v>
+        <v>#N/A Requesting Data...1393459358</v>
         <stp/>
         <stp>BDP|10477087317801173223</stp>
         <tr r="F125" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3215141961</v>
+        <v>#N/A Requesting Data...3925964477</v>
         <stp/>
         <stp>BDP|10431478218456128129</stp>
         <tr r="G32" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3438336661</v>
+        <v>#N/A Requesting Data...1424485760</v>
         <stp/>
         <stp>BDP|12817533695869473568</stp>
         <tr r="C82" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2870629886</v>
+        <v>#N/A Requesting Data...3281745538</v>
         <stp/>
         <stp>BDP|16722436137983528090</stp>
         <tr r="F127" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3123224657</v>
+        <v>#N/A Requesting Data...4286777584</v>
         <stp/>
         <stp>BDP|14949322880769358496</stp>
         <tr r="G16" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4289984785</v>
+        <v>#N/A Requesting Data...3684770275</v>
         <stp/>
         <stp>BDP|12620594347341901004</stp>
         <tr r="C76" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3642359522</v>
+        <v>#N/A Requesting Data...2930518243</v>
         <stp/>
         <stp>BDP|12047021516217693612</stp>
         <tr r="E126" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3421087051</v>
+        <v>#N/A Requesting Data...2862492979</v>
         <stp/>
         <stp>BDP|13612225533853005354</stp>
         <tr r="F102" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2822263374</v>
+        <v>#N/A Requesting Data...3299229236</v>
         <stp/>
         <stp>BDP|11536436753390219250</stp>
         <tr r="F129" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4283123396</v>
+        <v>#N/A Requesting Data...4281421307</v>
         <stp/>
         <stp>BDP|12946334758336119017</stp>
         <tr r="E72" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3106853985</v>
+        <v>#N/A Requesting Data...3239463413</v>
         <stp/>
         <stp>BDP|17733998071078953332</stp>
         <tr r="C23" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3201354049</v>
+        <v>#N/A Requesting Data...2632623876</v>
         <stp/>
         <stp>BDP|16362559715466602618</stp>
         <tr r="F68" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3471164248</v>
+        <v>#N/A Requesting Data...2870859491</v>
         <stp/>
         <stp>BDP|16070475881909673177</stp>
         <tr r="E112" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3889888640</v>
+        <v>#N/A Requesting Data...3697045609</v>
         <stp/>
         <stp>BDP|17590878194950224438</stp>
         <tr r="G87" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2941859110</v>
+        <v>#N/A Requesting Data...2348181560</v>
         <stp/>
         <stp>BDP|12427007793358727164</stp>
         <tr r="F100" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3376307111</v>
+        <v>#N/A Requesting Data...2108326371</v>
         <stp/>
         <stp>BDP|15601293270144483737</stp>
         <tr r="G15" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3323663205</v>
+        <v>#N/A Requesting Data...1836296878</v>
         <stp/>
         <stp>BDP|13723200346810339697</stp>
         <tr r="C38" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3517947391</v>
+        <v>#N/A Requesting Data...1939988835</v>
         <stp/>
         <stp>BDP|18086118189074176643</stp>
         <tr r="E88" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4254559982</v>
+        <v>#N/A Requesting Data...2370934574</v>
         <stp/>
         <stp>BDP|15679917748483251829</stp>
         <tr r="E6" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3057082792</v>
+        <v>#N/A Requesting Data...3900089418</v>
         <stp/>
         <stp>BDP|13421293548936861023</stp>
         <tr r="G66" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3434173098</v>
+        <v>#N/A Requesting Data...3027974146</v>
         <stp/>
         <stp>BDP|10594946509929542325</stp>
         <tr r="F5" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2980406535</v>
+        <v>#N/A Requesting Data...2019291772</v>
         <stp/>
         <stp>BDP|10668212108445960480</stp>
         <tr r="G57" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2909310052</v>
+        <v>#N/A Requesting Data...1744790959</v>
         <stp/>
         <stp>BDP|10103273213286136651</stp>
         <tr r="C6" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3130623975</v>
+        <v>#N/A Requesting Data...3769981935</v>
         <stp/>
         <stp>BDP|11259721862376480554</stp>
         <tr r="G69" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2954010115</v>
+        <v>#N/A Requesting Data...3896045412</v>
         <stp/>
         <stp>BDP|14885566279524266176</stp>
         <tr r="E30" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3276651313</v>
+        <v>#N/A Requesting Data...3251710513</v>
         <stp/>
         <stp>BDP|14519079130534129014</stp>
         <tr r="C49" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3196228548</v>
+        <v>#N/A Requesting Data...2951008670</v>
         <stp/>
         <stp>BDP|14873136635550817546</stp>
         <tr r="G130" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2982034160</v>
+        <v>#N/A Requesting Data...1489488722</v>
         <stp/>
         <stp>BDP|16641457892301341972</stp>
         <tr r="F130" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3837481944</v>
+        <v>#N/A Requesting Data...4266612368</v>
         <stp/>
         <stp>BDP|13231746637163726724</stp>
         <tr r="E7" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3370569590</v>
+        <v>#N/A Requesting Data...3307974199</v>
         <stp/>
         <stp>BDP|12945735048800380256</stp>
         <tr r="G118" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3206572543</v>
+        <v>#N/A Requesting Data...3613770822</v>
         <stp/>
         <stp>BDP|11265248170961260631</stp>
         <tr r="E47" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3134937604</v>
+        <v>#N/A Requesting Data...2639703909</v>
         <stp/>
         <stp>BDP|16351851074029385080</stp>
         <tr r="G35" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4075404805</v>
+        <v>#N/A Requesting Data...2242984194</v>
         <stp/>
         <stp>BDP|11944358991052271970</stp>
         <tr r="C103" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2865681934</v>
+        <v>#N/A Requesting Data...2179636281</v>
         <stp/>
         <stp>BDP|18410981990650283866</stp>
         <tr r="C99" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3123475173</v>
+        <v>#N/A Requesting Data...2955423364</v>
         <stp/>
         <stp>BDP|14383773052580838655</stp>
         <tr r="F104" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3938514490</v>
+        <v>#N/A Requesting Data...2032232724</v>
         <stp/>
         <stp>BDP|10871340643964419300</stp>
         <tr r="F95" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3375060653</v>
+        <v>#N/A Requesting Data...2842917741</v>
         <stp/>
         <stp>BDP|14690280185656044816</stp>
         <tr r="C94" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2895315652</v>
+        <v>#N/A Requesting Data...2263919505</v>
         <stp/>
         <stp>BDP|18305693996456795112</stp>
         <tr r="G80" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3929677029</v>
+        <v>#N/A Requesting Data...1406275635</v>
         <stp/>
         <stp>BDP|16273225567973824127</stp>
         <tr r="C79" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2855078856</v>
+        <v>#N/A Requesting Data...2038388235</v>
         <stp/>
         <stp>BDP|13313129291618997350</stp>
         <tr r="C43" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2984840695</v>
+        <v>#N/A Requesting Data...1503687974</v>
         <stp/>
         <stp>BDP|15444947284180871401</stp>
         <tr r="G27" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3562809039</v>
+        <v>#N/A Requesting Data...4012671131</v>
         <stp/>
         <stp>BDP|12935317504846234704</stp>
         <tr r="F98" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3210302191</v>
+        <v>#N/A Requesting Data...3172623705</v>
         <stp/>
         <stp>BDP|13057895365605005829</stp>
         <tr r="C138" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2843516909</v>
+        <v>#N/A Requesting Data...1435766850</v>
         <stp/>
         <stp>BDP|16160321537943284588</stp>
         <tr r="E76" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3734164499</v>
+        <v>#N/A Requesting Data...3705652788</v>
         <stp/>
         <stp>BDP|10621599828921836610</stp>
         <tr r="C12" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3907523536</v>
+        <v>#N/A Requesting Data...1812520809</v>
         <stp/>
         <stp>BDP|14881076967673386157</stp>
         <tr r="F122" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4253262100</v>
+        <v>#N/A Requesting Data...3588218431</v>
         <stp/>
         <stp>BDP|17321553610055816607</stp>
         <tr r="F96" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3120076080</v>
+        <v>#N/A Requesting Data...3574352712</v>
         <stp/>
         <stp>BDP|12793555755147383546</stp>
         <tr r="F42" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3712879135</v>
+        <v>#N/A Requesting Data...2739753116</v>
         <stp/>
         <stp>BDP|10194327202093986081</stp>
         <tr r="F132" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2880478802</v>
+        <v>#N/A Requesting Data...3469862533</v>
         <stp/>
         <stp>BDP|12798194599768683232</stp>
         <tr r="C42" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3245743450</v>
+        <v>#N/A Requesting Data...3135163883</v>
         <stp/>
         <stp>BDP|15675203172551734114</stp>
         <tr r="F12" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3270666737</v>
+        <v>#N/A Requesting Data...4287444738</v>
         <stp/>
         <stp>BDP|17779010845097021465</stp>
         <tr r="G23" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3312346884</v>
+        <v>#N/A Requesting Data...2771165657</v>
         <stp/>
         <stp>BDP|14698661432127374654</stp>
         <tr r="E53" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2895758733</v>
+        <v>#N/A Requesting Data...4141990334</v>
         <stp/>
         <stp>BDP|16055018629402477686</stp>
         <tr r="F18" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3045012400</v>
+        <v>#N/A Requesting Data...2810687208</v>
         <stp/>
         <stp>BDP|14191015466523343124</stp>
         <tr r="G42" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4228672402</v>
+        <v>#N/A Requesting Data...3151381700</v>
         <stp/>
         <stp>BDP|16690545673604064064</stp>
         <tr r="G6" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3059316729</v>
+        <v>#N/A Requesting Data...2247043750</v>
         <stp/>
         <stp>BDP|11057556593645206836</stp>
         <tr r="E116" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3050066149</v>
+        <v>#N/A Requesting Data...3976767860</v>
         <stp/>
         <stp>BDP|14753168038796700174</stp>
         <tr r="E131" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2932403689</v>
+        <v>#N/A Requesting Data...3222202652</v>
         <stp/>
         <stp>BDP|18400936140157917378</stp>
         <tr r="G108" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3818327005</v>
+        <v>#N/A Requesting Data...3268077019</v>
         <stp/>
         <stp>BDP|11308062409311166143</stp>
         <tr r="F138" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3193012347</v>
+        <v>#N/A Requesting Data...3360384624</v>
         <stp/>
         <stp>BDP|14929251921187622207</stp>
         <tr r="G120" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3903693164</v>
+        <v>#N/A Requesting Data...3988636259</v>
         <stp/>
         <stp>BDP|13312546151322475095</stp>
         <tr r="C117" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3203484125</v>
+        <v>#N/A Requesting Data...4235589222</v>
         <stp/>
         <stp>BDP|10370784365528062849</stp>
         <tr r="G51" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3666356861</v>
+        <v>#N/A Requesting Data...3599748916</v>
         <stp/>
         <stp>BDP|17808503947101138629</stp>
         <tr r="F128" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3615320097</v>
+        <v>#N/A Requesting Data...3481422141</v>
         <stp/>
         <stp>BDP|17640270888515662931</stp>
         <tr r="E20" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3697733238</v>
+        <v>#N/A Requesting Data...3995346465</v>
         <stp/>
         <stp>BDP|17853766030844520642</stp>
         <tr r="F65" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3014884871</v>
+        <v>#N/A Requesting Data...1663363588</v>
         <stp/>
         <stp>BDP|17345319339237647129</stp>
         <tr r="C10" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4235321095</v>
+        <v>#N/A Requesting Data...3659404394</v>
         <stp/>
         <stp>BDP|18428163184190295050</stp>
         <tr r="C48" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3037333283</v>
+        <v>#N/A Requesting Data...2800072319</v>
         <stp/>
         <stp>BDP|11469771160883398201</stp>
         <tr r="G20" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3324663258</v>
+        <v>#N/A Requesting Data...2413681687</v>
         <stp/>
         <stp>BDP|12945229628891094206</stp>
         <tr r="F36" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3422889246</v>
+        <v>#N/A Requesting Data...2503065814</v>
         <stp/>
         <stp>BDP|13088969316699575369</stp>
         <tr r="G17" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3540414031</v>
+        <v>#N/A Requesting Data...3938773652</v>
         <stp/>
         <stp>BDP|14386928546318260068</stp>
         <tr r="C78" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3228760504</v>
+        <v>#N/A Requesting Data...2758472340</v>
         <stp/>
         <stp>BDP|16250000632946565269</stp>
         <tr r="F32" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3036431803</v>
+        <v>#N/A Requesting Data...1956804053</v>
         <stp/>
         <stp>BDP|10062445544650347114</stp>
         <tr r="E69" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3547547409</v>
+        <v>#N/A Requesting Data...3333377564</v>
         <stp/>
         <stp>BDP|16445974490524697317</stp>
         <tr r="F140" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3700577988</v>
+        <v>#N/A Requesting Data...1644815191</v>
         <stp/>
         <stp>BDP|18056984346180923430</stp>
         <tr r="F67" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3926017848</v>
+        <v>#N/A Requesting Data...2734520616</v>
         <stp/>
         <stp>BDP|13607419850307697457</stp>
         <tr r="G55" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4033560388</v>
+        <v>#N/A Requesting Data...3228615101</v>
         <stp/>
         <stp>BDP|17151526894293450943</stp>
         <tr r="E34" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2926455923</v>
+        <v>#N/A Requesting Data...3075907650</v>
         <stp/>
         <stp>BDP|14769233272840536059</stp>
         <tr r="F48" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2968772534</v>
+        <v>#N/A Requesting Data...1527097503</v>
         <stp/>
         <stp>BDP|16347078018142331376</stp>
         <tr r="E59" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3550427227</v>
+        <v>#N/A Requesting Data...1992578297</v>
         <stp/>
         <stp>BDP|12157937398585487157</stp>
         <tr r="F69" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3713060286</v>
+        <v>#N/A Requesting Data...2369302478</v>
         <stp/>
         <stp>BDP|10450024654077121490</stp>
         <tr r="G29" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2933098451</v>
+        <v>#N/A Requesting Data...2750464602</v>
         <stp/>
         <stp>BDP|12405274734177384298</stp>
         <tr r="G109" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3263140418</v>
+        <v>#N/A Requesting Data...3343214300</v>
         <stp/>
         <stp>BDP|11693290023110245727</stp>
         <tr r="F93" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3785169457</v>
+        <v>#N/A Requesting Data...4264774414</v>
         <stp/>
         <stp>BDP|16857915317939051104</stp>
         <tr r="E4" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3017541406</v>
+        <v>#N/A Requesting Data...2772463189</v>
         <stp/>
         <stp>BDP|13092630751014311204</stp>
         <tr r="C29" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3201987539</v>
+        <v>#N/A Requesting Data...3435501932</v>
         <stp/>
         <stp>BDP|16560165422091315234</stp>
         <tr r="E74" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4030141395</v>
+        <v>#N/A Requesting Data...2247172129</v>
         <stp/>
         <stp>BDP|15578620992514708823</stp>
         <tr r="C74" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4248275813</v>
+        <v>#N/A Requesting Data...2463455148</v>
         <stp/>
         <stp>BDP|16311826266949112751</stp>
         <tr r="E137" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3753574777</v>
+        <v>#N/A Requesting Data...3477159304</v>
         <stp/>
         <stp>BDP|12423551309476829732</stp>
         <tr r="E29" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3116719107</v>
+        <v>#N/A Requesting Data...3296705775</v>
         <stp/>
         <stp>BDP|15334425393507822980</stp>
         <tr r="C71" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3123680364</v>
+        <v>#N/A Requesting Data...2746949391</v>
         <stp/>
         <stp>BDP|14187404668490888034</stp>
         <tr r="E115" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3227819191</v>
+        <v>#N/A Requesting Data...4113497608</v>
         <stp/>
         <stp>BDP|14038301256494491076</stp>
         <tr r="E12" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3835144933</v>
+        <v>#N/A Requesting Data...3952996650</v>
         <stp/>
         <stp>BDP|12212063840830333025</stp>
         <tr r="E132" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3166696204</v>
+        <v>#N/A Requesting Data...3576363193</v>
         <stp/>
         <stp>BDP|12411228970299104833</stp>
         <tr r="E40" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3746036288</v>
+        <v>#N/A Requesting Data...2230981362</v>
         <stp/>
         <stp>BDP|11324255971734653659</stp>
         <tr r="G93" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4153521855</v>
+        <v>#N/A Requesting Data...3928103727</v>
         <stp/>
         <stp>BDP|15080702944965265524</stp>
         <tr r="E5" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3614652136</v>
+        <v>#N/A Requesting Data...2972644235</v>
         <stp/>
         <stp>BDP|12709330545317601409</stp>
         <tr r="F78" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3978180887</v>
+        <v>#N/A Requesting Data...3093269170</v>
         <stp/>
         <stp>BDP|17558583635766924170</stp>
         <tr r="C139" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3085544851</v>
+        <v>#N/A Requesting Data...3669229457</v>
         <stp/>
         <stp>BDP|14043797868641345244</stp>
         <tr r="G127" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4088637252</v>
+        <v>#N/A Requesting Data...2162443640</v>
         <stp/>
         <stp>BDP|11097146762171726091</stp>
         <tr r="C125" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3490613606</v>
+        <v>#N/A Requesting Data...1852046987</v>
         <stp/>
         <stp>BDP|10083242995488903402</stp>
         <tr r="E22" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3008777124</v>
+        <v>#N/A Requesting Data...2043798815</v>
         <stp/>
         <stp>BDP|14104003677163905777</stp>
         <tr r="G89" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4108355798</v>
+        <v>#N/A Requesting Data...3238101340</v>
         <stp/>
         <stp>BDP|10493155251505330684</stp>
         <tr r="F113" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3188838273</v>
+        <v>#N/A Requesting Data...2960302772</v>
         <stp/>
         <stp>BDP|17307159600861837050</stp>
         <tr r="C28" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3921686605</v>
+        <v>#N/A Requesting Data...3751887325</v>
         <stp/>
         <stp>BDP|11974207352247436657</stp>
         <tr r="G84" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3901123669</v>
+        <v>#N/A Requesting Data...1723636273</v>
         <stp/>
         <stp>BDP|12417029733397010193</stp>
         <tr r="G129" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3338150778</v>
+        <v>#N/A Requesting Data...1955565328</v>
         <stp/>
         <stp>BDP|13696428749777505366</stp>
         <tr r="C128" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3542880533</v>
+        <v>#N/A Requesting Data...2180562666</v>
         <stp/>
         <stp>BDP|10265435339313984301</stp>
         <tr r="F136" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2968521732</v>
+        <v>#N/A Requesting Data...3617746815</v>
         <stp/>
         <stp>BDP|16742662035804692035</stp>
         <tr r="E24" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3362667557</v>
+        <v>#N/A Requesting Data...2122043703</v>
         <stp/>
         <stp>BDP|13311072247345018521</stp>
         <tr r="E129" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3265707827</v>
+        <v>#N/A Requesting Data...3100156071</v>
         <stp/>
         <stp>BDP|14635385909938704819</stp>
         <tr r="E106" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3553615013</v>
+        <v>#N/A Requesting Data...3490727707</v>
         <stp/>
         <stp>BDP|17965266240553639582</stp>
         <tr r="E10" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4104615352</v>
+        <v>#N/A Requesting Data...1558962269</v>
         <stp/>
         <stp>BDP|14559650107303581628</stp>
         <tr r="C72" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3741705306</v>
+        <v>#N/A Requesting Data...3818503785</v>
         <stp/>
         <stp>BDP|12078771150016496119</stp>
         <tr r="G102" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3557676016</v>
+        <v>#N/A Requesting Data...2005550047</v>
         <stp/>
         <stp>BDP|13437131854538783812</stp>
         <tr r="G22" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3562425229</v>
+        <v>#N/A Requesting Data...3289371084</v>
         <stp/>
         <stp>BDP|11816803688615161347</stp>
         <tr r="E51" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3470932676</v>
+        <v>#N/A Requesting Data...2562282826</v>
         <stp/>
         <stp>BDP|11136233214231371414</stp>
         <tr r="G139" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3529235315</v>
+        <v>#N/A Requesting Data...2340916361</v>
         <stp/>
         <stp>BDP|16387121100332435221</stp>
         <tr r="G96" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3950477347</v>
+        <v>#N/A Requesting Data...2392629728</v>
         <stp/>
         <stp>BDP|10044993787394494110</stp>
         <tr r="C113" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3447339292</v>
+        <v>#N/A Requesting Data...4243791307</v>
         <stp/>
         <stp>BDP|16851432539276999316</stp>
         <tr r="E44" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3309805529</v>
+        <v>#N/A Requesting Data...2373095162</v>
         <stp/>
         <stp>BDP|17514330731974993734</stp>
         <tr r="E65" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4162718272</v>
+        <v>#N/A Requesting Data...3016305302</v>
         <stp/>
         <stp>BDP|13397290692205579908</stp>
         <tr r="G128" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3063620381</v>
+        <v>#N/A Requesting Data...1796922134</v>
         <stp/>
         <stp>BDP|11770519860203890508</stp>
         <tr r="F106" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3543897830</v>
+        <v>#N/A Requesting Data...3920643093</v>
         <stp/>
         <stp>BDP|11828615722360397168</stp>
         <tr r="E71" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3741319537</v>
+        <v>#N/A Requesting Data...3918338333</v>
         <stp/>
         <stp>BDP|12429929188915695292</stp>
         <tr r="F109" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3569397650</v>
+        <v>#N/A Requesting Data...2074865065</v>
         <stp/>
         <stp>BDP|14807781952773549162</stp>
         <tr r="G33" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3003305290</v>
+        <v>#N/A Requesting Data...3519152879</v>
         <stp/>
         <stp>BDP|14141528956866623622</stp>
         <tr r="C134" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3568882905</v>
+        <v>#N/A Requesting Data...2505498763</v>
         <stp/>
         <stp>BDP|11925450918217650729</stp>
         <tr r="F86" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3255863311</v>
+        <v>#N/A Requesting Data...2680028096</v>
         <stp/>
         <stp>BDP|10075353521710450506</stp>
         <tr r="C109" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3624501703</v>
+        <v>#N/A Requesting Data...2195318962</v>
         <stp/>
         <stp>BDP|14507687284196916837</stp>
         <tr r="F6" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3543590214</v>
+        <v>#N/A Requesting Data...1682981708</v>
         <stp/>
         <stp>BDP|17592946715913980887</stp>
         <tr r="F7" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4261279443</v>
+        <v>#N/A Requesting Data...2731076426</v>
         <stp/>
         <stp>BDP|12670343566891576248</stp>
         <tr r="G36" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3984502342</v>
+        <v>#N/A Requesting Data...3623477587</v>
         <stp/>
         <stp>BDP|16059776447550017157</stp>
         <tr r="F63" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3928686742</v>
+        <v>#N/A Requesting Data...2825340567</v>
         <stp/>
         <stp>BDP|13709786759646324310</stp>
         <tr r="F46" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3877127740</v>
+        <v>#N/A Requesting Data...2933892585</v>
         <stp/>
         <stp>BDP|17680007951225535344</stp>
         <tr r="C93" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3711272879</v>
+        <v>#N/A Requesting Data...2013527617</v>
         <stp/>
         <stp>BDP|14249466628496635139</stp>
         <tr r="F26" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3871893626</v>
+        <v>#N/A Requesting Data...3331998893</v>
         <stp/>
         <stp>BDP|12616286245214000526</stp>
         <tr r="C114" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4049412807</v>
+        <v>#N/A Requesting Data...3026911059</v>
         <stp/>
         <stp>BDP|13229487552560837780</stp>
         <tr r="E139" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3254877130</v>
+        <v>#N/A Requesting Data...2619053853</v>
         <stp/>
         <stp>BDP|18412208651713792994</stp>
         <tr r="F118" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3533509888</v>
+        <v>#N/A Requesting Data...3119201056</v>
         <stp/>
         <stp>BDP|16919456577607807790</stp>
         <tr r="G56" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3660345855</v>
+        <v>#N/A Requesting Data...4281360410</v>
         <stp/>
         <stp>BDP|14958917677776306912</stp>
         <tr r="E124" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3185383879</v>
+        <v>#N/A Requesting Data...3275679316</v>
         <stp/>
         <stp>BDP|16906362551851442479</stp>
         <tr r="F14" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3074555127</v>
+        <v>#N/A Requesting Data...2865347900</v>
         <stp/>
         <stp>BDP|13303498173634341154</stp>
         <tr r="G72" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3871247137</v>
+        <v>#N/A Requesting Data...3194690039</v>
         <stp/>
         <stp>BDP|11394026073756494578</stp>
         <tr r="F4" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3613497175</v>
+        <v>#N/A Requesting Data...3304635782</v>
         <stp/>
         <stp>BDP|12821707660430898618</stp>
         <tr r="C40" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4216297996</v>
+        <v>#N/A Requesting Data...4282611269</v>
         <stp/>
         <stp>BDP|12207042919767891145</stp>
         <tr r="G131" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3072264173</v>
+        <v>#N/A Requesting Data...2350085671</v>
         <stp/>
         <stp>BDP|17617562141366516571</stp>
         <tr r="F24" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3567364580</v>
+        <v>#N/A Requesting Data...3042758639</v>
         <stp/>
         <stp>BDP|13776066979946925741</stp>
         <tr r="C90" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4205591163</v>
+        <v>#N/A Requesting Data...1752919145</v>
         <stp/>
         <stp>BDP|15429465971742273156</stp>
         <tr r="E67" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4283600386</v>
+        <v>#N/A Requesting Data...2395645628</v>
         <stp/>
         <stp>BDP|13319017160191784122</stp>
         <tr r="E43" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3592699457</v>
+        <v>#N/A Requesting Data...3328682314</v>
         <stp/>
         <stp>BDP|17197570677470339052</stp>
         <tr r="E33" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3203693925</v>
+        <v>#N/A Requesting Data...3038162273</v>
         <stp/>
         <stp>BDP|18198100188843948773</stp>
         <tr r="G60" s="1"/>
@@ -2670,1801 +2663,1801 @@
     </main>
     <main first="bofaddin.rtdserver">
       <tp t="s">
-        <v>#N/A Requesting Data...4127898546</v>
+        <v>#N/A Requesting Data...3501761888</v>
         <stp/>
         <stp>BDP|3930904544763426134</stp>
         <tr r="C55" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3842290632</v>
+        <v>#N/A Requesting Data...2406504416</v>
         <stp/>
         <stp>BDP|7103625188072362707</stp>
         <tr r="E98" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4180741187</v>
+        <v>#N/A Requesting Data...3779059422</v>
         <stp/>
         <stp>BDP|9365312653090978315</stp>
         <tr r="G136" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3252838831</v>
+        <v>#N/A Requesting Data...1688317654</v>
         <stp/>
         <stp>BDP|6412151529379694002</stp>
         <tr r="F110" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3904820845</v>
+        <v>#N/A Requesting Data...4240258683</v>
         <stp/>
         <stp>BDP|6245426297947871034</stp>
         <tr r="C80" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3784667267</v>
+        <v>#N/A Requesting Data...1577038780</v>
         <stp/>
         <stp>BDP|2350385774053258906</stp>
         <tr r="F72" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4031210860</v>
+        <v>#N/A Requesting Data...2404900694</v>
         <stp/>
         <stp>BDP|8530657130876609747</stp>
         <tr r="C44" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3451049161</v>
+        <v>#N/A Requesting Data...3092048773</v>
         <stp/>
         <stp>BDP|7198979431090342164</stp>
         <tr r="E50" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3847847198</v>
+        <v>#N/A Requesting Data...3588542765</v>
         <stp/>
         <stp>BDP|9075300299347332881</stp>
         <tr r="G79" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4108379532</v>
+        <v>#N/A Requesting Data...3432856801</v>
         <stp/>
         <stp>BDP|5029740995104753357</stp>
         <tr r="C111" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4209802416</v>
+        <v>#N/A Requesting Data...3145399215</v>
         <stp/>
         <stp>BDP|8128743572863334748</stp>
         <tr r="C47" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4058431943</v>
+        <v>#N/A Requesting Data...2450659991</v>
         <stp/>
         <stp>BDP|6339719327836450907</stp>
         <tr r="C98" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3453301240</v>
+        <v>#N/A Requesting Data...3851278770</v>
         <stp/>
         <stp>BDP|4200580269163222863</stp>
         <tr r="E25" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4207259834</v>
+        <v>#N/A Requesting Data...3955284567</v>
         <stp/>
         <stp>BDP|5989352249668473659</stp>
         <tr r="G50" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4070439983</v>
+        <v>#N/A Requesting Data...3611675635</v>
         <stp/>
         <stp>BDP|2484433252649720677</stp>
         <tr r="G68" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3307141636</v>
+        <v>#N/A Requesting Data...4280467411</v>
         <stp/>
         <stp>BDP|6249870436562567333</stp>
         <tr r="E49" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3410516563</v>
+        <v>#N/A Requesting Data...2792092074</v>
         <stp/>
         <stp>BDP|9572192910556051262</stp>
         <tr r="E134" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3554983073</v>
+        <v>#N/A Requesting Data...1765898525</v>
         <stp/>
         <stp>BDP|7540551159163224910</stp>
         <tr r="F51" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3286622899</v>
+        <v>#N/A Requesting Data...2375358303</v>
         <stp/>
         <stp>BDP|8451204331587951367</stp>
         <tr r="F52" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3333472376</v>
+        <v>#N/A Requesting Data...4159276883</v>
         <stp/>
         <stp>BDP|3109256470563958869</stp>
         <tr r="C52" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3970546065</v>
+        <v>#N/A Requesting Data...2221748086</v>
         <stp/>
         <stp>BDP|3590543194827878545</stp>
         <tr r="F59" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3359077578</v>
+        <v>#N/A Requesting Data...3706923174</v>
         <stp/>
         <stp>BDP|3009997314886390075</stp>
         <tr r="G100" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3992391523</v>
+        <v>#N/A Requesting Data...3223942964</v>
         <stp/>
         <stp>BDP|4777106988391072114</stp>
         <tr r="F103" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3826034645</v>
+        <v>#N/A Requesting Data...3999999667</v>
         <stp/>
         <stp>BDP|4303401897634933024</stp>
         <tr r="E93" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3762714897</v>
+        <v>#N/A Requesting Data...1660623745</v>
         <stp/>
         <stp>BDP|9055938583773500695</stp>
         <tr r="C34" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4216721832</v>
+        <v>#N/A Requesting Data...2845443282</v>
         <stp/>
         <stp>BDP|1573317174439842142</stp>
         <tr r="E133" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3031560125</v>
+        <v>#N/A Requesting Data...3186334255</v>
         <stp/>
         <stp>BDP|7180318607099335068</stp>
         <tr r="C9" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3886734507</v>
+        <v>#N/A Requesting Data...3850571551</v>
         <stp/>
         <stp>BDP|8371873502449565411</stp>
         <tr r="C62" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3833120609</v>
+        <v>#N/A Requesting Data...3537155778</v>
         <stp/>
         <stp>BDP|9300723062997279226</stp>
         <tr r="C124" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3878945515</v>
+        <v>#N/A Requesting Data...2397279501</v>
         <stp/>
         <stp>BDP|5492561896244379063</stp>
         <tr r="F70" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3970438499</v>
+        <v>#N/A Requesting Data...3088912906</v>
         <stp/>
         <stp>BDP|8460669760190400504</stp>
         <tr r="C27" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3257597727</v>
+        <v>#N/A Requesting Data...4049743230</v>
         <stp/>
         <stp>BDP|7634975275120208406</stp>
         <tr r="C31" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3560651931</v>
+        <v>#N/A Requesting Data...2810145035</v>
         <stp/>
         <stp>BDP|4040591290066838371</stp>
         <tr r="E13" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3375803885</v>
+        <v>#N/A Requesting Data...3977784739</v>
         <stp/>
         <stp>BDP|9247766641156585153</stp>
         <tr r="G94" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4249686850</v>
+        <v>#N/A Requesting Data...4129117296</v>
         <stp/>
         <stp>BDP|7940113982976758589</stp>
         <tr r="E95" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3099330205</v>
+        <v>#N/A Requesting Data...3811391379</v>
         <stp/>
         <stp>BDP|9093620553903200797</stp>
         <tr r="C105" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3796544466</v>
+        <v>#N/A Requesting Data...3568426287</v>
         <stp/>
         <stp>BDP|2405932012622401695</stp>
         <tr r="G77" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3448888983</v>
+        <v>#N/A Requesting Data...4173817192</v>
         <stp/>
         <stp>BDP|9175353808212225665</stp>
         <tr r="C66" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4202761723</v>
+        <v>#N/A Requesting Data...2087476565</v>
         <stp/>
         <stp>BDP|1414608591110891051</stp>
         <tr r="F9" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3454086833</v>
+        <v>#N/A Requesting Data...3282598994</v>
         <stp/>
         <stp>BDP|3649732806419915339</stp>
         <tr r="G14" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3274839784</v>
+        <v>#N/A Requesting Data...2428830740</v>
         <stp/>
         <stp>BDP|7006257261095505888</stp>
         <tr r="F54" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3113639140</v>
+        <v>#N/A Requesting Data...3056141960</v>
         <stp/>
         <stp>BDP|9781989741438009272</stp>
         <tr r="C39" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4186520241</v>
+        <v>#N/A Requesting Data...1845593315</v>
         <stp/>
         <stp>BDP|7532189862547338936</stp>
         <tr r="F58" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3519238674</v>
+        <v>#N/A Requesting Data...3486459641</v>
         <stp/>
         <stp>BDP|4286027170164748985</stp>
         <tr r="G113" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3876870603</v>
+        <v>#N/A Requesting Data...4119482471</v>
         <stp/>
         <stp>BDP|4691882821088256816</stp>
         <tr r="F126" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3737565232</v>
+        <v>#N/A Requesting Data...2604312792</v>
         <stp/>
         <stp>BDP|4974055815239706225</stp>
         <tr r="G110" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3517666935</v>
+        <v>#N/A Requesting Data...2513527340</v>
         <stp/>
         <stp>BDP|5916130291376545539</stp>
         <tr r="F73" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4165964701</v>
+        <v>#N/A Requesting Data...1719373654</v>
         <stp/>
         <stp>BDP|9535646277681935723</stp>
         <tr r="E60" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3722347818</v>
+        <v>#N/A Requesting Data...2945776682</v>
         <stp/>
         <stp>BDP|3472420329653378814</stp>
         <tr r="G4" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3688842606</v>
+        <v>#N/A Requesting Data...3898448080</v>
         <stp/>
         <stp>BDP|9676580711333862054</stp>
         <tr r="E135" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3967179829</v>
+        <v>#N/A Requesting Data...1794034688</v>
         <stp/>
         <stp>BDP|8651287802994649096</stp>
         <tr r="E77" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3269501175</v>
+        <v>#N/A Requesting Data...2082773024</v>
         <stp/>
         <stp>BDP|5552297197720045083</stp>
         <tr r="E118" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3570750541</v>
+        <v>#N/A Requesting Data...3056790281</v>
         <stp/>
         <stp>BDP|6195991527552839107</stp>
         <tr r="C61" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3306456989</v>
+        <v>#N/A Requesting Data...1954440445</v>
         <stp/>
         <stp>BDP|2785537291931900199</stp>
         <tr r="G91" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3583156305</v>
+        <v>#N/A Requesting Data...1834324591</v>
         <stp/>
         <stp>BDP|9875435960971965593</stp>
         <tr r="C11" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3405833854</v>
+        <v>#N/A Requesting Data...3198945456</v>
         <stp/>
         <stp>BDP|5969741853480600831</stp>
         <tr r="E140" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4105749264</v>
+        <v>#N/A Requesting Data...3546470755</v>
         <stp/>
         <stp>BDP|7662972721973338089</stp>
         <tr r="F107" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3799329837</v>
+        <v>#N/A Requesting Data...2774916299</v>
         <stp/>
         <stp>BDP|4282903616430488389</stp>
         <tr r="G9" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3937134252</v>
+        <v>#N/A Requesting Data...3077422606</v>
         <stp/>
         <stp>BDP|6606398548307737925</stp>
         <tr r="C70" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4271188354</v>
+        <v>#N/A Requesting Data...2673642066</v>
         <stp/>
         <stp>BDP|2310021551041423963</stp>
         <tr r="F123" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4012458805</v>
+        <v>#N/A Requesting Data...2942241074</v>
         <stp/>
         <stp>BDP|1666950877162018261</stp>
         <tr r="E87" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3822713064</v>
+        <v>#N/A Requesting Data...2135604687</v>
         <stp/>
         <stp>BDP|6280569068792932854</stp>
         <tr r="C46" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3407332934</v>
+        <v>#N/A Requesting Data...2986120527</v>
         <stp/>
         <stp>BDP|9635152443296662577</stp>
         <tr r="C16" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3470330971</v>
+        <v>#N/A Requesting Data...3748636851</v>
         <stp/>
         <stp>BDP|5935740968278021330</stp>
         <tr r="C96" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3170792825</v>
+        <v>#N/A Requesting Data...2073007319</v>
         <stp/>
         <stp>BDP|8225387168083679130</stp>
         <tr r="E57" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3837280717</v>
+        <v>#N/A Requesting Data...3736224853</v>
         <stp/>
         <stp>BDP|8741792397660502982</stp>
         <tr r="G24" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3994717510</v>
+        <v>#N/A Requesting Data...2792598094</v>
         <stp/>
         <stp>BDP|1988621838892198978</stp>
         <tr r="F82" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4068186572</v>
+        <v>#N/A Requesting Data...1663915535</v>
         <stp/>
         <stp>BDP|5160947801244572083</stp>
         <tr r="C97" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4183491763</v>
+        <v>#N/A Requesting Data...3389100644</v>
         <stp/>
         <stp>BDP|8781684350665372626</stp>
         <tr r="G64" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3755783815</v>
+        <v>#N/A Requesting Data...2630091139</v>
         <stp/>
         <stp>BDP|8866465832365619258</stp>
         <tr r="F120" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3375657336</v>
+        <v>#N/A Requesting Data...2514512430</v>
         <stp/>
         <stp>BDP|1231973558974048121</stp>
         <tr r="E123" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3814085669</v>
+        <v>#N/A Requesting Data...2994528356</v>
         <stp/>
         <stp>BDP|9011959145835954962</stp>
         <tr r="E102" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3461398416</v>
+        <v>#N/A Requesting Data...4207658614</v>
         <stp/>
         <stp>BDP|7048111723254898858</stp>
         <tr r="E70" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3923197273</v>
+        <v>#N/A Requesting Data...3868116129</v>
         <stp/>
         <stp>BDP|7514426398370500271</stp>
         <tr r="F84" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3318970365</v>
+        <v>#N/A Requesting Data...3616245534</v>
         <stp/>
         <stp>BDP|2286847884578687294</stp>
         <tr r="C64" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3509266547</v>
+        <v>#N/A Requesting Data...1930410336</v>
         <stp/>
         <stp>BDP|8581359335587083771</stp>
         <tr r="G40" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3306739498</v>
+        <v>#N/A Requesting Data...3655724587</v>
         <stp/>
         <stp>BDP|9176352611073152053</stp>
         <tr r="G52" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3596775250</v>
+        <v>#N/A Requesting Data...2571450515</v>
         <stp/>
         <stp>BDP|3761613276703138977</stp>
         <tr r="C22" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3338927065</v>
+        <v>#N/A Requesting Data...2709007450</v>
         <stp/>
         <stp>BDP|2402283480247992710</stp>
         <tr r="G65" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4151686791</v>
+        <v>#N/A Requesting Data...1933827057</v>
         <stp/>
         <stp>BDP|2496054182730824314</stp>
         <tr r="F108" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4239333209</v>
+        <v>#N/A Requesting Data...1804109621</v>
         <stp/>
         <stp>BDP|1156198294412416234</stp>
         <tr r="G48" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4278853750</v>
+        <v>#N/A Requesting Data...2653782713</v>
         <stp/>
         <stp>BDP|1935863512592400318</stp>
         <tr r="G99" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3139967666</v>
+        <v>#N/A Requesting Data...2013677964</v>
         <stp/>
         <stp>BDP|1182070188629538920</stp>
         <tr r="F85" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3521672933</v>
+        <v>#N/A Requesting Data...2957313728</v>
         <stp/>
         <stp>BDP|9924697901094165296</stp>
         <tr r="E38" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3270999973</v>
+        <v>#N/A Requesting Data...1827501361</v>
         <stp/>
         <stp>BDP|6412137247758825261</stp>
         <tr r="G10" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4268730341</v>
+        <v>#N/A Requesting Data...2220354440</v>
         <stp/>
         <stp>BDP|6277108296426856136</stp>
         <tr r="G122" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3181423138</v>
+        <v>#N/A Requesting Data...3749230045</v>
         <stp/>
         <stp>BDP|2351176324921816947</stp>
         <tr r="E117" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3778023970</v>
+        <v>#N/A Requesting Data...3963330299</v>
         <stp/>
         <stp>BDP|6406207188846485346</stp>
         <tr r="C37" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3354692407</v>
+        <v>#N/A Requesting Data...4247226656</v>
         <stp/>
         <stp>BDP|8112280367483097628</stp>
         <tr r="F16" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3331956861</v>
+        <v>#N/A Requesting Data...2304512307</v>
         <stp/>
         <stp>BDP|6484624822372932905</stp>
         <tr r="C108" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3596889940</v>
+        <v>#N/A Requesting Data...2148960187</v>
         <stp/>
         <stp>BDP|8605875253514357834</stp>
         <tr r="C116" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4281728520</v>
+        <v>#N/A Requesting Data...2068505088</v>
         <stp/>
         <stp>BDP|2842991807747556512</stp>
         <tr r="E110" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3720153643</v>
+        <v>#N/A Requesting Data...2695235279</v>
         <stp/>
         <stp>BDP|1377759003508711718</stp>
         <tr r="E55" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3124534328</v>
+        <v>#N/A Requesting Data...3579263356</v>
         <stp/>
         <stp>BDP|1711361391887412536</stp>
         <tr r="G47" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3495676791</v>
+        <v>#N/A Requesting Data...2432396723</v>
         <stp/>
         <stp>BDP|4564815655442574234</stp>
         <tr r="F114" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3151696464</v>
+        <v>#N/A Requesting Data...2933267252</v>
         <stp/>
         <stp>BDP|6557751567646791843</stp>
         <tr r="C85" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3598729284</v>
+        <v>#N/A Requesting Data...2764912294</v>
         <stp/>
         <stp>BDP|5018226780961297742</stp>
         <tr r="E138" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3126020400</v>
+        <v>#N/A Requesting Data...2214802789</v>
         <stp/>
         <stp>BDP|7190582290036507495</stp>
         <tr r="E48" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3586563248</v>
+        <v>#N/A Requesting Data...3423739007</v>
         <stp/>
         <stp>BDP|7268732641219205478</stp>
         <tr r="F111" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3254822982</v>
+        <v>#N/A Requesting Data...3027095045</v>
         <stp/>
         <stp>BDP|5085458293997400582</stp>
         <tr r="C30" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4049831472</v>
+        <v>#N/A Requesting Data...3681036704</v>
         <stp/>
         <stp>BDP|2916061605678582044</stp>
         <tr r="E27" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4039965322</v>
+        <v>#N/A Requesting Data...1957405794</v>
         <stp/>
         <stp>BDP|5645196194854205325</stp>
         <tr r="E19" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3321993992</v>
+        <v>#N/A Requesting Data...3883290273</v>
         <stp/>
         <stp>BDP|8929421222763426766</stp>
         <tr r="F112" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3914131707</v>
+        <v>#N/A Requesting Data...2355012901</v>
         <stp/>
         <stp>BDP|2815946348173965667</stp>
         <tr r="C137" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3578521973</v>
+        <v>#N/A Requesting Data...3835484703</v>
         <stp/>
         <stp>BDP|6645611732949919042</stp>
         <tr r="G95" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3197754989</v>
+        <v>#N/A Requesting Data...2044094107</v>
         <stp/>
         <stp>BDP|8744658502964028082</stp>
         <tr r="F139" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3588954652</v>
+        <v>#N/A Requesting Data...3254644198</v>
         <stp/>
         <stp>BDP|4077907452745230782</stp>
         <tr r="C130" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3301593044</v>
+        <v>#N/A Requesting Data...2760630562</v>
         <stp/>
         <stp>BDP|8975856381415089739</stp>
         <tr r="E75" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4118460467</v>
+        <v>#N/A Requesting Data...4198491593</v>
         <stp/>
         <stp>BDP|5738611839292209825</stp>
         <tr r="G107" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4260816938</v>
+        <v>#N/A Requesting Data...3098364358</v>
         <stp/>
         <stp>BDP|4996818111432201578</stp>
         <tr r="G134" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4057816618</v>
+        <v>#N/A Requesting Data...2333962592</v>
         <stp/>
         <stp>BDP|5458032582021895609</stp>
         <tr r="E89" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4039285219</v>
+        <v>#N/A Requesting Data...4160167520</v>
         <stp/>
         <stp>BDP|2612461303954522846</stp>
         <tr r="F21" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3888539752</v>
+        <v>#N/A Requesting Data...2655123782</v>
         <stp/>
         <stp>BDP|5852840000806674187</stp>
         <tr r="F75" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4146592119</v>
+        <v>#N/A Requesting Data...2490959240</v>
         <stp/>
         <stp>BDP|7947641811679527399</stp>
         <tr r="G13" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3271581710</v>
+        <v>#N/A Requesting Data...1898041741</v>
         <stp/>
         <stp>BDP|8407769428857900025</stp>
         <tr r="C132" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4224771703</v>
+        <v>#N/A Requesting Data...2475761758</v>
         <stp/>
         <stp>BDP|1313714864639868399</stp>
         <tr r="F87" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3491507266</v>
+        <v>#N/A Requesting Data...3113568693</v>
         <stp/>
         <stp>BDP|2531298252748844733</stp>
         <tr r="F115" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3500759436</v>
+        <v>#N/A Requesting Data...4112114671</v>
         <stp/>
         <stp>BDP|8965389266391509672</stp>
         <tr r="C41" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3577359430</v>
+        <v>#N/A Requesting Data...3295241036</v>
         <stp/>
         <stp>BDP|9146373380128430189</stp>
         <tr r="F60" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3411625044</v>
+        <v>#N/A Requesting Data...3582805952</v>
         <stp/>
         <stp>BDP|8769626454200391097</stp>
         <tr r="G85" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4232944995</v>
+        <v>#N/A Requesting Data...2128491147</v>
         <stp/>
         <stp>BDP|7701346097304455298</stp>
         <tr r="C73" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4058802486</v>
+        <v>#N/A Requesting Data...4278959883</v>
         <stp/>
         <stp>BDP|1201589979318261083</stp>
         <tr r="G123" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3767409005</v>
+        <v>#N/A Requesting Data...2457250209</v>
         <stp/>
         <stp>BDP|9994425762708075853</stp>
         <tr r="G88" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4248522402</v>
+        <v>#N/A Requesting Data...1755768459</v>
         <stp/>
         <stp>BDP|8238868892513701135</stp>
         <tr r="G137" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4086649094</v>
+        <v>#N/A Requesting Data...2796926154</v>
         <stp/>
         <stp>BDP|3321556007464177923</stp>
         <tr r="E109" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4030633269</v>
+        <v>#N/A Requesting Data...2983545734</v>
         <stp/>
         <stp>BDP|8367368187378355023</stp>
         <tr r="F64" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4281095132</v>
+        <v>#N/A Requesting Data...2674161216</v>
         <stp/>
         <stp>BDP|9054142235387080711</stp>
         <tr r="F11" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3301708265</v>
+        <v>#N/A Requesting Data...3544053887</v>
         <stp/>
         <stp>BDP|4797724273716399932</stp>
         <tr r="C5" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3931855608</v>
+        <v>#N/A Requesting Data...2780472061</v>
         <stp/>
         <stp>BDP|3084971212582403246</stp>
         <tr r="F121" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3800215435</v>
+        <v>#N/A Requesting Data...2476398226</v>
         <stp/>
         <stp>BDP|6948762204713990690</stp>
         <tr r="G90" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4259623538</v>
+        <v>#N/A Requesting Data...3409334277</v>
         <stp/>
         <stp>BDP|1832764578595986067</stp>
         <tr r="G119" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3815674201</v>
+        <v>#N/A Requesting Data...2575453126</v>
         <stp/>
         <stp>BDP|4156639623951685595</stp>
         <tr r="F13" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3873827169</v>
+        <v>#N/A Requesting Data...2414550167</v>
         <stp/>
         <stp>BDP|5919761437851372455</stp>
         <tr r="C2" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4060656627</v>
+        <v>#N/A Requesting Data...4285673479</v>
         <stp/>
         <stp>BDP|1551339666687413790</stp>
         <tr r="F40" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3522410875</v>
+        <v>#N/A Requesting Data...2192691104</v>
         <stp/>
         <stp>BDP|6420437202397070174</stp>
         <tr r="C8" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3309600731</v>
+        <v>#N/A Requesting Data...2497355537</v>
         <stp/>
         <stp>BDP|1708381902825815365</stp>
         <tr r="C101" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4120901966</v>
+        <v>#N/A Requesting Data...3366882330</v>
         <stp/>
         <stp>BDP|4945796250777738578</stp>
         <tr r="G21" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4043520016</v>
+        <v>#N/A Requesting Data...2976197998</v>
         <stp/>
         <stp>BDP|6746841414412327938</stp>
         <tr r="G75" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3321468579</v>
+        <v>#N/A Requesting Data...3834554600</v>
         <stp/>
         <stp>BDP|1709445403856801620</stp>
         <tr r="E85" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3610809965</v>
+        <v>#N/A Requesting Data...2065063537</v>
         <stp/>
         <stp>BDP|9398823419477440265</stp>
         <tr r="G125" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3497111973</v>
+        <v>#N/A Requesting Data...2985714081</v>
         <stp/>
         <stp>BDP|3430878723724827801</stp>
         <tr r="G41" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4287120550</v>
+        <v>#N/A Requesting Data...3420709920</v>
         <stp/>
         <stp>BDP|9698422803149077198</stp>
         <tr r="C100" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3947300423</v>
+        <v>#N/A Requesting Data...2744999247</v>
         <stp/>
         <stp>BDP|2887002514665714363</stp>
         <tr r="G59" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3444783158</v>
+        <v>#N/A Requesting Data...2120113269</v>
         <stp/>
         <stp>BDP|2668814054578766269</stp>
         <tr r="E31" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4167300005</v>
+        <v>#N/A Requesting Data...1905449081</v>
         <stp/>
         <stp>BDP|8894702939828266110</stp>
         <tr r="C7" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3833729951</v>
+        <v>#N/A Requesting Data...4233377268</v>
         <stp/>
         <stp>BDP|3410885660260666884</stp>
         <tr r="E64" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4055058390</v>
+        <v>#N/A Requesting Data...2170971970</v>
         <stp/>
         <stp>BDP|3658713905400418152</stp>
         <tr r="E35" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3291032528</v>
+        <v>#N/A Requesting Data...2916489368</v>
         <stp/>
         <stp>BDP|7570300716478486864</stp>
         <tr r="E32" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3764014497</v>
+        <v>#N/A Requesting Data...2464319888</v>
         <stp/>
         <stp>BDP|7851492951527237434</stp>
         <tr r="E52" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3224285335</v>
+        <v>#N/A Requesting Data...2121810251</v>
         <stp/>
         <stp>BDP|7352242467910007671</stp>
         <tr r="F124" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3257597804</v>
+        <v>#N/A Requesting Data...2897397419</v>
         <stp/>
         <stp>BDP|5657563513753480721</stp>
         <tr r="E80" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4210176999</v>
+        <v>#N/A Requesting Data...2659421956</v>
         <stp/>
         <stp>BDP|5976587264538865878</stp>
         <tr r="E62" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3210072381</v>
+        <v>#N/A Requesting Data...2297748359</v>
         <stp/>
         <stp>BDP|7151318027339523982</stp>
         <tr r="F91" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4277363795</v>
+        <v>#N/A Requesting Data...2820956237</v>
         <stp/>
         <stp>BDP|1896477110772260049</stp>
         <tr r="C91" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3200401212</v>
+        <v>#N/A Requesting Data...2333309695</v>
         <stp/>
         <stp>BDP|4252725967471187287</stp>
         <tr r="F44" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4047209830</v>
+        <v>#N/A Requesting Data...4183333807</v>
         <stp/>
         <stp>BDP|6943451920864586278</stp>
         <tr r="C118" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4167792558</v>
+        <v>#N/A Requesting Data...4216409302</v>
         <stp/>
         <stp>BDP|5838113265174067025</stp>
         <tr r="F39" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3236379718</v>
+        <v>#N/A Requesting Data...3541214316</v>
         <stp/>
         <stp>BDP|3456718228377624745</stp>
         <tr r="E111" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3977568599</v>
+        <v>#N/A Requesting Data...2258615252</v>
         <stp/>
         <stp>BDP|5917425194519245724</stp>
         <tr r="E79" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3212096699</v>
+        <v>#N/A Requesting Data...2497481640</v>
         <stp/>
         <stp>BDP|6787533358407016713</stp>
         <tr r="F135" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3580669539</v>
+        <v>#N/A Requesting Data...3620579220</v>
         <stp/>
         <stp>BDP|5576451913756991076</stp>
         <tr r="E16" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4250405252</v>
+        <v>#N/A Requesting Data...2550137951</v>
         <stp/>
         <stp>BDP|5284390591628042184</stp>
         <tr r="C24" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3783811011</v>
+        <v>#N/A Requesting Data...2312927361</v>
         <stp/>
         <stp>BDP|5412037028917536689</stp>
         <tr r="G115" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3523487621</v>
+        <v>#N/A Requesting Data...3112878656</v>
         <stp/>
         <stp>BDP|8966942938724477029</stp>
         <tr r="C15" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4221371425</v>
+        <v>#N/A Requesting Data...3977912003</v>
         <stp/>
         <stp>BDP|2938144706552859709</stp>
         <tr r="G81" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3793969253</v>
+        <v>#N/A Requesting Data...2236250828</v>
         <stp/>
         <stp>BDP|3632949480676633244</stp>
         <tr r="F31" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4207328227</v>
+        <v>#N/A Requesting Data...3734197764</v>
         <stp/>
         <stp>BDP|3513418606797579639</stp>
         <tr r="F90" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3457938999</v>
+        <v>#N/A Requesting Data...3664172856</v>
         <stp/>
         <stp>BDP|1733520919261908213</stp>
         <tr r="G73" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3238391496</v>
+        <v>#N/A Requesting Data...2908413023</v>
         <stp/>
         <stp>BDP|8368969127023380651</stp>
         <tr r="F28" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3857735224</v>
+        <v>#N/A Requesting Data...3161710385</v>
         <stp/>
         <stp>BDP|7172716621593553717</stp>
         <tr r="F53" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3920348048</v>
+        <v>#N/A Requesting Data...1837425809</v>
         <stp/>
         <stp>BDP|2954250373819174944</stp>
         <tr r="F119" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3879320114</v>
+        <v>#N/A Requesting Data...4277079299</v>
         <stp/>
         <stp>BDP|4728287753511799518</stp>
         <tr r="F3" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3767757742</v>
+        <v>#N/A Requesting Data...2103357315</v>
         <stp/>
         <stp>BDP|6348617969513327227</stp>
         <tr r="E104" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4141627736</v>
+        <v>#N/A Requesting Data...3726125795</v>
         <stp/>
         <stp>BDP|7694099704858685831</stp>
         <tr r="C107" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3608799074</v>
+        <v>#N/A Requesting Data...3379037412</v>
         <stp/>
         <stp>BDP|4106834752526835861</stp>
         <tr r="F55" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4256899566</v>
+        <v>#N/A Requesting Data...4274930654</v>
         <stp/>
         <stp>BDP|7951337561756108354</stp>
         <tr r="G112" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3277127080</v>
+        <v>#N/A Requesting Data...3038955291</v>
         <stp/>
         <stp>BDP|5468867501418549294</stp>
         <tr r="E86" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3455245953</v>
+        <v>#N/A Requesting Data...2009375124</v>
         <stp/>
         <stp>BDP|4546740053823447251</stp>
         <tr r="C32" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3322603277</v>
+        <v>#N/A Requesting Data...3270789562</v>
         <stp/>
         <stp>BDP|7484527599745538990</stp>
         <tr r="F76" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3549434008</v>
+        <v>#N/A Requesting Data...1867790560</v>
         <stp/>
         <stp>BDP|5578475423865159117</stp>
         <tr r="E61" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3232041522</v>
+        <v>#N/A Requesting Data...3871201231</v>
         <stp/>
         <stp>BDP|6158107237024797760</stp>
         <tr r="E45" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3547087796</v>
+        <v>#N/A Requesting Data...2658787723</v>
         <stp/>
         <stp>BDP|4143076943390197735</stp>
         <tr r="F97" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3602483091</v>
+        <v>#N/A Requesting Data...2006854516</v>
         <stp/>
         <stp>BDP|1762196091349932721</stp>
         <tr r="E82" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3615895366</v>
+        <v>#N/A Requesting Data...2760211759</v>
         <stp/>
         <stp>BDP|4189169184528349241</stp>
         <tr r="F137" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4226986208</v>
+        <v>#N/A Requesting Data...4201704560</v>
         <stp/>
         <stp>BDP|9103140635044368872</stp>
         <tr r="F29" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3606526203</v>
+        <v>#N/A Requesting Data...2411173674</v>
         <stp/>
         <stp>BDP|5519603296584718917</stp>
         <tr r="G54" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4190005593</v>
+        <v>#N/A Requesting Data...3399325895</v>
         <stp/>
         <stp>BDP|1156250824766982737</stp>
         <tr r="G44" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3288076673</v>
+        <v>#N/A Requesting Data...2452831534</v>
         <stp/>
         <stp>BDP|6031605254431729496</stp>
         <tr r="G86" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3362180538</v>
+        <v>#N/A Requesting Data...1873186553</v>
         <stp/>
         <stp>BDP|2649489454114394728</stp>
         <tr r="C14" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3301259250</v>
+        <v>#N/A Requesting Data...4180118379</v>
         <stp/>
         <stp>BDP|8999377595616850481</stp>
         <tr r="E108" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3252448476</v>
+        <v>#N/A Requesting Data...3083312594</v>
         <stp/>
         <stp>BDP|8988928209665280487</stp>
         <tr r="F71" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4289226121</v>
+        <v>#N/A Requesting Data...3635684369</v>
         <stp/>
         <stp>BDP|8368023487691952119</stp>
         <tr r="F88" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3652581951</v>
+        <v>#N/A Requesting Data...2094095576</v>
         <stp/>
         <stp>BDP|5199287207907438042</stp>
         <tr r="E66" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3488272324</v>
+        <v>#N/A Requesting Data...4049072242</v>
         <stp/>
         <stp>BDP|7460099446995728631</stp>
         <tr r="F134" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4290001978</v>
+        <v>#N/A Requesting Data...3249684893</v>
         <stp/>
         <stp>BDP|6160638673325976246</stp>
         <tr r="C104" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4221518252</v>
+        <v>#N/A Requesting Data...2785271618</v>
         <stp/>
         <stp>BDP|5660731962530222490</stp>
         <tr r="E128" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3612555265</v>
+        <v>#N/A Requesting Data...3373954882</v>
         <stp/>
         <stp>BDP|3355023726294311595</stp>
         <tr r="G114" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3852470074</v>
+        <v>#N/A Requesting Data...3493777186</v>
         <stp/>
         <stp>BDP|5604474461391860653</stp>
         <tr r="E130" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3613195965</v>
+        <v>#N/A Requesting Data...3583537855</v>
         <stp/>
         <stp>BDP|3542140114402066179</stp>
         <tr r="E78" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4173745152</v>
+        <v>#N/A Requesting Data...3866745018</v>
         <stp/>
         <stp>BDP|2942496252996870592</stp>
         <tr r="G121" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3681963352</v>
+        <v>#N/A Requesting Data...2532239204</v>
         <stp/>
         <stp>BDP|1823820926283534897</stp>
         <tr r="G18" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4117433273</v>
+        <v>#N/A Requesting Data...3083926893</v>
         <stp/>
         <stp>BDP|3716189405712826043</stp>
         <tr r="G92" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3867150879</v>
+        <v>#N/A Requesting Data...2029733841</v>
         <stp/>
         <stp>BDP|3228146609442097080</stp>
         <tr r="C140" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4162006672</v>
+        <v>#N/A Requesting Data...3319725661</v>
         <stp/>
         <stp>BDP|9344147089140006098</stp>
         <tr r="E83" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4198033188</v>
+        <v>#N/A Requesting Data...4032857707</v>
         <stp/>
         <stp>BDP|6993061706081965773</stp>
         <tr r="F81" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3967005976</v>
+        <v>#N/A Requesting Data...2823592321</v>
         <stp/>
         <stp>BDP|6176792116871092198</stp>
         <tr r="C68" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3716185406</v>
+        <v>#N/A Requesting Data...2632669104</v>
         <stp/>
         <stp>BDP|7185432584822399912</stp>
         <tr r="F131" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3828172390</v>
+        <v>#N/A Requesting Data...3360716697</v>
         <stp/>
         <stp>BDP|8280856169194643320</stp>
         <tr r="G49" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3633939730</v>
+        <v>#N/A Requesting Data...2102109281</v>
         <stp/>
         <stp>BDP|9399109618929306123</stp>
         <tr r="F37" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3950836335</v>
+        <v>#N/A Requesting Data...4207414606</v>
         <stp/>
         <stp>BDP|6669663699409638145</stp>
         <tr r="C123" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3871727816</v>
+        <v>#N/A Requesting Data...3851787647</v>
         <stp/>
         <stp>BDP|6175693122901836298</stp>
         <tr r="C36" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3631701761</v>
+        <v>#N/A Requesting Data...2215538981</v>
         <stp/>
         <stp>BDP|8135075327118072391</stp>
         <tr r="C17" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4062418478</v>
+        <v>#N/A Requesting Data...2441916576</v>
         <stp/>
         <stp>BDP|5726291712345411206</stp>
         <tr r="G28" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3832440114</v>
+        <v>#N/A Requesting Data...3616813101</v>
         <stp/>
         <stp>BDP|8698973352783506690</stp>
         <tr r="F25" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3353143826</v>
+        <v>#N/A Requesting Data...3467817127</v>
         <stp/>
         <stp>BDP|5493604681742158862</stp>
         <tr r="G63" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3909962847</v>
+        <v>#N/A Requesting Data...2689147348</v>
         <stp/>
         <stp>BDP|3239104742287612040</stp>
         <tr r="E39" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3694777490</v>
+        <v>#N/A Requesting Data...2996016871</v>
         <stp/>
         <stp>BDP|3381147726641663059</stp>
         <tr r="C122" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3916765599</v>
+        <v>#N/A Requesting Data...4076084125</v>
         <stp/>
         <stp>BDP|6625906764329795167</stp>
         <tr r="F56" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3995517850</v>
+        <v>#N/A Requesting Data...2933197974</v>
         <stp/>
         <stp>BDP|3325218238213801010</stp>
         <tr r="F57" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3906030789</v>
+        <v>#N/A Requesting Data...2376387914</v>
         <stp/>
         <stp>BDP|1313137390988032037</stp>
         <tr r="C83" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3515484328</v>
+        <v>#N/A Requesting Data...3244271648</v>
         <stp/>
         <stp>BDP|3702733300853619616</stp>
         <tr r="G34" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3272410470</v>
+        <v>#N/A Requesting Data...3487322708</v>
         <stp/>
         <stp>BDP|8558611930018338475</stp>
         <tr r="F35" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3912391473</v>
+        <v>#N/A Requesting Data...2696491406</v>
         <stp/>
         <stp>BDP|5387098906493173798</stp>
         <tr r="G62" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4029451677</v>
+        <v>#N/A Requesting Data...3293735453</v>
         <stp/>
         <stp>BDP|1951038018907673608</stp>
         <tr r="C126" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3436255114</v>
+        <v>#N/A Requesting Data...3256683358</v>
         <stp/>
         <stp>BDP|9253802402770546012</stp>
         <tr r="F74" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3938014052</v>
+        <v>#N/A Requesting Data...3441362351</v>
         <stp/>
         <stp>BDP|1884505914021260664</stp>
         <tr r="E96" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4224200212</v>
+        <v>#N/A Requesting Data...2192914588</v>
         <stp/>
         <stp>BDP|3540127028674193608</stp>
         <tr r="F94" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4033814369</v>
+        <v>#N/A Requesting Data...3676422996</v>
         <stp/>
         <stp>BDP|5372375359741187031</stp>
         <tr r="F27" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3961896174</v>
+        <v>#N/A Requesting Data...2741773758</v>
         <stp/>
         <stp>BDP|5121625602631825066</stp>
         <tr r="E81" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3812954628</v>
+        <v>#N/A Requesting Data...4266234109</v>
         <stp/>
         <stp>BDP|5282708515920897138</stp>
         <tr r="F43" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4235694448</v>
+        <v>#N/A Requesting Data...3688250309</v>
         <stp/>
         <stp>BDP|1250299291741371958</stp>
         <tr r="G31" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4287328255</v>
+        <v>#N/A Requesting Data...2419382463</v>
         <stp/>
         <stp>BDP|4253176148933327033</stp>
         <tr r="C133" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4226790259</v>
+        <v>#N/A Requesting Data...3377077765</v>
         <stp/>
         <stp>BDP|9704751602229087502</stp>
         <tr r="F49" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4127607640</v>
+        <v>#N/A Requesting Data...4205856852</v>
         <stp/>
         <stp>BDP|6775233901286469015</stp>
         <tr r="E125" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3681205116</v>
+        <v>#N/A Requesting Data...3469482753</v>
         <stp/>
         <stp>BDP|7918289416910309647</stp>
         <tr r="C56" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3961746484</v>
+        <v>#N/A Requesting Data...2241305872</v>
         <stp/>
         <stp>BDP|3731272815900600241</stp>
         <tr r="C53" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3993170471</v>
+        <v>#N/A Requesting Data...3509419193</v>
         <stp/>
         <stp>BDP|1685459166489439868</stp>
         <tr r="F133" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3988378899</v>
+        <v>#N/A Requesting Data...3788820337</v>
         <stp/>
         <stp>BDP|2506644172580171154</stp>
         <tr r="C119" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3861457355</v>
+        <v>#N/A Requesting Data...2268845963</v>
         <stp/>
         <stp>BDP|1995353227627490580</stp>
         <tr r="E119" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3805516937</v>
+        <v>#N/A Requesting Data...2872664958</v>
         <stp/>
         <stp>BDP|9173868178561206592</stp>
         <tr r="C77" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3977166590</v>
+        <v>#N/A Requesting Data...2292272627</v>
         <stp/>
         <stp>BDP|4008096672221657096</stp>
         <tr r="G43" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4041616888</v>
+        <v>#N/A Requesting Data...3925611815</v>
         <stp/>
         <stp>BDP|5434663182001395869</stp>
         <tr r="E107" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3888035600</v>
+        <v>#N/A Requesting Data...2868357349</v>
         <stp/>
         <stp>BDP|8686279502629263146</stp>
         <tr r="C129" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3734509465</v>
+        <v>#N/A Requesting Data...4077397490</v>
         <stp/>
         <stp>BDP|4576300957588172984</stp>
         <tr r="E63" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3543607500</v>
+        <v>#N/A Requesting Data...2823587102</v>
         <stp/>
         <stp>BDP|7469671678835895086</stp>
         <tr r="E2" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3368146960</v>
+        <v>#N/A Requesting Data...3137102726</v>
         <stp/>
         <stp>BDP|5444751401066968714</stp>
         <tr r="E73" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3700760982</v>
+        <v>#N/A Requesting Data...3731376385</v>
         <stp/>
         <stp>BDP|2824124077350027748</stp>
         <tr r="E136" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4175374604</v>
+        <v>#N/A Requesting Data...3507125160</v>
         <stp/>
         <stp>BDP|3708851985886704699</stp>
         <tr r="C19" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4225769835</v>
+        <v>#N/A Requesting Data...2501617796</v>
         <stp/>
         <stp>BDP|1006071828475585561</stp>
         <tr r="F116" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3712595018</v>
+        <v>#N/A Requesting Data...4205973170</v>
         <stp/>
         <stp>BDP|1086712249007771639</stp>
         <tr r="G26" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3731263641</v>
+        <v>#N/A Requesting Data...3377172863</v>
         <stp/>
         <stp>BDP|6634730869724168016</stp>
         <tr r="E103" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3759336942</v>
+        <v>#N/A Requesting Data...3759347543</v>
         <stp/>
         <stp>BDP|3520366017777816505</stp>
         <tr r="E97" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3576995096</v>
+        <v>#N/A Requesting Data...3229486341</v>
         <stp/>
         <stp>BDP|2995135217932647367</stp>
         <tr r="F105" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4249694710</v>
+        <v>#N/A Requesting Data...3240619502</v>
         <stp/>
         <stp>BDP|3565057922625094707</stp>
         <tr r="G45" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3729335535</v>
+        <v>#N/A Requesting Data...2485406064</v>
         <stp/>
         <stp>BDP|1485569542807651461</stp>
         <tr r="C86" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3986720287</v>
+        <v>#N/A Requesting Data...4070245329</v>
         <stp/>
         <stp>BDP|1159006460850353421</stp>
         <tr r="E46" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4239436412</v>
+        <v>#N/A Requesting Data...2029636777</v>
         <stp/>
         <stp>BDP|5113311422502283510</stp>
         <tr r="C84" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3491292008</v>
+        <v>#N/A Requesting Data...2431026835</v>
         <stp/>
         <stp>BDP|4420649803735408460</stp>
         <tr r="F117" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4248941026</v>
+        <v>#N/A Requesting Data...2986269047</v>
         <stp/>
         <stp>BDP|9873235984695079585</stp>
         <tr r="C60" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3393827043</v>
+        <v>#N/A Requesting Data...2304639060</v>
         <stp/>
         <stp>BDP|4726106605717010168</stp>
         <tr r="G46" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4123398726</v>
+        <v>#N/A Requesting Data...3638953723</v>
         <stp/>
         <stp>BDP|97453184744598227</stp>
         <tr r="G135" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4242454654</v>
+        <v>#N/A Requesting Data...2446730215</v>
         <stp/>
         <stp>BDP|71129432364790944</stp>
         <tr r="E105" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3777799552</v>
+        <v>#N/A Requesting Data...3850761440</v>
         <stp/>
         <stp>BDP|13870968378316918</stp>
         <tr r="F38" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3871524618</v>
+        <v>#N/A Requesting Data...4087556597</v>
         <stp/>
         <stp>BDP|545017254499479967</stp>
         <tr r="E23" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3791904534</v>
+        <v>#N/A Requesting Data...3953828866</v>
         <stp/>
         <stp>BDP|562457211792430265</stp>
         <tr r="G116" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4135389559</v>
+        <v>#N/A Requesting Data...2097389340</v>
         <stp/>
         <stp>BDP|752318736222262646</stp>
         <tr r="F83" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3754575532</v>
+        <v>#N/A Requesting Data...2139279915</v>
         <stp/>
         <stp>BDP|926433161397617222</stp>
         <tr r="F10" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3734385702</v>
+        <v>#N/A Requesting Data...3262787735</v>
         <stp/>
         <stp>BDP|455507803480864317</stp>
         <tr r="C51" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3472130856</v>
+        <v>#N/A Requesting Data...2036073995</v>
         <stp/>
         <stp>BDP|738430784972633891</stp>
         <tr r="F41" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4228669598</v>
+        <v>#N/A Requesting Data...3690480777</v>
         <stp/>
         <stp>BDP|226270545351892196</stp>
         <tr r="F61" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3913506296</v>
+        <v>#N/A Requesting Data...3776176325</v>
         <stp/>
         <stp>BDP|478534605105814154</stp>
         <tr r="G12" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3385159322</v>
+        <v>#N/A Requesting Data...2643541089</v>
         <stp/>
         <stp>BDP|292697057297288557</stp>
         <tr r="C106" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4066966870</v>
+        <v>#N/A Requesting Data...3637702590</v>
         <stp/>
         <stp>BDP|449489448517477649</stp>
         <tr r="E99" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4005186801</v>
+        <v>#N/A Requesting Data...2474426678</v>
         <stp/>
         <stp>BDP|477239144286521179</stp>
         <tr r="G138" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3975008187</v>
+        <v>#N/A Requesting Data...3117274719</v>
         <stp/>
         <stp>BDP|136361134742057301</stp>
         <tr r="C57" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4093815377</v>
+        <v>#N/A Requesting Data...2777001628</v>
         <stp/>
         <stp>BDP|282958180978155995</stp>
         <tr r="C59" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4108855137</v>
+        <v>#N/A Requesting Data...3744046389</v>
         <stp/>
         <stp>BDP|991366924295531418</stp>
         <tr r="F2" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3839129508</v>
+        <v>#N/A Requesting Data...3910948421</v>
         <stp/>
         <stp>BDP|934073235795196633</stp>
         <tr r="F62" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4169186508</v>
+        <v>#N/A Requesting Data...2189727606</v>
         <stp/>
         <stp>BDP|266608211912165570</stp>
         <tr r="E113" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3538560063</v>
+        <v>#N/A Requesting Data...2824800763</v>
         <stp/>
         <stp>BDP|910156400954699593</stp>
         <tr r="G8" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3367151503</v>
+        <v>#N/A Requesting Data...3720428457</v>
         <stp/>
         <stp>BDP|794293317440269040</stp>
         <tr r="E100" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3446056465</v>
+        <v>#N/A Requesting Data...3855826184</v>
         <stp/>
         <stp>BDP|206766873121157269</stp>
         <tr r="E41" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4014435919</v>
+        <v>#N/A Requesting Data...2521406317</v>
         <stp/>
         <stp>BDP|315261912951356153</stp>
         <tr r="E21" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3407353884</v>
+        <v>#N/A Requesting Data...2775329017</v>
         <stp/>
         <stp>BDP|169080827246056602</stp>
         <tr r="G126" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3730968186</v>
+        <v>#N/A Requesting Data...4111998338</v>
         <stp/>
         <stp>BDP|454779781439338455</stp>
         <tr r="E36" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3592463437</v>
+        <v>#N/A Requesting Data...1981506268</v>
         <stp/>
         <stp>BDP|198524097739196711</stp>
         <tr r="F92" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3762459495</v>
+        <v>#N/A Requesting Data...2905238605</v>
         <stp/>
         <stp>BDP|618726407191106421</stp>
         <tr r="C92" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3384044430</v>
+        <v>#N/A Requesting Data...3780438030</v>
         <stp/>
         <stp>BDP|442808307356626303</stp>
         <tr r="F20" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3574600734</v>
+        <v>#N/A Requesting Data...3718889607</v>
         <stp/>
         <stp>BDP|624014897144495064</stp>
         <tr r="G140" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4163819432</v>
+        <v>#N/A Requesting Data...4090741106</v>
         <stp/>
         <stp>BDP|304889655090792147</stp>
         <tr r="E58" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4121885464</v>
+        <v>#N/A Requesting Data...2501750904</v>
         <stp/>
         <stp>BDP|427627592191043219</stp>
         <tr r="C87" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3663877978</v>
+        <v>#N/A Requesting Data...2230173793</v>
         <stp/>
         <stp>BDP|768711067038142524</stp>
         <tr r="G25" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3909845099</v>
+        <v>#N/A Requesting Data...2623161876</v>
         <stp/>
         <stp>BDP|447365482187669383</stp>
         <tr r="C95" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3950218913</v>
+        <v>#N/A Requesting Data...3383014403</v>
         <stp/>
         <stp>BDP|901925773788783965</stp>
         <tr r="G67" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3588455144</v>
+        <v>#N/A Requesting Data...2742034895</v>
         <stp/>
         <stp>BDP|511429594874391764</stp>
         <tr r="G117" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4290112107</v>
+        <v>#N/A Requesting Data...3597773264</v>
         <stp/>
         <stp>BDP|544620567958067604</stp>
         <tr r="C131" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3589662090</v>
+        <v>#N/A Requesting Data...2333718357</v>
         <stp/>
         <stp>BDP|945569483354328027</stp>
         <tr r="C21" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3442120859</v>
+        <v>#N/A Requesting Data...3099950668</v>
         <stp/>
         <stp>BDP|691281527639744142</stp>
         <tr r="E8" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4063788951</v>
+        <v>#N/A Requesting Data...2911352300</v>
         <stp/>
         <stp>BDP|968314719543295935</stp>
         <tr r="E68" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3444406536</v>
+        <v>#N/A Requesting Data...3260874804</v>
         <stp/>
         <stp>BDP|760426044168153386</stp>
         <tr r="G7" s="1"/>
@@ -4770,7 +4763,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FDB3339-948E-458F-BDF3-DE9E0EAF9A7A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E140"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -4836,7 +4829,7 @@
         <v>302</v>
       </c>
       <c r="D4" t="s">
-        <v>288</v>
+        <v>305</v>
       </c>
       <c r="E4" t="s">
         <v>305</v>
@@ -4904,7 +4897,7 @@
         <v>323</v>
       </c>
       <c r="D8" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="E8" t="s">
         <v>295</v>
@@ -4921,7 +4914,7 @@
         <v>297</v>
       </c>
       <c r="D9" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E9" t="s">
         <v>296</v>
@@ -5247,7 +5240,7 @@
         <v>284</v>
       </c>
       <c r="E28" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
@@ -5281,7 +5274,7 @@
         <v>284</v>
       </c>
       <c r="E30" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
@@ -5553,7 +5546,7 @@
         <v>299</v>
       </c>
       <c r="E46" t="s">
-        <v>288</v>
+        <v>306</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
@@ -5819,7 +5812,7 @@
         <v>245</v>
       </c>
       <c r="C62" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="D62" t="s">
         <v>308</v>
@@ -5836,7 +5829,7 @@
         <v>38</v>
       </c>
       <c r="C63" t="s">
-        <v>303</v>
+        <v>283</v>
       </c>
       <c r="D63" t="s">
         <v>284</v>
@@ -5941,7 +5934,7 @@
         <v>315</v>
       </c>
       <c r="D69" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="E69" t="s">
         <v>319</v>
@@ -5972,7 +5965,7 @@
         <v>276</v>
       </c>
       <c r="C71" t="s">
-        <v>287</v>
+        <v>322</v>
       </c>
       <c r="D71" t="s">
         <v>305</v>
@@ -6094,7 +6087,7 @@
         <v>299</v>
       </c>
       <c r="D78" t="s">
-        <v>331</v>
+        <v>286</v>
       </c>
       <c r="E78" t="s">
         <v>299</v>
@@ -6403,7 +6396,7 @@
         <v>295</v>
       </c>
       <c r="E96" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.3">
@@ -6468,7 +6461,7 @@
         <v>323</v>
       </c>
       <c r="D100" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E100" t="s">
         <v>294</v>
@@ -6655,7 +6648,7 @@
         <v>302</v>
       </c>
       <c r="D111" t="s">
-        <v>332</v>
+        <v>305</v>
       </c>
       <c r="E111" t="s">
         <v>299</v>
@@ -6998,7 +6991,7 @@
         <v>320</v>
       </c>
       <c r="E131" t="s">
-        <v>321</v>
+        <v>288</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.3">
@@ -7080,7 +7073,7 @@
         <v>283</v>
       </c>
       <c r="D136" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="E136" t="s">
         <v>284</v>
@@ -7131,10 +7124,10 @@
         <v>322</v>
       </c>
       <c r="D139" t="s">
-        <v>320</v>
+        <v>305</v>
       </c>
       <c r="E139" t="s">
-        <v>321</v>
+        <v>286</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.3">
@@ -7160,7 +7153,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5352835-5CFD-46EC-8CDA-5672A55A22F5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G140"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7266,7 +7259,7 @@
       </c>
       <c r="F4" t="str">
         <f>_xll.BDP(D4,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>CCC</v>
+        <v>CCC+</v>
       </c>
       <c r="G4" t="str">
         <f>_xll.BDP(D4,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
@@ -7374,7 +7367,7 @@
       </c>
       <c r="F8" t="str">
         <f>_xll.BDP(D8,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>BB+</v>
+        <v>NR</v>
       </c>
       <c r="G8" t="str">
         <f>_xll.BDP(D8,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
@@ -7401,7 +7394,7 @@
       </c>
       <c r="F9" t="str">
         <f>_xll.BDP(D9,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>B+</v>
+        <v>B</v>
       </c>
       <c r="G9" t="str">
         <f>_xll.BDP(D9,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
@@ -7918,7 +7911,7 @@
       </c>
       <c r="G28" t="str">
         <f>_xll.BDP(D28,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
-        <v>BB+</v>
+        <v>BB</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
@@ -7972,7 +7965,7 @@
       </c>
       <c r="G30" t="str">
         <f>_xll.BDP(D30,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
-        <v>BB-</v>
+        <v>BB</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
@@ -8404,7 +8397,7 @@
       </c>
       <c r="G46" t="str">
         <f>_xll.BDP(D46,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
-        <v>CCC</v>
+        <v>CCC-</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
@@ -8828,7 +8821,7 @@
       </c>
       <c r="E62" t="str">
         <f>_xll.BDP(D62,"RTG_MDY_FC_CURR_ISSUER_RATING")</f>
-        <v>Baa3u</v>
+        <v>Baa2u</v>
       </c>
       <c r="F62" t="str">
         <f>_xll.BDP(D62,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
@@ -8855,7 +8848,7 @@
       </c>
       <c r="E63" t="str">
         <f>_xll.BDP(D63,"RTG_MDY_FC_CURR_ISSUER_RATING")</f>
-        <v>B1</v>
+        <v>Ba3</v>
       </c>
       <c r="F63" t="str">
         <f>_xll.BDP(D63,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
@@ -8863,7 +8856,7 @@
       </c>
       <c r="G63" t="str">
         <f>_xll.BDP(D63,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
-        <v>BB-u</v>
+        <v>BB-</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
@@ -9021,7 +9014,7 @@
       </c>
       <c r="F69" t="str">
         <f>_xll.BDP(D69,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>A+</v>
+        <v>AA-</v>
       </c>
       <c r="G69" t="str">
         <f>_xll.BDP(D69,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
@@ -9071,7 +9064,7 @@
       </c>
       <c r="E71" t="str">
         <f>_xll.BDP(D71,"RTG_MDY_FC_CURR_ISSUER_RATING")</f>
-        <v>Caa3</v>
+        <v>Caa2</v>
       </c>
       <c r="F71" t="str">
         <f>_xll.BDP(D71,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
@@ -9754,7 +9747,7 @@
       </c>
       <c r="G96" t="str">
         <f>_xll.BDP(D96,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
-        <v>BB+</v>
+        <v>BBB-</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.3">
@@ -9858,7 +9851,7 @@
       </c>
       <c r="F100" t="str">
         <f>_xll.BDP(D100,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>BB+</v>
+        <v>BBB-</v>
       </c>
       <c r="G100" t="str">
         <f>_xll.BDP(D100,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
@@ -10699,7 +10692,7 @@
       </c>
       <c r="G131" t="str">
         <f>_xll.BDP(D131,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
-        <v>RD</v>
+        <v>CCC</v>
       </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.3">
@@ -10830,7 +10823,7 @@
       </c>
       <c r="F136" t="str">
         <f>_xll.BDP(D136,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>BB-</v>
+        <v>BB</v>
       </c>
       <c r="G136" t="str">
         <f>_xll.BDP(D136,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
@@ -10911,11 +10904,11 @@
       </c>
       <c r="F139" t="str">
         <f>_xll.BDP(D139,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>SD</v>
+        <v>CCC+</v>
       </c>
       <c r="G139" t="str">
         <f>_xll.BDP(D139,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
-        <v>RD</v>
+        <v>B-</v>
       </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
updated raw and transform with 2026 apr weo data
</commit_message>
<xml_diff>
--- a/index_bbg_rating_live.xlsx
+++ b/index_bbg_rating_live.xlsx
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="333">
   <si>
     <t>Turkey</t>
   </si>
@@ -1040,6 +1040,12 @@
   </si>
   <si>
     <t>3700Z US Equity</t>
+  </si>
+  <si>
+    <t>B- *-</t>
+  </si>
+  <si>
+    <t>AA *-</t>
   </si>
 </sst>
 </file>
@@ -1125,1537 +1131,1537 @@
   <volType type="realTimeData">
     <main first="bofaddin.rtdserver">
       <tp t="s">
-        <v>#N/A Requesting Data...1495171584</v>
+        <v>#N/A Requesting Data...4281538805</v>
         <stp/>
         <stp>BDP|13719527809048657439</stp>
         <tr r="E3" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2816117322</v>
+        <v>#N/A Requesting Data...4242699382</v>
         <stp/>
         <stp>BDP|12363409739849183621</stp>
         <tr r="G98" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1589674933</v>
+        <v>#N/A Requesting Data...4223301270</v>
         <stp/>
         <stp>BDP|17606584297068117917</stp>
         <tr r="G105" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3948050665</v>
+        <v>#N/A Requesting Data...4243747063</v>
         <stp/>
         <stp>BDP|12825277506793769973</stp>
         <tr r="F22" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2115447891</v>
+        <v>#N/A Requesting Data...4283279877</v>
         <stp/>
         <stp>BDP|13615906068526188051</stp>
         <tr r="G101" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1231332740</v>
+        <v>#N/A Requesting Data...4282835338</v>
         <stp/>
         <stp>BDP|10912677687245148127</stp>
         <tr r="G106" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3964442118</v>
+        <v>#N/A Requesting Data...4244907434</v>
         <stp/>
         <stp>BDP|16221541486007837625</stp>
         <tr r="G58" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3388407610</v>
+        <v>#N/A Requesting Data...4289212215</v>
         <stp/>
         <stp>BDP|14989839765876665645</stp>
         <tr r="C81" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3824768112</v>
+        <v>#N/A Requesting Data...4289928383</v>
         <stp/>
         <stp>BDP|16792452589360294083</stp>
         <tr r="E11" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1763441809</v>
+        <v>#N/A Requesting Data...4241930810</v>
         <stp/>
         <stp>BDP|16409240184993364568</stp>
         <tr r="E54" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4148341142</v>
+        <v>#N/A Requesting Data...4293600657</v>
         <stp/>
         <stp>BDP|12376141866138693768</stp>
         <tr r="C88" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3311461251</v>
+        <v>#N/A Requesting Data...4266622738</v>
         <stp/>
         <stp>BDP|13146963289471890960</stp>
         <tr r="C18" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3394323663</v>
+        <v>#N/A Requesting Data...4259169197</v>
         <stp/>
         <stp>BDP|10167725043130019931</stp>
         <tr r="C110" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2947382196</v>
+        <v>#N/A Requesting Data...4273819085</v>
         <stp/>
         <stp>BDP|10589422899161895655</stp>
         <tr r="G76" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3258021052</v>
+        <v>#N/A Requesting Data...4267735319</v>
         <stp/>
         <stp>BDP|15228795190517586693</stp>
         <tr r="E84" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1609234337</v>
+        <v>#N/A Requesting Data...4260393429</v>
         <stp/>
         <stp>BDP|10096201946458505444</stp>
         <tr r="G97" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2187136403</v>
+        <v>#N/A Requesting Data...4294805787</v>
         <stp/>
         <stp>BDP|18253401034836307331</stp>
         <tr r="F99" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3965951927</v>
+        <v>#N/A Requesting Data...4265513641</v>
         <stp/>
         <stp>BDP|10867273920449518201</stp>
         <tr r="G71" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2420823896</v>
+        <v>#N/A Requesting Data...4264428759</v>
         <stp/>
         <stp>BDP|14811872563886412749</stp>
         <tr r="E114" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3792712175</v>
+        <v>#N/A Requesting Data...4283156717</v>
         <stp/>
         <stp>BDP|15237334583701669483</stp>
         <tr r="C112" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3339809001</v>
+        <v>#N/A Requesting Data...4270611429</v>
         <stp/>
         <stp>BDP|14006145231309322495</stp>
         <tr r="C65" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2866653552</v>
+        <v>#N/A Requesting Data...4271543903</v>
         <stp/>
         <stp>BDP|14761213634019822741</stp>
         <tr r="G2" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2593199478</v>
+        <v>#N/A Requesting Data...4291679866</v>
         <stp/>
         <stp>BDP|15399231330039360601</stp>
         <tr r="E42" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3615282683</v>
+        <v>#N/A Requesting Data...4278067948</v>
         <stp/>
         <stp>BDP|11120752607359953480</stp>
         <tr r="G61" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3497773119</v>
+        <v>#N/A Requesting Data...4285189688</v>
         <stp/>
         <stp>BDP|15939978441203902037</stp>
         <tr r="C26" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3795047610</v>
+        <v>#N/A Requesting Data...4292634386</v>
         <stp/>
         <stp>BDP|18066043829836356791</stp>
         <tr r="G78" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3176072306</v>
+        <v>#N/A Requesting Data...4294789977</v>
         <stp/>
         <stp>BDP|14168806967588813989</stp>
         <tr r="F77" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2180479652</v>
+        <v>#N/A Requesting Data...4292318761</v>
         <stp/>
         <stp>BDP|18397803367339867766</stp>
         <tr r="F101" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1231560785</v>
+        <v>#N/A Requesting Data...4286674282</v>
         <stp/>
         <stp>BDP|15895803206017416271</stp>
         <tr r="C33" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3268214886</v>
+        <v>#N/A Requesting Data...4292689074</v>
         <stp/>
         <stp>BDP|14908732543227691836</stp>
         <tr r="E94" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3973355893</v>
+        <v>#N/A Requesting Data...4289650716</v>
         <stp/>
         <stp>BDP|12957817799052931996</stp>
         <tr r="E120" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3902533854</v>
+        <v>#N/A Requesting Data...4286903926</v>
         <stp/>
         <stp>BDP|16275205432289392600</stp>
         <tr r="E101" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3844535882</v>
+        <v>#N/A Requesting Data...4288341068</v>
         <stp/>
         <stp>BDP|10407655300028223605</stp>
         <tr r="F47" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2963815830</v>
+        <v>#N/A Requesting Data...4289182940</v>
         <stp/>
         <stp>BDP|14031612538318230186</stp>
         <tr r="C136" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4007954854</v>
+        <v>#N/A Requesting Data...4290663879</v>
         <stp/>
         <stp>BDP|13840587393604095357</stp>
         <tr r="G3" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3158666686</v>
+        <v>#N/A Requesting Data...4293572198</v>
         <stp/>
         <stp>BDP|18397555740376217727</stp>
         <tr r="F17" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1607063208</v>
+        <v>#N/A Requesting Data...4290767945</v>
         <stp/>
         <stp>BDP|15886108592084595196</stp>
         <tr r="F19" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3133823169</v>
+        <v>#N/A Requesting Data...4293067475</v>
         <stp/>
         <stp>BDP|12574943311804341655</stp>
         <tr r="C58" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3560689914</v>
+        <v>#N/A Requesting Data...4293994787</v>
         <stp/>
         <stp>BDP|15276164033266227932</stp>
         <tr r="C121" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1389590046</v>
+        <v>#N/A Requesting Data...4293002775</v>
         <stp/>
         <stp>BDP|11413915902765857449</stp>
         <tr r="C135" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3258538480</v>
+        <v>#N/A Requesting Data...4294791825</v>
         <stp/>
         <stp>BDP|10888161880627674738</stp>
         <tr r="G74" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2057699158</v>
+        <v>#N/A Requesting Data...2506562413</v>
         <stp/>
         <stp>BDP|18252264749434830399</stp>
         <tr r="E91" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2477954752</v>
+        <v>#N/A Requesting Data...3934356438</v>
         <stp/>
         <stp>BDP|16230814927561165496</stp>
         <tr r="C25" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4250437320</v>
+        <v>#N/A Requesting Data...2085942493</v>
         <stp/>
         <stp>BDP|11669407615485914850</stp>
         <tr r="E28" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3809152726</v>
+        <v>#N/A Requesting Data...2234996456</v>
         <stp/>
         <stp>BDP|15385895124225473341</stp>
         <tr r="F89" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1277339091</v>
+        <v>#N/A Requesting Data...2695312321</v>
         <stp/>
         <stp>BDP|16215575297831427265</stp>
         <tr r="G19" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2536867880</v>
+        <v>#N/A Requesting Data...3254501146</v>
         <stp/>
         <stp>BDP|15664489079057139842</stp>
         <tr r="C50" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1921269186</v>
+        <v>#N/A Requesting Data...1979052416</v>
         <stp/>
         <stp>BDP|13556466380534139208</stp>
         <tr r="C63" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1820075382</v>
+        <v>#N/A Requesting Data...315028421</v>
         <stp/>
         <stp>BDP|12426034393664290636</stp>
         <tr r="G70" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1616211561</v>
+        <v>#N/A Requesting Data...3280205165</v>
         <stp/>
         <stp>BDP|11206974657257798316</stp>
         <tr r="G5" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1696468943</v>
+        <v>#N/A Requesting Data...4176285346</v>
         <stp/>
         <stp>BDP|15687672872765725835</stp>
         <tr r="G133" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3592081734</v>
+        <v>#N/A Requesting Data...427713182</v>
         <stp/>
         <stp>BDP|10646340980557108540</stp>
         <tr r="G83" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3762622912</v>
+        <v>#N/A Requesting Data...1084929359</v>
         <stp/>
         <stp>BDP|13932387258969800286</stp>
         <tr r="G30" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4164585596</v>
+        <v>#N/A Requesting Data...3063882440</v>
         <stp/>
         <stp>BDP|14685689793557045247</stp>
         <tr r="G11" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1870502319</v>
+        <v>#N/A Requesting Data...1876683399</v>
         <stp/>
         <stp>BDP|11792528289940283264</stp>
         <tr r="G39" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3164844209</v>
+        <v>#N/A Requesting Data...408436630</v>
         <stp/>
         <stp>BDP|14038814629908297802</stp>
         <tr r="E14" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2549516750</v>
+        <v>#N/A Requesting Data...2653094264</v>
         <stp/>
         <stp>BDP|17960836852555549100</stp>
         <tr r="F79" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2217171053</v>
+        <v>#N/A Requesting Data...438682416</v>
         <stp/>
         <stp>BDP|12258786923690042954</stp>
         <tr r="G82" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1492747077</v>
+        <v>#N/A Requesting Data...56462515</v>
         <stp/>
         <stp>BDP|11831892951331348329</stp>
         <tr r="C35" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1987474935</v>
+        <v>#N/A Requesting Data...3574043701</v>
         <stp/>
         <stp>BDP|12634554786653062247</stp>
         <tr r="F34" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3211782278</v>
+        <v>#N/A Requesting Data...4034418762</v>
         <stp/>
         <stp>BDP|10304787173197381988</stp>
         <tr r="G53" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4136355566</v>
+        <v>#N/A Requesting Data...4289880550</v>
         <stp/>
         <stp>BDP|15772343051115104818</stp>
         <tr r="C127" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2727339208</v>
+        <v>#N/A Requesting Data...299324302</v>
         <stp/>
         <stp>BDP|13619322587163510542</stp>
         <tr r="C45" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2408081287</v>
+        <v>#N/A Requesting Data...2856067250</v>
         <stp/>
         <stp>BDP|13709828003397613269</stp>
         <tr r="C54" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3949131276</v>
+        <v>#N/A Requesting Data...2478454406</v>
         <stp/>
         <stp>BDP|11596891797659679653</stp>
         <tr r="C89" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2342232692</v>
+        <v>#N/A Requesting Data...1412898430</v>
         <stp/>
         <stp>BDP|18339290641951108002</stp>
         <tr r="E17" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3357693919</v>
+        <v>#N/A Requesting Data...160163862</v>
         <stp/>
         <stp>BDP|10418265688390464525</stp>
         <tr r="E18" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1655422539</v>
+        <v>#N/A Requesting Data...1834675267</v>
         <stp/>
         <stp>BDP|14859691791600738447</stp>
         <tr r="F45" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1525360372</v>
+        <v>#N/A Requesting Data...3389868748</v>
         <stp/>
         <stp>BDP|18255708956124343152</stp>
         <tr r="E26" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3909913868</v>
+        <v>#N/A Requesting Data...1365767767</v>
         <stp/>
         <stp>BDP|16855823919014233436</stp>
         <tr r="F30" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4078176081</v>
+        <v>#N/A Requesting Data...422104685</v>
         <stp/>
         <stp>BDP|12821872971201299383</stp>
         <tr r="G124" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3903012952</v>
+        <v>#N/A Requesting Data...2091465056</v>
         <stp/>
         <stp>BDP|11466185903217969815</stp>
         <tr r="F33" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3186572290</v>
+        <v>#N/A Requesting Data...3051475109</v>
         <stp/>
         <stp>BDP|13711300257260836914</stp>
         <tr r="C102" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3019588603</v>
+        <v>#N/A Requesting Data...979650779</v>
         <stp/>
         <stp>BDP|11622318103537999967</stp>
         <tr r="F15" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4114757111</v>
+        <v>#N/A Requesting Data...1710015160</v>
         <stp/>
         <stp>BDP|10597445640754361898</stp>
         <tr r="F50" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3762632851</v>
+        <v>#N/A Requesting Data...2954260565</v>
         <stp/>
         <stp>BDP|13987588094432951117</stp>
         <tr r="E127" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2556387781</v>
+        <v>#N/A Requesting Data...2227858768</v>
         <stp/>
         <stp>BDP|11655961067423868102</stp>
         <tr r="G104" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2675205110</v>
+        <v>#N/A Requesting Data...781535297</v>
         <stp/>
         <stp>BDP|12468839190466923900</stp>
         <tr r="C20" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2355863096</v>
+        <v>#N/A Requesting Data...2894154755</v>
         <stp/>
         <stp>BDP|18411047804853597705</stp>
         <tr r="C67" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3196119112</v>
+        <v>#N/A Requesting Data...3523597466</v>
         <stp/>
         <stp>BDP|18331339124097518219</stp>
         <tr r="F66" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3383986848</v>
+        <v>#N/A Requesting Data...1178573464</v>
         <stp/>
         <stp>BDP|14983531083496973331</stp>
         <tr r="G132" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2779977571</v>
+        <v>#N/A Requesting Data...3188584140</v>
         <stp/>
         <stp>BDP|14115869171127460078</stp>
         <tr r="G37" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3526591944</v>
+        <v>#N/A Requesting Data...2966647750</v>
         <stp/>
         <stp>BDP|16963038037211063893</stp>
         <tr r="C13" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2300757572</v>
+        <v>#N/A Requesting Data...4005866698</v>
         <stp/>
         <stp>BDP|13900268704084418991</stp>
         <tr r="E37" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3608837704</v>
+        <v>#N/A Requesting Data...1186578925</v>
         <stp/>
         <stp>BDP|16311230542528118454</stp>
         <tr r="E9" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3498682125</v>
+        <v>#N/A Requesting Data...4142762822</v>
         <stp/>
         <stp>BDP|12403550728001134908</stp>
         <tr r="G38" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4189086861</v>
+        <v>#N/A Requesting Data...219719260</v>
         <stp/>
         <stp>BDP|10528694388950747396</stp>
         <tr r="F80" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1575411060</v>
+        <v>#N/A Requesting Data...2986645018</v>
         <stp/>
         <stp>BDP|17962073596443790028</stp>
         <tr r="F23" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1489762608</v>
+        <v>#N/A Requesting Data...3297457101</v>
         <stp/>
         <stp>BDP|11322749828038387103</stp>
         <tr r="E122" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2138552600</v>
+        <v>#N/A Requesting Data...2457242402</v>
         <stp/>
         <stp>BDP|14872467854648029062</stp>
         <tr r="C75" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2858844170</v>
+        <v>#N/A Requesting Data...903977434</v>
         <stp/>
         <stp>BDP|14951668809329151689</stp>
         <tr r="E56" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3894978481</v>
+        <v>#N/A Requesting Data...1041824577</v>
         <stp/>
         <stp>BDP|14211231849266296941</stp>
         <tr r="G103" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3921690586</v>
+        <v>#N/A Requesting Data...2852519003</v>
         <stp/>
         <stp>BDP|15282935006718574931</stp>
         <tr r="E92" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3129436206</v>
+        <v>#N/A Requesting Data...2314127336</v>
         <stp/>
         <stp>BDP|16389940868391785591</stp>
         <tr r="C120" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2380532310</v>
+        <v>#N/A Requesting Data...1497348691</v>
         <stp/>
         <stp>BDP|10830300668358540045</stp>
         <tr r="C115" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2260120275</v>
+        <v>#N/A Requesting Data...3217463440</v>
         <stp/>
         <stp>BDP|15417892931237679498</stp>
         <tr r="F8" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2490689595</v>
+        <v>#N/A Requesting Data...4167175547</v>
         <stp/>
         <stp>BDP|13776760394691002167</stp>
         <tr r="C4" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1761590865</v>
+        <v>#N/A Requesting Data...243359572</v>
         <stp/>
         <stp>BDP|12950924085148446689</stp>
         <tr r="E121" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3469795525</v>
+        <v>#N/A Requesting Data...1032303005</v>
         <stp/>
         <stp>BDP|11202744698684518690</stp>
         <tr r="G111" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2509242644</v>
+        <v>#N/A Requesting Data...2813291994</v>
         <stp/>
         <stp>BDP|11005719894013994183</stp>
         <tr r="C3" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2767688116</v>
+        <v>#N/A Requesting Data...3273660796</v>
         <stp/>
         <stp>BDP|17061881470574956177</stp>
         <tr r="C69" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1513761494</v>
+        <v>#N/A Requesting Data...3882177113</v>
         <stp/>
         <stp>BDP|10195299258766033392</stp>
         <tr r="E90" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3450186891</v>
+        <v>#N/A Requesting Data...4065688802</v>
         <stp/>
         <stp>BDP|17559180385128709479</stp>
         <tr r="E15" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1393459358</v>
+        <v>#N/A Requesting Data...3138392778</v>
         <stp/>
         <stp>BDP|10477087317801173223</stp>
         <tr r="F125" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3925964477</v>
+        <v>#N/A Requesting Data...1263795305</v>
         <stp/>
         <stp>BDP|10431478218456128129</stp>
         <tr r="G32" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1424485760</v>
+        <v>#N/A Requesting Data...3754327315</v>
         <stp/>
         <stp>BDP|12817533695869473568</stp>
         <tr r="C82" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3281745538</v>
+        <v>#N/A Requesting Data...668955891</v>
         <stp/>
         <stp>BDP|16722436137983528090</stp>
         <tr r="F127" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4286777584</v>
+        <v>#N/A Requesting Data...2617440960</v>
         <stp/>
         <stp>BDP|14949322880769358496</stp>
         <tr r="G16" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3684770275</v>
+        <v>#N/A Requesting Data...1736864264</v>
         <stp/>
         <stp>BDP|12620594347341901004</stp>
         <tr r="C76" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2930518243</v>
+        <v>#N/A Requesting Data...722782012</v>
         <stp/>
         <stp>BDP|12047021516217693612</stp>
         <tr r="E126" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2862492979</v>
+        <v>#N/A Requesting Data...3179508051</v>
         <stp/>
         <stp>BDP|13612225533853005354</stp>
         <tr r="F102" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3299229236</v>
+        <v>#N/A Requesting Data...300716337</v>
         <stp/>
         <stp>BDP|11536436753390219250</stp>
         <tr r="F129" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4281421307</v>
+        <v>#N/A Requesting Data...3247968499</v>
         <stp/>
         <stp>BDP|12946334758336119017</stp>
         <tr r="E72" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3239463413</v>
+        <v>#N/A Requesting Data...2921657825</v>
         <stp/>
         <stp>BDP|17733998071078953332</stp>
         <tr r="C23" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2632623876</v>
+        <v>#N/A Requesting Data...4280063119</v>
         <stp/>
         <stp>BDP|16362559715466602618</stp>
         <tr r="F68" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2870859491</v>
+        <v>#N/A Requesting Data...2495972136</v>
         <stp/>
         <stp>BDP|16070475881909673177</stp>
         <tr r="E112" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3697045609</v>
+        <v>#N/A Requesting Data...480593425</v>
         <stp/>
         <stp>BDP|17590878194950224438</stp>
         <tr r="G87" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2348181560</v>
+        <v>#N/A Requesting Data...1140799514</v>
         <stp/>
         <stp>BDP|12427007793358727164</stp>
         <tr r="F100" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2108326371</v>
+        <v>#N/A Requesting Data...613996177</v>
         <stp/>
         <stp>BDP|15601293270144483737</stp>
         <tr r="G15" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1836296878</v>
+        <v>#N/A Requesting Data...2053219848</v>
         <stp/>
         <stp>BDP|13723200346810339697</stp>
         <tr r="C38" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1939988835</v>
+        <v>#N/A Requesting Data...627913633</v>
         <stp/>
         <stp>BDP|18086118189074176643</stp>
         <tr r="E88" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2370934574</v>
+        <v>#N/A Requesting Data...3748970072</v>
         <stp/>
         <stp>BDP|15679917748483251829</stp>
         <tr r="E6" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3900089418</v>
+        <v>#N/A Requesting Data...1513483301</v>
         <stp/>
         <stp>BDP|13421293548936861023</stp>
         <tr r="G66" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3027974146</v>
+        <v>#N/A Requesting Data...2781785852</v>
         <stp/>
         <stp>BDP|10594946509929542325</stp>
         <tr r="F5" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2019291772</v>
+        <v>#N/A Requesting Data...2306473804</v>
         <stp/>
         <stp>BDP|10668212108445960480</stp>
         <tr r="G57" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1744790959</v>
+        <v>#N/A Requesting Data...2139949289</v>
         <stp/>
         <stp>BDP|10103273213286136651</stp>
         <tr r="C6" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3769981935</v>
+        <v>#N/A Requesting Data...2503901128</v>
         <stp/>
         <stp>BDP|11259721862376480554</stp>
         <tr r="G69" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3896045412</v>
+        <v>#N/A Requesting Data...1439001086</v>
         <stp/>
         <stp>BDP|14885566279524266176</stp>
         <tr r="E30" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3251710513</v>
+        <v>#N/A Requesting Data...3165351925</v>
         <stp/>
         <stp>BDP|14519079130534129014</stp>
         <tr r="C49" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2951008670</v>
+        <v>#N/A Requesting Data...976798771</v>
         <stp/>
         <stp>BDP|14873136635550817546</stp>
         <tr r="G130" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1489488722</v>
+        <v>#N/A Requesting Data...3375761963</v>
         <stp/>
         <stp>BDP|16641457892301341972</stp>
         <tr r="F130" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4266612368</v>
+        <v>#N/A Requesting Data...873422538</v>
         <stp/>
         <stp>BDP|13231746637163726724</stp>
         <tr r="E7" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3307974199</v>
+        <v>#N/A Requesting Data...924236668</v>
         <stp/>
         <stp>BDP|12945735048800380256</stp>
         <tr r="G118" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3613770822</v>
+        <v>#N/A Requesting Data...2232869679</v>
         <stp/>
         <stp>BDP|11265248170961260631</stp>
         <tr r="E47" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2639703909</v>
+        <v>#N/A Requesting Data...355767762</v>
         <stp/>
         <stp>BDP|16351851074029385080</stp>
         <tr r="G35" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2242984194</v>
+        <v>#N/A Requesting Data...1848109280</v>
         <stp/>
         <stp>BDP|11944358991052271970</stp>
         <tr r="C103" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2179636281</v>
+        <v>#N/A Requesting Data...3501155202</v>
         <stp/>
         <stp>BDP|18410981990650283866</stp>
         <tr r="C99" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2955423364</v>
+        <v>#N/A Requesting Data...401828935</v>
         <stp/>
         <stp>BDP|14383773052580838655</stp>
         <tr r="F104" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2032232724</v>
+        <v>#N/A Requesting Data...2821974899</v>
         <stp/>
         <stp>BDP|10871340643964419300</stp>
         <tr r="F95" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2842917741</v>
+        <v>#N/A Requesting Data...3635348580</v>
         <stp/>
         <stp>BDP|14690280185656044816</stp>
         <tr r="C94" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2263919505</v>
+        <v>#N/A Requesting Data...3519296729</v>
         <stp/>
         <stp>BDP|18305693996456795112</stp>
         <tr r="G80" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1406275635</v>
+        <v>#N/A Requesting Data...2388517896</v>
         <stp/>
         <stp>BDP|16273225567973824127</stp>
         <tr r="C79" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2038388235</v>
+        <v>#N/A Requesting Data...4292377611</v>
         <stp/>
         <stp>BDP|13313129291618997350</stp>
         <tr r="C43" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1503687974</v>
+        <v>#N/A Requesting Data...2368042199</v>
         <stp/>
         <stp>BDP|15444947284180871401</stp>
         <tr r="G27" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4012671131</v>
+        <v>#N/A Requesting Data...1541831443</v>
         <stp/>
         <stp>BDP|12935317504846234704</stp>
         <tr r="F98" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3172623705</v>
+        <v>#N/A Requesting Data...1608344860</v>
         <stp/>
         <stp>BDP|13057895365605005829</stp>
         <tr r="C138" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1435766850</v>
+        <v>#N/A Requesting Data...2532978598</v>
         <stp/>
         <stp>BDP|16160321537943284588</stp>
         <tr r="E76" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3705652788</v>
+        <v>#N/A Requesting Data...2718903413</v>
         <stp/>
         <stp>BDP|10621599828921836610</stp>
         <tr r="C12" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1812520809</v>
+        <v>#N/A Requesting Data...1494994779</v>
         <stp/>
         <stp>BDP|14881076967673386157</stp>
         <tr r="F122" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3588218431</v>
+        <v>#N/A Requesting Data...2325848620</v>
         <stp/>
         <stp>BDP|17321553610055816607</stp>
         <tr r="F96" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3574352712</v>
+        <v>#N/A Requesting Data...4132732032</v>
         <stp/>
         <stp>BDP|12793555755147383546</stp>
         <tr r="F42" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2739753116</v>
+        <v>#N/A Requesting Data...875791330</v>
         <stp/>
         <stp>BDP|10194327202093986081</stp>
         <tr r="F132" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3469862533</v>
+        <v>#N/A Requesting Data...3164846488</v>
         <stp/>
         <stp>BDP|12798194599768683232</stp>
         <tr r="C42" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3135163883</v>
+        <v>#N/A Requesting Data...1976797481</v>
         <stp/>
         <stp>BDP|15675203172551734114</stp>
         <tr r="F12" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4287444738</v>
+        <v>#N/A Requesting Data...459810095</v>
         <stp/>
         <stp>BDP|17779010845097021465</stp>
         <tr r="G23" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2771165657</v>
+        <v>#N/A Requesting Data...3618408954</v>
         <stp/>
         <stp>BDP|14698661432127374654</stp>
         <tr r="E53" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4141990334</v>
+        <v>#N/A Requesting Data...2491506460</v>
         <stp/>
         <stp>BDP|16055018629402477686</stp>
         <tr r="F18" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2810687208</v>
+        <v>#N/A Requesting Data...2476945193</v>
         <stp/>
         <stp>BDP|14191015466523343124</stp>
         <tr r="G42" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3151381700</v>
+        <v>#N/A Requesting Data...3515706798</v>
         <stp/>
         <stp>BDP|16690545673604064064</stp>
         <tr r="G6" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2247043750</v>
+        <v>#N/A Requesting Data...942368492</v>
         <stp/>
         <stp>BDP|11057556593645206836</stp>
         <tr r="E116" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3976767860</v>
+        <v>#N/A Requesting Data...1443171146</v>
         <stp/>
         <stp>BDP|14753168038796700174</stp>
         <tr r="E131" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3222202652</v>
+        <v>#N/A Requesting Data...3240183006</v>
         <stp/>
         <stp>BDP|18400936140157917378</stp>
         <tr r="G108" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3268077019</v>
+        <v>#N/A Requesting Data...410904291</v>
         <stp/>
         <stp>BDP|11308062409311166143</stp>
         <tr r="F138" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3360384624</v>
+        <v>#N/A Requesting Data...2668032502</v>
         <stp/>
         <stp>BDP|14929251921187622207</stp>
         <tr r="G120" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3988636259</v>
+        <v>#N/A Requesting Data...2575722059</v>
         <stp/>
         <stp>BDP|13312546151322475095</stp>
         <tr r="C117" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4235589222</v>
+        <v>#N/A Requesting Data...2155279298</v>
         <stp/>
         <stp>BDP|10370784365528062849</stp>
         <tr r="G51" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3599748916</v>
+        <v>#N/A Requesting Data...1269219249</v>
         <stp/>
         <stp>BDP|17808503947101138629</stp>
         <tr r="F128" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3481422141</v>
+        <v>#N/A Requesting Data...1999760448</v>
         <stp/>
         <stp>BDP|17640270888515662931</stp>
         <tr r="E20" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3995346465</v>
+        <v>#N/A Requesting Data...2641231122</v>
         <stp/>
         <stp>BDP|17853766030844520642</stp>
         <tr r="F65" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1663363588</v>
+        <v>#N/A Requesting Data...2119696437</v>
         <stp/>
         <stp>BDP|17345319339237647129</stp>
         <tr r="C10" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3659404394</v>
+        <v>#N/A Requesting Data...3180933814</v>
         <stp/>
         <stp>BDP|18428163184190295050</stp>
         <tr r="C48" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2800072319</v>
+        <v>#N/A Requesting Data...1087564142</v>
         <stp/>
         <stp>BDP|11469771160883398201</stp>
         <tr r="G20" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2413681687</v>
+        <v>#N/A Requesting Data...1927762788</v>
         <stp/>
         <stp>BDP|12945229628891094206</stp>
         <tr r="F36" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2503065814</v>
+        <v>#N/A Requesting Data...3239947956</v>
         <stp/>
         <stp>BDP|13088969316699575369</stp>
         <tr r="G17" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3938773652</v>
+        <v>#N/A Requesting Data...598327478</v>
         <stp/>
         <stp>BDP|14386928546318260068</stp>
         <tr r="C78" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2758472340</v>
+        <v>#N/A Requesting Data...759352258</v>
         <stp/>
         <stp>BDP|16250000632946565269</stp>
         <tr r="F32" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1956804053</v>
+        <v>#N/A Requesting Data...2330606770</v>
         <stp/>
         <stp>BDP|10062445544650347114</stp>
         <tr r="E69" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3333377564</v>
+        <v>#N/A Requesting Data...2099397601</v>
         <stp/>
         <stp>BDP|16445974490524697317</stp>
         <tr r="F140" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1644815191</v>
+        <v>#N/A Requesting Data...2670499590</v>
         <stp/>
         <stp>BDP|18056984346180923430</stp>
         <tr r="F67" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2734520616</v>
+        <v>#N/A Requesting Data...1388029963</v>
         <stp/>
         <stp>BDP|13607419850307697457</stp>
         <tr r="G55" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3228615101</v>
+        <v>#N/A Requesting Data...3727837507</v>
         <stp/>
         <stp>BDP|17151526894293450943</stp>
         <tr r="E34" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3075907650</v>
+        <v>#N/A Requesting Data...4247745882</v>
         <stp/>
         <stp>BDP|14769233272840536059</stp>
         <tr r="F48" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1527097503</v>
+        <v>#N/A Requesting Data...1845222275</v>
         <stp/>
         <stp>BDP|16347078018142331376</stp>
         <tr r="E59" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1992578297</v>
+        <v>#N/A Requesting Data...3269256939</v>
         <stp/>
         <stp>BDP|12157937398585487157</stp>
         <tr r="F69" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2369302478</v>
+        <v>#N/A Requesting Data...2677249979</v>
         <stp/>
         <stp>BDP|10450024654077121490</stp>
         <tr r="G29" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2750464602</v>
+        <v>#N/A Requesting Data...1726899211</v>
         <stp/>
         <stp>BDP|12405274734177384298</stp>
         <tr r="G109" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3343214300</v>
+        <v>#N/A Requesting Data...1329921153</v>
         <stp/>
         <stp>BDP|11693290023110245727</stp>
         <tr r="F93" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4264774414</v>
+        <v>#N/A Requesting Data...854339115</v>
         <stp/>
         <stp>BDP|16857915317939051104</stp>
         <tr r="E4" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2772463189</v>
+        <v>#N/A Requesting Data...2332188480</v>
         <stp/>
         <stp>BDP|13092630751014311204</stp>
         <tr r="C29" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3435501932</v>
+        <v>#N/A Requesting Data...772345592</v>
         <stp/>
         <stp>BDP|16560165422091315234</stp>
         <tr r="E74" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2247172129</v>
+        <v>#N/A Requesting Data...1104159411</v>
         <stp/>
         <stp>BDP|15578620992514708823</stp>
         <tr r="C74" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2463455148</v>
+        <v>#N/A Requesting Data...3611707592</v>
         <stp/>
         <stp>BDP|16311826266949112751</stp>
         <tr r="E137" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3477159304</v>
+        <v>#N/A Requesting Data...1650928770</v>
         <stp/>
         <stp>BDP|12423551309476829732</stp>
         <tr r="E29" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3296705775</v>
+        <v>#N/A Requesting Data...2509466141</v>
         <stp/>
         <stp>BDP|15334425393507822980</stp>
         <tr r="C71" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2746949391</v>
+        <v>#N/A Requesting Data...4157593917</v>
         <stp/>
         <stp>BDP|14187404668490888034</stp>
         <tr r="E115" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4113497608</v>
+        <v>#N/A Requesting Data...2402065436</v>
         <stp/>
         <stp>BDP|14038301256494491076</stp>
         <tr r="E12" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3952996650</v>
+        <v>#N/A Requesting Data...3731901525</v>
         <stp/>
         <stp>BDP|12212063840830333025</stp>
         <tr r="E132" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3576363193</v>
+        <v>#N/A Requesting Data...2379508885</v>
         <stp/>
         <stp>BDP|12411228970299104833</stp>
         <tr r="E40" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2230981362</v>
+        <v>#N/A Requesting Data...687610854</v>
         <stp/>
         <stp>BDP|11324255971734653659</stp>
         <tr r="G93" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3928103727</v>
+        <v>#N/A Requesting Data...2604241971</v>
         <stp/>
         <stp>BDP|15080702944965265524</stp>
         <tr r="E5" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2972644235</v>
+        <v>#N/A Requesting Data...2313720552</v>
         <stp/>
         <stp>BDP|12709330545317601409</stp>
         <tr r="F78" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3093269170</v>
+        <v>#N/A Requesting Data...2571946984</v>
         <stp/>
         <stp>BDP|17558583635766924170</stp>
         <tr r="C139" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3669229457</v>
+        <v>#N/A Requesting Data...2687247238</v>
         <stp/>
         <stp>BDP|14043797868641345244</stp>
         <tr r="G127" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2162443640</v>
+        <v>#N/A Requesting Data...824601074</v>
         <stp/>
         <stp>BDP|11097146762171726091</stp>
         <tr r="C125" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1852046987</v>
+        <v>#N/A Requesting Data...3786840278</v>
         <stp/>
         <stp>BDP|10083242995488903402</stp>
         <tr r="E22" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2043798815</v>
+        <v>#N/A Requesting Data...662024065</v>
         <stp/>
         <stp>BDP|14104003677163905777</stp>
         <tr r="G89" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3238101340</v>
+        <v>#N/A Requesting Data...1506135412</v>
         <stp/>
         <stp>BDP|10493155251505330684</stp>
         <tr r="F113" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2960302772</v>
+        <v>#N/A Requesting Data...3298459031</v>
         <stp/>
         <stp>BDP|17307159600861837050</stp>
         <tr r="C28" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3751887325</v>
+        <v>#N/A Requesting Data...1840326041</v>
         <stp/>
         <stp>BDP|11974207352247436657</stp>
         <tr r="G84" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1723636273</v>
+        <v>#N/A Requesting Data...470652296</v>
         <stp/>
         <stp>BDP|12417029733397010193</stp>
         <tr r="G129" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1955565328</v>
+        <v>#N/A Requesting Data...3187696211</v>
         <stp/>
         <stp>BDP|13696428749777505366</stp>
         <tr r="C128" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2180562666</v>
+        <v>#N/A Requesting Data...2903772977</v>
         <stp/>
         <stp>BDP|10265435339313984301</stp>
         <tr r="F136" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3617746815</v>
+        <v>#N/A Requesting Data...2883870625</v>
         <stp/>
         <stp>BDP|16742662035804692035</stp>
         <tr r="E24" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2122043703</v>
+        <v>#N/A Requesting Data...2835485463</v>
         <stp/>
         <stp>BDP|13311072247345018521</stp>
         <tr r="E129" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3100156071</v>
+        <v>#N/A Requesting Data...1642508288</v>
         <stp/>
         <stp>BDP|14635385909938704819</stp>
         <tr r="E106" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3490727707</v>
+        <v>#N/A Requesting Data...2400914228</v>
         <stp/>
         <stp>BDP|17965266240553639582</stp>
         <tr r="E10" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1558962269</v>
+        <v>#N/A Requesting Data...2492408394</v>
         <stp/>
         <stp>BDP|14559650107303581628</stp>
         <tr r="C72" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3818503785</v>
+        <v>#N/A Requesting Data...3621123176</v>
         <stp/>
         <stp>BDP|12078771150016496119</stp>
         <tr r="G102" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2005550047</v>
+        <v>#N/A Requesting Data...1991409140</v>
         <stp/>
         <stp>BDP|13437131854538783812</stp>
         <tr r="G22" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3289371084</v>
+        <v>#N/A Requesting Data...4081142123</v>
         <stp/>
         <stp>BDP|11816803688615161347</stp>
         <tr r="E51" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2562282826</v>
+        <v>#N/A Requesting Data...4126194847</v>
         <stp/>
         <stp>BDP|11136233214231371414</stp>
         <tr r="G139" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2340916361</v>
+        <v>#N/A Requesting Data...2978940767</v>
         <stp/>
         <stp>BDP|16387121100332435221</stp>
         <tr r="G96" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2392629728</v>
+        <v>#N/A Requesting Data...3404127902</v>
         <stp/>
         <stp>BDP|10044993787394494110</stp>
         <tr r="C113" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4243791307</v>
+        <v>#N/A Requesting Data...2973637078</v>
         <stp/>
         <stp>BDP|16851432539276999316</stp>
         <tr r="E44" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2373095162</v>
+        <v>#N/A Requesting Data...803621145</v>
         <stp/>
         <stp>BDP|17514330731974993734</stp>
         <tr r="E65" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3016305302</v>
+        <v>#N/A Requesting Data...2358648386</v>
         <stp/>
         <stp>BDP|13397290692205579908</stp>
         <tr r="G128" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1796922134</v>
+        <v>#N/A Requesting Data...3545675663</v>
         <stp/>
         <stp>BDP|11770519860203890508</stp>
         <tr r="F106" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3920643093</v>
+        <v>#N/A Requesting Data...3016117083</v>
         <stp/>
         <stp>BDP|11828615722360397168</stp>
         <tr r="E71" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3918338333</v>
+        <v>#N/A Requesting Data...4248024259</v>
         <stp/>
         <stp>BDP|12429929188915695292</stp>
         <tr r="F109" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2074865065</v>
+        <v>#N/A Requesting Data...2213616416</v>
         <stp/>
         <stp>BDP|14807781952773549162</stp>
         <tr r="G33" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3519152879</v>
+        <v>#N/A Requesting Data...4078705538</v>
         <stp/>
         <stp>BDP|14141528956866623622</stp>
         <tr r="C134" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2505498763</v>
+        <v>#N/A Requesting Data...3206755032</v>
         <stp/>
         <stp>BDP|11925450918217650729</stp>
         <tr r="F86" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2680028096</v>
+        <v>#N/A Requesting Data...1916871612</v>
         <stp/>
         <stp>BDP|10075353521710450506</stp>
         <tr r="C109" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2195318962</v>
+        <v>#N/A Requesting Data...3407952105</v>
         <stp/>
         <stp>BDP|14507687284196916837</stp>
         <tr r="F6" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1682981708</v>
+        <v>#N/A Requesting Data...1960356371</v>
         <stp/>
         <stp>BDP|17592946715913980887</stp>
         <tr r="F7" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2731076426</v>
+        <v>#N/A Requesting Data...983071769</v>
         <stp/>
         <stp>BDP|12670343566891576248</stp>
         <tr r="G36" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3623477587</v>
+        <v>#N/A Requesting Data...2706611284</v>
         <stp/>
         <stp>BDP|16059776447550017157</stp>
         <tr r="F63" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2825340567</v>
+        <v>#N/A Requesting Data...1454986582</v>
         <stp/>
         <stp>BDP|13709786759646324310</stp>
         <tr r="F46" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2933892585</v>
+        <v>#N/A Requesting Data...849074466</v>
         <stp/>
         <stp>BDP|17680007951225535344</stp>
         <tr r="C93" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2013527617</v>
+        <v>#N/A Requesting Data...3125202582</v>
         <stp/>
         <stp>BDP|14249466628496635139</stp>
         <tr r="F26" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3331998893</v>
+        <v>#N/A Requesting Data...2116278067</v>
         <stp/>
         <stp>BDP|12616286245214000526</stp>
         <tr r="C114" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3026911059</v>
+        <v>#N/A Requesting Data...1718762596</v>
         <stp/>
         <stp>BDP|13229487552560837780</stp>
         <tr r="E139" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2619053853</v>
+        <v>#N/A Requesting Data...794669539</v>
         <stp/>
         <stp>BDP|18412208651713792994</stp>
         <tr r="F118" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3119201056</v>
+        <v>#N/A Requesting Data...2659019485</v>
         <stp/>
         <stp>BDP|16919456577607807790</stp>
         <tr r="G56" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4281360410</v>
+        <v>#N/A Requesting Data...1773924770</v>
         <stp/>
         <stp>BDP|14958917677776306912</stp>
         <tr r="E124" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3275679316</v>
+        <v>#N/A Requesting Data...3272172021</v>
         <stp/>
         <stp>BDP|16906362551851442479</stp>
         <tr r="F14" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2865347900</v>
+        <v>#N/A Requesting Data...1634360491</v>
         <stp/>
         <stp>BDP|13303498173634341154</stp>
         <tr r="G72" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3194690039</v>
+        <v>#N/A Requesting Data...4044351873</v>
         <stp/>
         <stp>BDP|11394026073756494578</stp>
         <tr r="F4" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3304635782</v>
+        <v>#N/A Requesting Data...2089610352</v>
         <stp/>
         <stp>BDP|12821707660430898618</stp>
         <tr r="C40" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4282611269</v>
+        <v>#N/A Requesting Data...554502583</v>
         <stp/>
         <stp>BDP|12207042919767891145</stp>
         <tr r="G131" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2350085671</v>
+        <v>#N/A Requesting Data...3936254852</v>
         <stp/>
         <stp>BDP|17617562141366516571</stp>
         <tr r="F24" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3042758639</v>
+        <v>#N/A Requesting Data...1533541328</v>
         <stp/>
         <stp>BDP|13776066979946925741</stp>
         <tr r="C90" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1752919145</v>
+        <v>#N/A Requesting Data...4290292627</v>
         <stp/>
         <stp>BDP|15429465971742273156</stp>
         <tr r="E67" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2395645628</v>
+        <v>#N/A Requesting Data...3028729700</v>
         <stp/>
         <stp>BDP|13319017160191784122</stp>
         <tr r="E43" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3328682314</v>
+        <v>#N/A Requesting Data...3016118179</v>
         <stp/>
         <stp>BDP|17197570677470339052</stp>
         <tr r="E33" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3038162273</v>
+        <v>#N/A Requesting Data...436032487</v>
         <stp/>
         <stp>BDP|18198100188843948773</stp>
         <tr r="G60" s="1"/>
@@ -2663,1801 +2669,1801 @@
     </main>
     <main first="bofaddin.rtdserver">
       <tp t="s">
-        <v>#N/A Requesting Data...3501761888</v>
+        <v>#N/A Requesting Data...518081408</v>
         <stp/>
         <stp>BDP|3930904544763426134</stp>
         <tr r="C55" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2406504416</v>
+        <v>#N/A Requesting Data...3312975017</v>
         <stp/>
         <stp>BDP|7103625188072362707</stp>
         <tr r="E98" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3779059422</v>
+        <v>#N/A Requesting Data...3721352243</v>
         <stp/>
         <stp>BDP|9365312653090978315</stp>
         <tr r="G136" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1688317654</v>
+        <v>#N/A Requesting Data...3296472822</v>
         <stp/>
         <stp>BDP|6412151529379694002</stp>
         <tr r="F110" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4240258683</v>
+        <v>#N/A Requesting Data...2918484837</v>
         <stp/>
         <stp>BDP|6245426297947871034</stp>
         <tr r="C80" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1577038780</v>
+        <v>#N/A Requesting Data...3213940049</v>
         <stp/>
         <stp>BDP|2350385774053258906</stp>
         <tr r="F72" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2404900694</v>
+        <v>#N/A Requesting Data...723846039</v>
         <stp/>
         <stp>BDP|8530657130876609747</stp>
         <tr r="C44" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3092048773</v>
+        <v>#N/A Requesting Data...3755700195</v>
         <stp/>
         <stp>BDP|7198979431090342164</stp>
         <tr r="E50" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3588542765</v>
+        <v>#N/A Requesting Data...2572649853</v>
         <stp/>
         <stp>BDP|9075300299347332881</stp>
         <tr r="G79" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3432856801</v>
+        <v>#N/A Requesting Data...1752361126</v>
         <stp/>
         <stp>BDP|5029740995104753357</stp>
         <tr r="C111" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3145399215</v>
+        <v>#N/A Requesting Data...612292400</v>
         <stp/>
         <stp>BDP|8128743572863334748</stp>
         <tr r="C47" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2450659991</v>
+        <v>#N/A Requesting Data...2381951656</v>
         <stp/>
         <stp>BDP|6339719327836450907</stp>
         <tr r="C98" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3851278770</v>
+        <v>#N/A Requesting Data...2993222217</v>
         <stp/>
         <stp>BDP|4200580269163222863</stp>
         <tr r="E25" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3955284567</v>
+        <v>#N/A Requesting Data...1478811038</v>
         <stp/>
         <stp>BDP|5989352249668473659</stp>
         <tr r="G50" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3611675635</v>
+        <v>#N/A Requesting Data...4168175214</v>
         <stp/>
         <stp>BDP|2484433252649720677</stp>
         <tr r="G68" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4280467411</v>
+        <v>#N/A Requesting Data...1754565155</v>
         <stp/>
         <stp>BDP|6249870436562567333</stp>
         <tr r="E49" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2792092074</v>
+        <v>#N/A Requesting Data...1621839680</v>
         <stp/>
         <stp>BDP|9572192910556051262</stp>
         <tr r="E134" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1765898525</v>
+        <v>#N/A Requesting Data...974651891</v>
         <stp/>
         <stp>BDP|7540551159163224910</stp>
         <tr r="F51" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2375358303</v>
+        <v>#N/A Requesting Data...733891678</v>
         <stp/>
         <stp>BDP|8451204331587951367</stp>
         <tr r="F52" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4159276883</v>
+        <v>#N/A Requesting Data...3031939181</v>
         <stp/>
         <stp>BDP|3109256470563958869</stp>
         <tr r="C52" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2221748086</v>
+        <v>#N/A Requesting Data...1527204154</v>
         <stp/>
         <stp>BDP|3590543194827878545</stp>
         <tr r="F59" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3706923174</v>
+        <v>#N/A Requesting Data...2357555056</v>
         <stp/>
         <stp>BDP|3009997314886390075</stp>
         <tr r="G100" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3223942964</v>
+        <v>#N/A Requesting Data...2642193557</v>
         <stp/>
         <stp>BDP|4777106988391072114</stp>
         <tr r="F103" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3999999667</v>
+        <v>#N/A Requesting Data...1197602393</v>
         <stp/>
         <stp>BDP|4303401897634933024</stp>
         <tr r="E93" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1660623745</v>
+        <v>#N/A Requesting Data...2603315318</v>
         <stp/>
         <stp>BDP|9055938583773500695</stp>
         <tr r="C34" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2845443282</v>
+        <v>#N/A Requesting Data...3999619995</v>
         <stp/>
         <stp>BDP|1573317174439842142</stp>
         <tr r="E133" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3186334255</v>
+        <v>#N/A Requesting Data...4064223356</v>
         <stp/>
         <stp>BDP|7180318607099335068</stp>
         <tr r="C9" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3850571551</v>
+        <v>#N/A Requesting Data...3206411133</v>
         <stp/>
         <stp>BDP|8371873502449565411</stp>
         <tr r="C62" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3537155778</v>
+        <v>#N/A Requesting Data...4213591357</v>
         <stp/>
         <stp>BDP|9300723062997279226</stp>
         <tr r="C124" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2397279501</v>
+        <v>#N/A Requesting Data...585915646</v>
         <stp/>
         <stp>BDP|5492561896244379063</stp>
         <tr r="F70" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3088912906</v>
+        <v>#N/A Requesting Data...1002116051</v>
         <stp/>
         <stp>BDP|8460669760190400504</stp>
         <tr r="C27" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4049743230</v>
+        <v>#N/A Requesting Data...1819947569</v>
         <stp/>
         <stp>BDP|7634975275120208406</stp>
         <tr r="C31" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2810145035</v>
+        <v>#N/A Requesting Data...3087356478</v>
         <stp/>
         <stp>BDP|4040591290066838371</stp>
         <tr r="E13" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3977784739</v>
+        <v>#N/A Requesting Data...2242541524</v>
         <stp/>
         <stp>BDP|9247766641156585153</stp>
         <tr r="G94" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4129117296</v>
+        <v>#N/A Requesting Data...3238336452</v>
         <stp/>
         <stp>BDP|7940113982976758589</stp>
         <tr r="E95" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3811391379</v>
+        <v>#N/A Requesting Data...1709438463</v>
         <stp/>
         <stp>BDP|9093620553903200797</stp>
         <tr r="C105" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3568426287</v>
+        <v>#N/A Requesting Data...4135381288</v>
         <stp/>
         <stp>BDP|2405932012622401695</stp>
         <tr r="G77" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4173817192</v>
+        <v>#N/A Requesting Data...1030181717</v>
         <stp/>
         <stp>BDP|9175353808212225665</stp>
         <tr r="C66" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2087476565</v>
+        <v>#N/A Requesting Data...3984799757</v>
         <stp/>
         <stp>BDP|1414608591110891051</stp>
         <tr r="F9" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3282598994</v>
+        <v>#N/A Requesting Data...2658441348</v>
         <stp/>
         <stp>BDP|3649732806419915339</stp>
         <tr r="G14" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2428830740</v>
+        <v>#N/A Requesting Data...3779564969</v>
         <stp/>
         <stp>BDP|7006257261095505888</stp>
         <tr r="F54" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3056141960</v>
+        <v>#N/A Requesting Data...553895234</v>
         <stp/>
         <stp>BDP|9781989741438009272</stp>
         <tr r="C39" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1845593315</v>
+        <v>#N/A Requesting Data...3323518437</v>
         <stp/>
         <stp>BDP|7532189862547338936</stp>
         <tr r="F58" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3486459641</v>
+        <v>#N/A Requesting Data...1761689657</v>
         <stp/>
         <stp>BDP|4286027170164748985</stp>
         <tr r="G113" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4119482471</v>
+        <v>#N/A Requesting Data...3452668293</v>
         <stp/>
         <stp>BDP|4691882821088256816</stp>
         <tr r="F126" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2604312792</v>
+        <v>#N/A Requesting Data...3641591917</v>
         <stp/>
         <stp>BDP|4974055815239706225</stp>
         <tr r="G110" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2513527340</v>
+        <v>#N/A Requesting Data...2719265765</v>
         <stp/>
         <stp>BDP|5916130291376545539</stp>
         <tr r="F73" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1719373654</v>
+        <v>#N/A Requesting Data...2002845267</v>
         <stp/>
         <stp>BDP|9535646277681935723</stp>
         <tr r="E60" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2945776682</v>
+        <v>#N/A Requesting Data...1704704250</v>
         <stp/>
         <stp>BDP|3472420329653378814</stp>
         <tr r="G4" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3898448080</v>
+        <v>#N/A Requesting Data...2897983389</v>
         <stp/>
         <stp>BDP|9676580711333862054</stp>
         <tr r="E135" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1794034688</v>
+        <v>#N/A Requesting Data...504095762</v>
         <stp/>
         <stp>BDP|8651287802994649096</stp>
         <tr r="E77" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2082773024</v>
+        <v>#N/A Requesting Data...3560125160</v>
         <stp/>
         <stp>BDP|5552297197720045083</stp>
         <tr r="E118" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3056790281</v>
+        <v>#N/A Requesting Data...3994770493</v>
         <stp/>
         <stp>BDP|6195991527552839107</stp>
         <tr r="C61" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1954440445</v>
+        <v>#N/A Requesting Data...2908490669</v>
         <stp/>
         <stp>BDP|2785537291931900199</stp>
         <tr r="G91" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1834324591</v>
+        <v>#N/A Requesting Data...751735664</v>
         <stp/>
         <stp>BDP|9875435960971965593</stp>
         <tr r="C11" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3198945456</v>
+        <v>#N/A Requesting Data...1889383436</v>
         <stp/>
         <stp>BDP|5969741853480600831</stp>
         <tr r="E140" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3546470755</v>
+        <v>#N/A Requesting Data...4247879507</v>
         <stp/>
         <stp>BDP|7662972721973338089</stp>
         <tr r="F107" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2774916299</v>
+        <v>#N/A Requesting Data...1085846442</v>
         <stp/>
         <stp>BDP|4282903616430488389</stp>
         <tr r="G9" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3077422606</v>
+        <v>#N/A Requesting Data...3261427135</v>
         <stp/>
         <stp>BDP|6606398548307737925</stp>
         <tr r="C70" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2673642066</v>
+        <v>#N/A Requesting Data...1889545589</v>
         <stp/>
         <stp>BDP|2310021551041423963</stp>
         <tr r="F123" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2942241074</v>
+        <v>#N/A Requesting Data...476686701</v>
         <stp/>
         <stp>BDP|1666950877162018261</stp>
         <tr r="E87" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2135604687</v>
+        <v>#N/A Requesting Data...4069151528</v>
         <stp/>
         <stp>BDP|6280569068792932854</stp>
         <tr r="C46" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2986120527</v>
+        <v>#N/A Requesting Data...4023058504</v>
         <stp/>
         <stp>BDP|9635152443296662577</stp>
         <tr r="C16" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3748636851</v>
+        <v>#N/A Requesting Data...2816128063</v>
         <stp/>
         <stp>BDP|5935740968278021330</stp>
         <tr r="C96" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2073007319</v>
+        <v>#N/A Requesting Data...4215053680</v>
         <stp/>
         <stp>BDP|8225387168083679130</stp>
         <tr r="E57" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3736224853</v>
+        <v>#N/A Requesting Data...2385728029</v>
         <stp/>
         <stp>BDP|8741792397660502982</stp>
         <tr r="G24" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2792598094</v>
+        <v>#N/A Requesting Data...4004691321</v>
         <stp/>
         <stp>BDP|1988621838892198978</stp>
         <tr r="F82" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1663915535</v>
+        <v>#N/A Requesting Data...3987017588</v>
         <stp/>
         <stp>BDP|5160947801244572083</stp>
         <tr r="C97" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3389100644</v>
+        <v>#N/A Requesting Data...2911829596</v>
         <stp/>
         <stp>BDP|8781684350665372626</stp>
         <tr r="G64" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2630091139</v>
+        <v>#N/A Requesting Data...4087962396</v>
         <stp/>
         <stp>BDP|8866465832365619258</stp>
         <tr r="F120" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2514512430</v>
+        <v>#N/A Requesting Data...4275591433</v>
         <stp/>
         <stp>BDP|1231973558974048121</stp>
         <tr r="E123" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2994528356</v>
+        <v>#N/A Requesting Data...786492112</v>
         <stp/>
         <stp>BDP|9011959145835954962</stp>
         <tr r="E102" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4207658614</v>
+        <v>#N/A Requesting Data...2471186271</v>
         <stp/>
         <stp>BDP|7048111723254898858</stp>
         <tr r="E70" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3868116129</v>
+        <v>#N/A Requesting Data...1629652438</v>
         <stp/>
         <stp>BDP|7514426398370500271</stp>
         <tr r="F84" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3616245534</v>
+        <v>#N/A Requesting Data...1073851964</v>
         <stp/>
         <stp>BDP|2286847884578687294</stp>
         <tr r="C64" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1930410336</v>
+        <v>#N/A Requesting Data...991935531</v>
         <stp/>
         <stp>BDP|8581359335587083771</stp>
         <tr r="G40" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3655724587</v>
+        <v>#N/A Requesting Data...1748497322</v>
         <stp/>
         <stp>BDP|9176352611073152053</stp>
         <tr r="G52" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2571450515</v>
+        <v>#N/A Requesting Data...820948897</v>
         <stp/>
         <stp>BDP|3761613276703138977</stp>
         <tr r="C22" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2709007450</v>
+        <v>#N/A Requesting Data...2470048004</v>
         <stp/>
         <stp>BDP|2402283480247992710</stp>
         <tr r="G65" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1933827057</v>
+        <v>#N/A Requesting Data...1368564087</v>
         <stp/>
         <stp>BDP|2496054182730824314</stp>
         <tr r="F108" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1804109621</v>
+        <v>#N/A Requesting Data...984842409</v>
         <stp/>
         <stp>BDP|1156198294412416234</stp>
         <tr r="G48" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2653782713</v>
+        <v>#N/A Requesting Data...1724358332</v>
         <stp/>
         <stp>BDP|1935863512592400318</stp>
         <tr r="G99" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2013677964</v>
+        <v>#N/A Requesting Data...3120157438</v>
         <stp/>
         <stp>BDP|1182070188629538920</stp>
         <tr r="F85" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2957313728</v>
+        <v>#N/A Requesting Data...550341735</v>
         <stp/>
         <stp>BDP|9924697901094165296</stp>
         <tr r="E38" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1827501361</v>
+        <v>#N/A Requesting Data...3279436840</v>
         <stp/>
         <stp>BDP|6412137247758825261</stp>
         <tr r="G10" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2220354440</v>
+        <v>#N/A Requesting Data...2522449051</v>
         <stp/>
         <stp>BDP|6277108296426856136</stp>
         <tr r="G122" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3749230045</v>
+        <v>#N/A Requesting Data...2565148026</v>
         <stp/>
         <stp>BDP|2351176324921816947</stp>
         <tr r="E117" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3963330299</v>
+        <v>#N/A Requesting Data...1373088927</v>
         <stp/>
         <stp>BDP|6406207188846485346</stp>
         <tr r="C37" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4247226656</v>
+        <v>#N/A Requesting Data...3373975656</v>
         <stp/>
         <stp>BDP|8112280367483097628</stp>
         <tr r="F16" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2304512307</v>
+        <v>#N/A Requesting Data...2416176471</v>
         <stp/>
         <stp>BDP|6484624822372932905</stp>
         <tr r="C108" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2148960187</v>
+        <v>#N/A Requesting Data...4232546691</v>
         <stp/>
         <stp>BDP|8605875253514357834</stp>
         <tr r="C116" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2068505088</v>
+        <v>#N/A Requesting Data...4100730872</v>
         <stp/>
         <stp>BDP|2842991807747556512</stp>
         <tr r="E110" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2695235279</v>
+        <v>#N/A Requesting Data...3261368088</v>
         <stp/>
         <stp>BDP|1377759003508711718</stp>
         <tr r="E55" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3579263356</v>
+        <v>#N/A Requesting Data...595397678</v>
         <stp/>
         <stp>BDP|1711361391887412536</stp>
         <tr r="G47" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2432396723</v>
+        <v>#N/A Requesting Data...1532257708</v>
         <stp/>
         <stp>BDP|4564815655442574234</stp>
         <tr r="F114" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2933267252</v>
+        <v>#N/A Requesting Data...3375130925</v>
         <stp/>
         <stp>BDP|6557751567646791843</stp>
         <tr r="C85" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2764912294</v>
+        <v>#N/A Requesting Data...2553465493</v>
         <stp/>
         <stp>BDP|5018226780961297742</stp>
         <tr r="E138" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2214802789</v>
+        <v>#N/A Requesting Data...1123431736</v>
         <stp/>
         <stp>BDP|7190582290036507495</stp>
         <tr r="E48" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3423739007</v>
+        <v>#N/A Requesting Data...3465237305</v>
         <stp/>
         <stp>BDP|7268732641219205478</stp>
         <tr r="F111" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3027095045</v>
+        <v>#N/A Requesting Data...3017135004</v>
         <stp/>
         <stp>BDP|5085458293997400582</stp>
         <tr r="C30" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3681036704</v>
+        <v>#N/A Requesting Data...2092337772</v>
         <stp/>
         <stp>BDP|2916061605678582044</stp>
         <tr r="E27" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1957405794</v>
+        <v>#N/A Requesting Data...2641737701</v>
         <stp/>
         <stp>BDP|5645196194854205325</stp>
         <tr r="E19" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3883290273</v>
+        <v>#N/A Requesting Data...2731811761</v>
         <stp/>
         <stp>BDP|8929421222763426766</stp>
         <tr r="F112" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2355012901</v>
+        <v>#N/A Requesting Data...1718300892</v>
         <stp/>
         <stp>BDP|2815946348173965667</stp>
         <tr r="C137" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3835484703</v>
+        <v>#N/A Requesting Data...1439557279</v>
         <stp/>
         <stp>BDP|6645611732949919042</stp>
         <tr r="G95" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2044094107</v>
+        <v>#N/A Requesting Data...2104998059</v>
         <stp/>
         <stp>BDP|8744658502964028082</stp>
         <tr r="F139" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3254644198</v>
+        <v>#N/A Requesting Data...1747626743</v>
         <stp/>
         <stp>BDP|4077907452745230782</stp>
         <tr r="C130" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2760630562</v>
+        <v>#N/A Requesting Data...3879305424</v>
         <stp/>
         <stp>BDP|8975856381415089739</stp>
         <tr r="E75" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4198491593</v>
+        <v>#N/A Requesting Data...796117279</v>
         <stp/>
         <stp>BDP|5738611839292209825</stp>
         <tr r="G107" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3098364358</v>
+        <v>#N/A Requesting Data...1545288890</v>
         <stp/>
         <stp>BDP|4996818111432201578</stp>
         <tr r="G134" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2333962592</v>
+        <v>#N/A Requesting Data...1581317174</v>
         <stp/>
         <stp>BDP|5458032582021895609</stp>
         <tr r="E89" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4160167520</v>
+        <v>#N/A Requesting Data...4256604020</v>
         <stp/>
         <stp>BDP|2612461303954522846</stp>
         <tr r="F21" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2655123782</v>
+        <v>#N/A Requesting Data...2798959077</v>
         <stp/>
         <stp>BDP|5852840000806674187</stp>
         <tr r="F75" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2490959240</v>
+        <v>#N/A Requesting Data...2116181778</v>
         <stp/>
         <stp>BDP|7947641811679527399</stp>
         <tr r="G13" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1898041741</v>
+        <v>#N/A Requesting Data...3293266350</v>
         <stp/>
         <stp>BDP|8407769428857900025</stp>
         <tr r="C132" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2475761758</v>
+        <v>#N/A Requesting Data...3190428866</v>
         <stp/>
         <stp>BDP|1313714864639868399</stp>
         <tr r="F87" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3113568693</v>
+        <v>#N/A Requesting Data...1171654374</v>
         <stp/>
         <stp>BDP|2531298252748844733</stp>
         <tr r="F115" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4112114671</v>
+        <v>#N/A Requesting Data...2618312757</v>
         <stp/>
         <stp>BDP|8965389266391509672</stp>
         <tr r="C41" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3295241036</v>
+        <v>#N/A Requesting Data...2937843852</v>
         <stp/>
         <stp>BDP|9146373380128430189</stp>
         <tr r="F60" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3582805952</v>
+        <v>#N/A Requesting Data...3726882109</v>
         <stp/>
         <stp>BDP|8769626454200391097</stp>
         <tr r="G85" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2128491147</v>
+        <v>#N/A Requesting Data...3690847788</v>
         <stp/>
         <stp>BDP|7701346097304455298</stp>
         <tr r="C73" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4278959883</v>
+        <v>#N/A Requesting Data...3881378377</v>
         <stp/>
         <stp>BDP|1201589979318261083</stp>
         <tr r="G123" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2457250209</v>
+        <v>#N/A Requesting Data...3905305442</v>
         <stp/>
         <stp>BDP|9994425762708075853</stp>
         <tr r="G88" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1755768459</v>
+        <v>#N/A Requesting Data...1680813820</v>
         <stp/>
         <stp>BDP|8238868892513701135</stp>
         <tr r="G137" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2796926154</v>
+        <v>#N/A Requesting Data...2422385173</v>
         <stp/>
         <stp>BDP|3321556007464177923</stp>
         <tr r="E109" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2983545734</v>
+        <v>#N/A Requesting Data...1662561277</v>
         <stp/>
         <stp>BDP|8367368187378355023</stp>
         <tr r="F64" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2674161216</v>
+        <v>#N/A Requesting Data...2708459257</v>
         <stp/>
         <stp>BDP|9054142235387080711</stp>
         <tr r="F11" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3544053887</v>
+        <v>#N/A Requesting Data...1876545857</v>
         <stp/>
         <stp>BDP|4797724273716399932</stp>
         <tr r="C5" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2780472061</v>
+        <v>#N/A Requesting Data...1089566942</v>
         <stp/>
         <stp>BDP|3084971212582403246</stp>
         <tr r="F121" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2476398226</v>
+        <v>#N/A Requesting Data...2993439464</v>
         <stp/>
         <stp>BDP|6948762204713990690</stp>
         <tr r="G90" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3409334277</v>
+        <v>#N/A Requesting Data...1879853452</v>
         <stp/>
         <stp>BDP|1832764578595986067</stp>
         <tr r="G119" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2575453126</v>
+        <v>#N/A Requesting Data...2713902386</v>
         <stp/>
         <stp>BDP|4156639623951685595</stp>
         <tr r="F13" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2414550167</v>
+        <v>#N/A Requesting Data...3045217043</v>
         <stp/>
         <stp>BDP|5919761437851372455</stp>
         <tr r="C2" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4285673479</v>
+        <v>#N/A Requesting Data...2042070077</v>
         <stp/>
         <stp>BDP|1551339666687413790</stp>
         <tr r="F40" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2192691104</v>
+        <v>#N/A Requesting Data...3020176732</v>
         <stp/>
         <stp>BDP|6420437202397070174</stp>
         <tr r="C8" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2497355537</v>
+        <v>#N/A Requesting Data...2307001691</v>
         <stp/>
         <stp>BDP|1708381902825815365</stp>
         <tr r="C101" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3366882330</v>
+        <v>#N/A Requesting Data...3739861855</v>
         <stp/>
         <stp>BDP|4945796250777738578</stp>
         <tr r="G21" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2976197998</v>
+        <v>#N/A Requesting Data...2737792707</v>
         <stp/>
         <stp>BDP|6746841414412327938</stp>
         <tr r="G75" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3834554600</v>
+        <v>#N/A Requesting Data...3452257742</v>
         <stp/>
         <stp>BDP|1709445403856801620</stp>
         <tr r="E85" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2065063537</v>
+        <v>#N/A Requesting Data...3175338502</v>
         <stp/>
         <stp>BDP|9398823419477440265</stp>
         <tr r="G125" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2985714081</v>
+        <v>#N/A Requesting Data...3653286519</v>
         <stp/>
         <stp>BDP|3430878723724827801</stp>
         <tr r="G41" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3420709920</v>
+        <v>#N/A Requesting Data...1933149826</v>
         <stp/>
         <stp>BDP|9698422803149077198</stp>
         <tr r="C100" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2744999247</v>
+        <v>#N/A Requesting Data...1153823662</v>
         <stp/>
         <stp>BDP|2887002514665714363</stp>
         <tr r="G59" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2120113269</v>
+        <v>#N/A Requesting Data...4135634195</v>
         <stp/>
         <stp>BDP|2668814054578766269</stp>
         <tr r="E31" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1905449081</v>
+        <v>#N/A Requesting Data...3520025410</v>
         <stp/>
         <stp>BDP|8894702939828266110</stp>
         <tr r="C7" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4233377268</v>
+        <v>#N/A Requesting Data...2988772910</v>
         <stp/>
         <stp>BDP|3410885660260666884</stp>
         <tr r="E64" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2170971970</v>
+        <v>#N/A Requesting Data...1568660127</v>
         <stp/>
         <stp>BDP|3658713905400418152</stp>
         <tr r="E35" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2916489368</v>
+        <v>#N/A Requesting Data...3230746206</v>
         <stp/>
         <stp>BDP|7570300716478486864</stp>
         <tr r="E32" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2464319888</v>
+        <v>#N/A Requesting Data...3645675523</v>
         <stp/>
         <stp>BDP|7851492951527237434</stp>
         <tr r="E52" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2121810251</v>
+        <v>#N/A Requesting Data...2586454802</v>
         <stp/>
         <stp>BDP|7352242467910007671</stp>
         <tr r="F124" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2897397419</v>
+        <v>#N/A Requesting Data...1720337171</v>
         <stp/>
         <stp>BDP|5657563513753480721</stp>
         <tr r="E80" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2659421956</v>
+        <v>#N/A Requesting Data...2876498037</v>
         <stp/>
         <stp>BDP|5976587264538865878</stp>
         <tr r="E62" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2297748359</v>
+        <v>#N/A Requesting Data...3573779692</v>
         <stp/>
         <stp>BDP|7151318027339523982</stp>
         <tr r="F91" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2820956237</v>
+        <v>#N/A Requesting Data...2271282359</v>
         <stp/>
         <stp>BDP|1896477110772260049</stp>
         <tr r="C91" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2333309695</v>
+        <v>#N/A Requesting Data...2711614910</v>
         <stp/>
         <stp>BDP|4252725967471187287</stp>
         <tr r="F44" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4183333807</v>
+        <v>#N/A Requesting Data...1663092124</v>
         <stp/>
         <stp>BDP|6943451920864586278</stp>
         <tr r="C118" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4216409302</v>
+        <v>#N/A Requesting Data...3384823905</v>
         <stp/>
         <stp>BDP|5838113265174067025</stp>
         <tr r="F39" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3541214316</v>
+        <v>#N/A Requesting Data...1151104038</v>
         <stp/>
         <stp>BDP|3456718228377624745</stp>
         <tr r="E111" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2258615252</v>
+        <v>#N/A Requesting Data...2871425608</v>
         <stp/>
         <stp>BDP|5917425194519245724</stp>
         <tr r="E79" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2497481640</v>
+        <v>#N/A Requesting Data...905661700</v>
         <stp/>
         <stp>BDP|6787533358407016713</stp>
         <tr r="F135" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3620579220</v>
+        <v>#N/A Requesting Data...2005895380</v>
         <stp/>
         <stp>BDP|5576451913756991076</stp>
         <tr r="E16" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2550137951</v>
+        <v>#N/A Requesting Data...4019845859</v>
         <stp/>
         <stp>BDP|5284390591628042184</stp>
         <tr r="C24" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2312927361</v>
+        <v>#N/A Requesting Data...2086988448</v>
         <stp/>
         <stp>BDP|5412037028917536689</stp>
         <tr r="G115" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3112878656</v>
+        <v>#N/A Requesting Data...4133588642</v>
         <stp/>
         <stp>BDP|8966942938724477029</stp>
         <tr r="C15" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3977912003</v>
+        <v>#N/A Requesting Data...2017128733</v>
         <stp/>
         <stp>BDP|2938144706552859709</stp>
         <tr r="G81" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2236250828</v>
+        <v>#N/A Requesting Data...3595983902</v>
         <stp/>
         <stp>BDP|3632949480676633244</stp>
         <tr r="F31" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3734197764</v>
+        <v>#N/A Requesting Data...2876852706</v>
         <stp/>
         <stp>BDP|3513418606797579639</stp>
         <tr r="F90" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3664172856</v>
+        <v>#N/A Requesting Data...3154671867</v>
         <stp/>
         <stp>BDP|1733520919261908213</stp>
         <tr r="G73" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2908413023</v>
+        <v>#N/A Requesting Data...3740638374</v>
         <stp/>
         <stp>BDP|8368969127023380651</stp>
         <tr r="F28" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3161710385</v>
+        <v>#N/A Requesting Data...3452678272</v>
         <stp/>
         <stp>BDP|7172716621593553717</stp>
         <tr r="F53" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1837425809</v>
+        <v>#N/A Requesting Data...4113270740</v>
         <stp/>
         <stp>BDP|2954250373819174944</stp>
         <tr r="F119" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4277079299</v>
+        <v>#N/A Requesting Data...2174932365</v>
         <stp/>
         <stp>BDP|4728287753511799518</stp>
         <tr r="F3" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2103357315</v>
+        <v>#N/A Requesting Data...1991476781</v>
         <stp/>
         <stp>BDP|6348617969513327227</stp>
         <tr r="E104" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3726125795</v>
+        <v>#N/A Requesting Data...3129896262</v>
         <stp/>
         <stp>BDP|7694099704858685831</stp>
         <tr r="C107" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3379037412</v>
+        <v>#N/A Requesting Data...711748480</v>
         <stp/>
         <stp>BDP|4106834752526835861</stp>
         <tr r="F55" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4274930654</v>
+        <v>#N/A Requesting Data...1915963077</v>
         <stp/>
         <stp>BDP|7951337561756108354</stp>
         <tr r="G112" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3038955291</v>
+        <v>#N/A Requesting Data...2534670081</v>
         <stp/>
         <stp>BDP|5468867501418549294</stp>
         <tr r="E86" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2009375124</v>
+        <v>#N/A Requesting Data...2198089130</v>
         <stp/>
         <stp>BDP|4546740053823447251</stp>
         <tr r="C32" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3270789562</v>
+        <v>#N/A Requesting Data...1731885443</v>
         <stp/>
         <stp>BDP|7484527599745538990</stp>
         <tr r="F76" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1867790560</v>
+        <v>#N/A Requesting Data...3497278369</v>
         <stp/>
         <stp>BDP|5578475423865159117</stp>
         <tr r="E61" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3871201231</v>
+        <v>#N/A Requesting Data...3301520664</v>
         <stp/>
         <stp>BDP|6158107237024797760</stp>
         <tr r="E45" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2658787723</v>
+        <v>#N/A Requesting Data...2507934999</v>
         <stp/>
         <stp>BDP|4143076943390197735</stp>
         <tr r="F97" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2006854516</v>
+        <v>#N/A Requesting Data...3774029430</v>
         <stp/>
         <stp>BDP|1762196091349932721</stp>
         <tr r="E82" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2760211759</v>
+        <v>#N/A Requesting Data...760238303</v>
         <stp/>
         <stp>BDP|4189169184528349241</stp>
         <tr r="F137" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4201704560</v>
+        <v>#N/A Requesting Data...2711260551</v>
         <stp/>
         <stp>BDP|9103140635044368872</stp>
         <tr r="F29" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2411173674</v>
+        <v>#N/A Requesting Data...1188475633</v>
         <stp/>
         <stp>BDP|5519603296584718917</stp>
         <tr r="G54" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3399325895</v>
+        <v>#N/A Requesting Data...2923461068</v>
         <stp/>
         <stp>BDP|1156250824766982737</stp>
         <tr r="G44" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2452831534</v>
+        <v>#N/A Requesting Data...2782375172</v>
         <stp/>
         <stp>BDP|6031605254431729496</stp>
         <tr r="G86" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1873186553</v>
+        <v>#N/A Requesting Data...1562793937</v>
         <stp/>
         <stp>BDP|2649489454114394728</stp>
         <tr r="C14" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4180118379</v>
+        <v>#N/A Requesting Data...3678833377</v>
         <stp/>
         <stp>BDP|8999377595616850481</stp>
         <tr r="E108" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3083312594</v>
+        <v>#N/A Requesting Data...2251178461</v>
         <stp/>
         <stp>BDP|8988928209665280487</stp>
         <tr r="F71" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3635684369</v>
+        <v>#N/A Requesting Data...2187063806</v>
         <stp/>
         <stp>BDP|8368023487691952119</stp>
         <tr r="F88" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2094095576</v>
+        <v>#N/A Requesting Data...2814852972</v>
         <stp/>
         <stp>BDP|5199287207907438042</stp>
         <tr r="E66" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4049072242</v>
+        <v>#N/A Requesting Data...3792145531</v>
         <stp/>
         <stp>BDP|7460099446995728631</stp>
         <tr r="F134" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3249684893</v>
+        <v>#N/A Requesting Data...3829242541</v>
         <stp/>
         <stp>BDP|6160638673325976246</stp>
         <tr r="C104" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2785271618</v>
+        <v>#N/A Requesting Data...1431281087</v>
         <stp/>
         <stp>BDP|5660731962530222490</stp>
         <tr r="E128" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3373954882</v>
+        <v>#N/A Requesting Data...3961437347</v>
         <stp/>
         <stp>BDP|3355023726294311595</stp>
         <tr r="G114" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3493777186</v>
+        <v>#N/A Requesting Data...2270856093</v>
         <stp/>
         <stp>BDP|5604474461391860653</stp>
         <tr r="E130" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3583537855</v>
+        <v>#N/A Requesting Data...3875016615</v>
         <stp/>
         <stp>BDP|3542140114402066179</stp>
         <tr r="E78" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3866745018</v>
+        <v>#N/A Requesting Data...1435459493</v>
         <stp/>
         <stp>BDP|2942496252996870592</stp>
         <tr r="G121" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2532239204</v>
+        <v>#N/A Requesting Data...4156512207</v>
         <stp/>
         <stp>BDP|1823820926283534897</stp>
         <tr r="G18" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3083926893</v>
+        <v>#N/A Requesting Data...1044844626</v>
         <stp/>
         <stp>BDP|3716189405712826043</stp>
         <tr r="G92" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2029733841</v>
+        <v>#N/A Requesting Data...1833322969</v>
         <stp/>
         <stp>BDP|3228146609442097080</stp>
         <tr r="C140" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3319725661</v>
+        <v>#N/A Requesting Data...4086450329</v>
         <stp/>
         <stp>BDP|9344147089140006098</stp>
         <tr r="E83" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4032857707</v>
+        <v>#N/A Requesting Data...2427302753</v>
         <stp/>
         <stp>BDP|6993061706081965773</stp>
         <tr r="F81" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2823592321</v>
+        <v>#N/A Requesting Data...3238679746</v>
         <stp/>
         <stp>BDP|6176792116871092198</stp>
         <tr r="C68" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2632669104</v>
+        <v>#N/A Requesting Data...3780260838</v>
         <stp/>
         <stp>BDP|7185432584822399912</stp>
         <tr r="F131" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3360716697</v>
+        <v>#N/A Requesting Data...3945989859</v>
         <stp/>
         <stp>BDP|8280856169194643320</stp>
         <tr r="G49" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2102109281</v>
+        <v>#N/A Requesting Data...3896284611</v>
         <stp/>
         <stp>BDP|9399109618929306123</stp>
         <tr r="F37" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4207414606</v>
+        <v>#N/A Requesting Data...1268168318</v>
         <stp/>
         <stp>BDP|6669663699409638145</stp>
         <tr r="C123" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3851787647</v>
+        <v>#N/A Requesting Data...3962840489</v>
         <stp/>
         <stp>BDP|6175693122901836298</stp>
         <tr r="C36" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2215538981</v>
+        <v>#N/A Requesting Data...1208355585</v>
         <stp/>
         <stp>BDP|8135075327118072391</stp>
         <tr r="C17" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2441916576</v>
+        <v>#N/A Requesting Data...1005430097</v>
         <stp/>
         <stp>BDP|5726291712345411206</stp>
         <tr r="G28" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3616813101</v>
+        <v>#N/A Requesting Data...3425673010</v>
         <stp/>
         <stp>BDP|8698973352783506690</stp>
         <tr r="F25" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3467817127</v>
+        <v>#N/A Requesting Data...3844235823</v>
         <stp/>
         <stp>BDP|5493604681742158862</stp>
         <tr r="G63" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2689147348</v>
+        <v>#N/A Requesting Data...1732042222</v>
         <stp/>
         <stp>BDP|3239104742287612040</stp>
         <tr r="E39" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2996016871</v>
+        <v>#N/A Requesting Data...3393203262</v>
         <stp/>
         <stp>BDP|3381147726641663059</stp>
         <tr r="C122" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4076084125</v>
+        <v>#N/A Requesting Data...1011684232</v>
         <stp/>
         <stp>BDP|6625906764329795167</stp>
         <tr r="F56" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2933197974</v>
+        <v>#N/A Requesting Data...3929985876</v>
         <stp/>
         <stp>BDP|3325218238213801010</stp>
         <tr r="F57" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2376387914</v>
+        <v>#N/A Requesting Data...2856733874</v>
         <stp/>
         <stp>BDP|1313137390988032037</stp>
         <tr r="C83" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3244271648</v>
+        <v>#N/A Requesting Data...2350954742</v>
         <stp/>
         <stp>BDP|3702733300853619616</stp>
         <tr r="G34" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3487322708</v>
+        <v>#N/A Requesting Data...2975749398</v>
         <stp/>
         <stp>BDP|8558611930018338475</stp>
         <tr r="F35" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2696491406</v>
+        <v>#N/A Requesting Data...3437496015</v>
         <stp/>
         <stp>BDP|5387098906493173798</stp>
         <tr r="G62" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3293735453</v>
+        <v>#N/A Requesting Data...2816734399</v>
         <stp/>
         <stp>BDP|1951038018907673608</stp>
         <tr r="C126" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3256683358</v>
+        <v>#N/A Requesting Data...4026968796</v>
         <stp/>
         <stp>BDP|9253802402770546012</stp>
         <tr r="F74" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3441362351</v>
+        <v>#N/A Requesting Data...3943826564</v>
         <stp/>
         <stp>BDP|1884505914021260664</stp>
         <tr r="E96" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2192914588</v>
+        <v>#N/A Requesting Data...1812095089</v>
         <stp/>
         <stp>BDP|3540127028674193608</stp>
         <tr r="F94" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3676422996</v>
+        <v>#N/A Requesting Data...3079863195</v>
         <stp/>
         <stp>BDP|5372375359741187031</stp>
         <tr r="F27" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2741773758</v>
+        <v>#N/A Requesting Data...989572123</v>
         <stp/>
         <stp>BDP|5121625602631825066</stp>
         <tr r="E81" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4266234109</v>
+        <v>#N/A Requesting Data...3130239438</v>
         <stp/>
         <stp>BDP|5282708515920897138</stp>
         <tr r="F43" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3688250309</v>
+        <v>#N/A Requesting Data...2271172753</v>
         <stp/>
         <stp>BDP|1250299291741371958</stp>
         <tr r="G31" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2419382463</v>
+        <v>#N/A Requesting Data...1755087098</v>
         <stp/>
         <stp>BDP|4253176148933327033</stp>
         <tr r="C133" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3377077765</v>
+        <v>#N/A Requesting Data...4049502931</v>
         <stp/>
         <stp>BDP|9704751602229087502</stp>
         <tr r="F49" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4205856852</v>
+        <v>#N/A Requesting Data...854290810</v>
         <stp/>
         <stp>BDP|6775233901286469015</stp>
         <tr r="E125" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3469482753</v>
+        <v>#N/A Requesting Data...1120715169</v>
         <stp/>
         <stp>BDP|7918289416910309647</stp>
         <tr r="C56" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2241305872</v>
+        <v>#N/A Requesting Data...2441058251</v>
         <stp/>
         <stp>BDP|3731272815900600241</stp>
         <tr r="C53" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3509419193</v>
+        <v>#N/A Requesting Data...3534989116</v>
         <stp/>
         <stp>BDP|1685459166489439868</stp>
         <tr r="F133" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3788820337</v>
+        <v>#N/A Requesting Data...1142040634</v>
         <stp/>
         <stp>BDP|2506644172580171154</stp>
         <tr r="C119" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2268845963</v>
+        <v>#N/A Requesting Data...1374031940</v>
         <stp/>
         <stp>BDP|1995353227627490580</stp>
         <tr r="E119" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2872664958</v>
+        <v>#N/A Requesting Data...3205491158</v>
         <stp/>
         <stp>BDP|9173868178561206592</stp>
         <tr r="C77" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2292272627</v>
+        <v>#N/A Requesting Data...2917154479</v>
         <stp/>
         <stp>BDP|4008096672221657096</stp>
         <tr r="G43" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3925611815</v>
+        <v>#N/A Requesting Data...2574984111</v>
         <stp/>
         <stp>BDP|5434663182001395869</stp>
         <tr r="E107" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2868357349</v>
+        <v>#N/A Requesting Data...1499522446</v>
         <stp/>
         <stp>BDP|8686279502629263146</stp>
         <tr r="C129" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4077397490</v>
+        <v>#N/A Requesting Data...2107797109</v>
         <stp/>
         <stp>BDP|4576300957588172984</stp>
         <tr r="E63" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2823587102</v>
+        <v>#N/A Requesting Data...1729453523</v>
         <stp/>
         <stp>BDP|7469671678835895086</stp>
         <tr r="E2" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3137102726</v>
+        <v>#N/A Requesting Data...1838897942</v>
         <stp/>
         <stp>BDP|5444751401066968714</stp>
         <tr r="E73" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3731376385</v>
+        <v>#N/A Requesting Data...1086082105</v>
         <stp/>
         <stp>BDP|2824124077350027748</stp>
         <tr r="E136" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3507125160</v>
+        <v>#N/A Requesting Data...1391433013</v>
         <stp/>
         <stp>BDP|3708851985886704699</stp>
         <tr r="C19" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2501617796</v>
+        <v>#N/A Requesting Data...3634805172</v>
         <stp/>
         <stp>BDP|1006071828475585561</stp>
         <tr r="F116" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4205973170</v>
+        <v>#N/A Requesting Data...2062177258</v>
         <stp/>
         <stp>BDP|1086712249007771639</stp>
         <tr r="G26" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3377172863</v>
+        <v>#N/A Requesting Data...3985107186</v>
         <stp/>
         <stp>BDP|6634730869724168016</stp>
         <tr r="E103" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3759347543</v>
+        <v>#N/A Requesting Data...2415887883</v>
         <stp/>
         <stp>BDP|3520366017777816505</stp>
         <tr r="E97" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3229486341</v>
+        <v>#N/A Requesting Data...2087003033</v>
         <stp/>
         <stp>BDP|2995135217932647367</stp>
         <tr r="F105" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3240619502</v>
+        <v>#N/A Requesting Data...3347567706</v>
         <stp/>
         <stp>BDP|3565057922625094707</stp>
         <tr r="G45" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2485406064</v>
+        <v>#N/A Requesting Data...2506305386</v>
         <stp/>
         <stp>BDP|1485569542807651461</stp>
         <tr r="C86" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4070245329</v>
+        <v>#N/A Requesting Data...1274587287</v>
         <stp/>
         <stp>BDP|1159006460850353421</stp>
         <tr r="E46" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2029636777</v>
+        <v>#N/A Requesting Data...2654480716</v>
         <stp/>
         <stp>BDP|5113311422502283510</stp>
         <tr r="C84" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2431026835</v>
+        <v>#N/A Requesting Data...2171277543</v>
         <stp/>
         <stp>BDP|4420649803735408460</stp>
         <tr r="F117" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2986269047</v>
+        <v>#N/A Requesting Data...2051895516</v>
         <stp/>
         <stp>BDP|9873235984695079585</stp>
         <tr r="C60" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2304639060</v>
+        <v>#N/A Requesting Data...2154915284</v>
         <stp/>
         <stp>BDP|4726106605717010168</stp>
         <tr r="G46" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3638953723</v>
+        <v>#N/A Requesting Data...3258907437</v>
         <stp/>
         <stp>BDP|97453184744598227</stp>
         <tr r="G135" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2446730215</v>
+        <v>#N/A Requesting Data...1115661231</v>
         <stp/>
         <stp>BDP|71129432364790944</stp>
         <tr r="E105" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3850761440</v>
+        <v>#N/A Requesting Data...2301437588</v>
         <stp/>
         <stp>BDP|13870968378316918</stp>
         <tr r="F38" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4087556597</v>
+        <v>#N/A Requesting Data...1554907126</v>
         <stp/>
         <stp>BDP|545017254499479967</stp>
         <tr r="E23" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3953828866</v>
+        <v>#N/A Requesting Data...3686684491</v>
         <stp/>
         <stp>BDP|562457211792430265</stp>
         <tr r="G116" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2097389340</v>
+        <v>#N/A Requesting Data...2654882844</v>
         <stp/>
         <stp>BDP|752318736222262646</stp>
         <tr r="F83" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2139279915</v>
+        <v>#N/A Requesting Data...1898584463</v>
         <stp/>
         <stp>BDP|926433161397617222</stp>
         <tr r="F10" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3262787735</v>
+        <v>#N/A Requesting Data...2696222718</v>
         <stp/>
         <stp>BDP|455507803480864317</stp>
         <tr r="C51" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2036073995</v>
+        <v>#N/A Requesting Data...2161484984</v>
         <stp/>
         <stp>BDP|738430784972633891</stp>
         <tr r="F41" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3690480777</v>
+        <v>#N/A Requesting Data...3341530035</v>
         <stp/>
         <stp>BDP|226270545351892196</stp>
         <tr r="F61" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3776176325</v>
+        <v>#N/A Requesting Data...2051949616</v>
         <stp/>
         <stp>BDP|478534605105814154</stp>
         <tr r="G12" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2643541089</v>
+        <v>#N/A Requesting Data...1980328135</v>
         <stp/>
         <stp>BDP|292697057297288557</stp>
         <tr r="C106" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3637702590</v>
+        <v>#N/A Requesting Data...1021928372</v>
         <stp/>
         <stp>BDP|449489448517477649</stp>
         <tr r="E99" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2474426678</v>
+        <v>#N/A Requesting Data...2391817801</v>
         <stp/>
         <stp>BDP|477239144286521179</stp>
         <tr r="G138" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3117274719</v>
+        <v>#N/A Requesting Data...3534648721</v>
         <stp/>
         <stp>BDP|136361134742057301</stp>
         <tr r="C57" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2777001628</v>
+        <v>#N/A Requesting Data...1086730295</v>
         <stp/>
         <stp>BDP|282958180978155995</stp>
         <tr r="C59" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3744046389</v>
+        <v>#N/A Requesting Data...2903784918</v>
         <stp/>
         <stp>BDP|991366924295531418</stp>
         <tr r="F2" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3910948421</v>
+        <v>#N/A Requesting Data...1884815789</v>
         <stp/>
         <stp>BDP|934073235795196633</stp>
         <tr r="F62" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2189727606</v>
+        <v>#N/A Requesting Data...2563791705</v>
         <stp/>
         <stp>BDP|266608211912165570</stp>
         <tr r="E113" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2824800763</v>
+        <v>#N/A Requesting Data...3057108061</v>
         <stp/>
         <stp>BDP|910156400954699593</stp>
         <tr r="G8" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3720428457</v>
+        <v>#N/A Requesting Data...949952724</v>
         <stp/>
         <stp>BDP|794293317440269040</stp>
         <tr r="E100" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3855826184</v>
+        <v>#N/A Requesting Data...3688105301</v>
         <stp/>
         <stp>BDP|206766873121157269</stp>
         <tr r="E41" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2521406317</v>
+        <v>#N/A Requesting Data...2368675557</v>
         <stp/>
         <stp>BDP|315261912951356153</stp>
         <tr r="E21" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2775329017</v>
+        <v>#N/A Requesting Data...3793664019</v>
         <stp/>
         <stp>BDP|169080827246056602</stp>
         <tr r="G126" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4111998338</v>
+        <v>#N/A Requesting Data...3089408073</v>
         <stp/>
         <stp>BDP|454779781439338455</stp>
         <tr r="E36" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1981506268</v>
+        <v>#N/A Requesting Data...1188566924</v>
         <stp/>
         <stp>BDP|198524097739196711</stp>
         <tr r="F92" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2905238605</v>
+        <v>#N/A Requesting Data...1173514560</v>
         <stp/>
         <stp>BDP|618726407191106421</stp>
         <tr r="C92" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3780438030</v>
+        <v>#N/A Requesting Data...820464992</v>
         <stp/>
         <stp>BDP|442808307356626303</stp>
         <tr r="F20" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3718889607</v>
+        <v>#N/A Requesting Data...4256063393</v>
         <stp/>
         <stp>BDP|624014897144495064</stp>
         <tr r="G140" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4090741106</v>
+        <v>#N/A Requesting Data...1783031425</v>
         <stp/>
         <stp>BDP|304889655090792147</stp>
         <tr r="E58" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2501750904</v>
+        <v>#N/A Requesting Data...2527661743</v>
         <stp/>
         <stp>BDP|427627592191043219</stp>
         <tr r="C87" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2230173793</v>
+        <v>#N/A Requesting Data...1418598446</v>
         <stp/>
         <stp>BDP|768711067038142524</stp>
         <tr r="G25" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2623161876</v>
+        <v>#N/A Requesting Data...3788159422</v>
         <stp/>
         <stp>BDP|447365482187669383</stp>
         <tr r="C95" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3383014403</v>
+        <v>#N/A Requesting Data...4140118475</v>
         <stp/>
         <stp>BDP|901925773788783965</stp>
         <tr r="G67" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2742034895</v>
+        <v>#N/A Requesting Data...772544483</v>
         <stp/>
         <stp>BDP|511429594874391764</stp>
         <tr r="G117" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3597773264</v>
+        <v>#N/A Requesting Data...4182151723</v>
         <stp/>
         <stp>BDP|544620567958067604</stp>
         <tr r="C131" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2333718357</v>
+        <v>#N/A Requesting Data...1235115029</v>
         <stp/>
         <stp>BDP|945569483354328027</stp>
         <tr r="C21" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3099950668</v>
+        <v>#N/A Requesting Data...4280471265</v>
         <stp/>
         <stp>BDP|691281527639744142</stp>
         <tr r="E8" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2911352300</v>
+        <v>#N/A Requesting Data...1832172342</v>
         <stp/>
         <stp>BDP|968314719543295935</stp>
         <tr r="E68" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3260874804</v>
+        <v>#N/A Requesting Data...2064194954</v>
         <stp/>
         <stp>BDP|760426044168153386</stp>
         <tr r="G7" s="1"/>
@@ -4917,7 +4923,7 @@
         <v>298</v>
       </c>
       <c r="E9" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -5033,10 +5039,10 @@
         <v>304</v>
       </c>
       <c r="D16" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E16" t="s">
-        <v>306</v>
+        <v>288</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -5067,7 +5073,7 @@
         <v>309</v>
       </c>
       <c r="D18" t="s">
-        <v>310</v>
+        <v>295</v>
       </c>
       <c r="E18" t="s">
         <v>299</v>
@@ -5135,7 +5141,7 @@
         <v>299</v>
       </c>
       <c r="D22" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="E22" t="s">
         <v>298</v>
@@ -5237,7 +5243,7 @@
         <v>323</v>
       </c>
       <c r="D28" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="E28" t="s">
         <v>284</v>
@@ -5288,7 +5294,7 @@
         <v>307</v>
       </c>
       <c r="D31" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E31" t="s">
         <v>314</v>
@@ -5387,13 +5393,13 @@
         <v>18</v>
       </c>
       <c r="C37" t="s">
-        <v>287</v>
+        <v>302</v>
       </c>
       <c r="D37" t="s">
         <v>286</v>
       </c>
       <c r="E37" t="s">
-        <v>305</v>
+        <v>286</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
@@ -5716,7 +5722,7 @@
         <v>316</v>
       </c>
       <c r="E56" t="s">
-        <v>313</v>
+        <v>300</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
@@ -5764,7 +5770,7 @@
         <v>302</v>
       </c>
       <c r="D59" t="s">
-        <v>286</v>
+        <v>331</v>
       </c>
       <c r="E59" t="s">
         <v>286</v>
@@ -5781,7 +5787,7 @@
         <v>301</v>
       </c>
       <c r="D60" t="s">
-        <v>324</v>
+        <v>292</v>
       </c>
       <c r="E60" t="s">
         <v>324</v>
@@ -5897,7 +5903,7 @@
         <v>74</v>
       </c>
       <c r="C67" t="s">
-        <v>302</v>
+        <v>285</v>
       </c>
       <c r="D67" t="s">
         <v>298</v>
@@ -6155,7 +6161,7 @@
         <v>323</v>
       </c>
       <c r="D82" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="E82" t="s">
         <v>299</v>
@@ -6186,7 +6192,7 @@
         <v>200</v>
       </c>
       <c r="C84" t="s">
-        <v>285</v>
+        <v>297</v>
       </c>
       <c r="D84" t="s">
         <v>289</v>
@@ -6549,7 +6555,7 @@
         <v>324</v>
       </c>
       <c r="E105" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.3">
@@ -6730,7 +6736,7 @@
         <v>218</v>
       </c>
       <c r="C116" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="D116" t="s">
         <v>324</v>
@@ -6988,7 +6994,7 @@
         <v>304</v>
       </c>
       <c r="D131" t="s">
-        <v>320</v>
+        <v>305</v>
       </c>
       <c r="E131" t="s">
         <v>288</v>
@@ -7398,7 +7404,7 @@
       </c>
       <c r="G9" t="str">
         <f>_xll.BDP(D9,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
-        <v>B+</v>
+        <v>B</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -7583,11 +7589,11 @@
       </c>
       <c r="F16" t="str">
         <f>_xll.BDP(D16,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>CCC-</v>
+        <v>CCC+</v>
       </c>
       <c r="G16" t="str">
         <f>_xll.BDP(D16,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
-        <v>CCC-</v>
+        <v>CCC</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -7637,7 +7643,7 @@
       </c>
       <c r="F18" t="str">
         <f>_xll.BDP(D18,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>BBB</v>
+        <v>BBB-</v>
       </c>
       <c r="G18" t="str">
         <f>_xll.BDP(D18,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
@@ -7745,7 +7751,7 @@
       </c>
       <c r="F22" t="str">
         <f>_xll.BDP(D22,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>B</v>
+        <v>B+</v>
       </c>
       <c r="G22" t="str">
         <f>_xll.BDP(D22,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
@@ -7907,7 +7913,7 @@
       </c>
       <c r="F28" t="str">
         <f>_xll.BDP(D28,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>BB</v>
+        <v>BB-</v>
       </c>
       <c r="G28" t="str">
         <f>_xll.BDP(D28,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
@@ -7988,7 +7994,7 @@
       </c>
       <c r="F31" t="str">
         <f>_xll.BDP(D31,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>A-</v>
+        <v>A</v>
       </c>
       <c r="G31" t="str">
         <f>_xll.BDP(D31,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
@@ -8146,7 +8152,7 @@
       </c>
       <c r="E37" t="str">
         <f>_xll.BDP(D37,"RTG_MDY_FC_CURR_ISSUER_RATING")</f>
-        <v>Caa3</v>
+        <v>Caa1</v>
       </c>
       <c r="F37" t="str">
         <f>_xll.BDP(D37,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
@@ -8154,7 +8160,7 @@
       </c>
       <c r="G37" t="str">
         <f>_xll.BDP(D37,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
-        <v>CCC+</v>
+        <v>B-</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
@@ -8667,7 +8673,7 @@
       </c>
       <c r="G56" t="str">
         <f>_xll.BDP(D56,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
-        <v>A</v>
+        <v>WD</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
@@ -8744,7 +8750,7 @@
       </c>
       <c r="F59" t="str">
         <f>_xll.BDP(D59,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>B-</v>
+        <v>B- *-</v>
       </c>
       <c r="G59" t="str">
         <f>_xll.BDP(D59,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
@@ -8771,7 +8777,7 @@
       </c>
       <c r="F60" t="str">
         <f>_xll.BDP(D60,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>AA</v>
+        <v>AA+</v>
       </c>
       <c r="G60" t="str">
         <f>_xll.BDP(D60,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
@@ -8956,7 +8962,7 @@
       </c>
       <c r="E67" t="str">
         <f>_xll.BDP(D67,"RTG_MDY_FC_CURR_ISSUER_RATING")</f>
-        <v>Caa1u</v>
+        <v>B3u</v>
       </c>
       <c r="F67" t="str">
         <f>_xll.BDP(D67,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
@@ -9257,7 +9263,7 @@
       </c>
       <c r="F78" t="str">
         <f>_xll.BDP(D78,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>B- *-</v>
+        <v>B-</v>
       </c>
       <c r="G78" t="str">
         <f>_xll.BDP(D78,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
@@ -9365,7 +9371,7 @@
       </c>
       <c r="F82" t="str">
         <f>_xll.BDP(D82,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>BBB-</v>
+        <v>NR</v>
       </c>
       <c r="G82" t="str">
         <f>_xll.BDP(D82,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
@@ -9415,7 +9421,7 @@
       </c>
       <c r="E84" t="str">
         <f>_xll.BDP(D84,"RTG_MDY_FC_CURR_ISSUER_RATING")</f>
-        <v>B3</v>
+        <v>B2</v>
       </c>
       <c r="F84" t="str">
         <f>_xll.BDP(D84,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
@@ -9990,7 +9996,7 @@
       </c>
       <c r="G105" t="str">
         <f>_xll.BDP(D105,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
-        <v>AA</v>
+        <v>AA *-</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.3">
@@ -10148,7 +10154,7 @@
       </c>
       <c r="F111" t="str">
         <f>_xll.BDP(D111,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>CCC+ *</v>
+        <v>CCC+</v>
       </c>
       <c r="G111" t="str">
         <f>_xll.BDP(D111,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
@@ -10279,7 +10285,7 @@
       </c>
       <c r="E116" t="str">
         <f>_xll.BDP(D116,"RTG_MDY_FC_CURR_ISSUER_RATING")</f>
-        <v>A3</v>
+        <v>A2</v>
       </c>
       <c r="F116" t="str">
         <f>_xll.BDP(D116,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
@@ -10688,7 +10694,7 @@
       </c>
       <c r="F131" t="str">
         <f>_xll.BDP(D131,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>SD</v>
+        <v>CCC+</v>
       </c>
       <c r="G131" t="str">
         <f>_xll.BDP(D131,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>

</xml_diff>

<commit_message>
updated public ratings from bbg
</commit_message>
<xml_diff>
--- a/index_bbg_rating_live.xlsx
+++ b/index_bbg_rating_live.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kkhaw\Desktop\credit-rating-deploy\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kaimin Khaw\Desktop\credit-rating-deploy\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{521B1915-DF86-4567-9F0D-3A498D632E17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-72" windowWidth="23256" windowHeight="12456"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="hard_code" sheetId="2" r:id="rId1"/>
@@ -37,7 +38,7 @@
     <definedName name="TreeMap">"TreeMap"</definedName>
     <definedName name="Waterfall">"Waterfall"</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1051,7 +1052,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1111,7 +1112,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1131,1537 +1132,1537 @@
   <volType type="realTimeData">
     <main first="bofaddin.rtdserver">
       <tp t="s">
-        <v>#N/A Requesting Data...4281538805</v>
+        <v>#N/A Requesting Data...3816845956</v>
         <stp/>
         <stp>BDP|13719527809048657439</stp>
         <tr r="E3" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4242699382</v>
+        <v>#N/A Requesting Data...4095047269</v>
         <stp/>
         <stp>BDP|12363409739849183621</stp>
         <tr r="G98" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4223301270</v>
+        <v>#N/A Requesting Data...3650224282</v>
         <stp/>
         <stp>BDP|17606584297068117917</stp>
         <tr r="G105" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4243747063</v>
+        <v>#N/A Requesting Data...3651891288</v>
         <stp/>
         <stp>BDP|12825277506793769973</stp>
         <tr r="F22" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4283279877</v>
+        <v>#N/A Requesting Data...3489037522</v>
         <stp/>
         <stp>BDP|13615906068526188051</stp>
         <tr r="G101" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4282835338</v>
+        <v>#N/A Requesting Data...3913477817</v>
         <stp/>
         <stp>BDP|10912677687245148127</stp>
         <tr r="G106" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4244907434</v>
+        <v>#N/A Requesting Data...3797712885</v>
         <stp/>
         <stp>BDP|16221541486007837625</stp>
         <tr r="G58" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4289212215</v>
+        <v>#N/A Requesting Data...3943981043</v>
         <stp/>
         <stp>BDP|14989839765876665645</stp>
         <tr r="C81" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4289928383</v>
+        <v>#N/A Requesting Data...3629162638</v>
         <stp/>
         <stp>BDP|16792452589360294083</stp>
         <tr r="E11" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4241930810</v>
+        <v>#N/A Requesting Data...3744126319</v>
         <stp/>
         <stp>BDP|16409240184993364568</stp>
         <tr r="E54" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4293600657</v>
+        <v>#N/A Requesting Data...3729583743</v>
         <stp/>
         <stp>BDP|12376141866138693768</stp>
         <tr r="C88" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4266622738</v>
+        <v>#N/A Requesting Data...3939982973</v>
         <stp/>
         <stp>BDP|13146963289471890960</stp>
         <tr r="C18" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4259169197</v>
+        <v>#N/A Requesting Data...3823392801</v>
         <stp/>
         <stp>BDP|10167725043130019931</stp>
         <tr r="C110" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4273819085</v>
+        <v>#N/A Requesting Data...4075829776</v>
         <stp/>
         <stp>BDP|10589422899161895655</stp>
         <tr r="G76" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4267735319</v>
+        <v>#N/A Requesting Data...3799867343</v>
         <stp/>
         <stp>BDP|15228795190517586693</stp>
         <tr r="E84" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4260393429</v>
+        <v>#N/A Requesting Data...3584678721</v>
         <stp/>
         <stp>BDP|10096201946458505444</stp>
         <tr r="G97" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4294805787</v>
+        <v>#N/A Requesting Data...3622708845</v>
         <stp/>
         <stp>BDP|18253401034836307331</stp>
         <tr r="F99" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4265513641</v>
+        <v>#N/A Requesting Data...4271974943</v>
         <stp/>
         <stp>BDP|10867273920449518201</stp>
         <tr r="G71" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4264428759</v>
+        <v>#N/A Requesting Data...3680350095</v>
         <stp/>
         <stp>BDP|14811872563886412749</stp>
         <tr r="E114" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4283156717</v>
+        <v>#N/A Requesting Data...4146820712</v>
         <stp/>
         <stp>BDP|15237334583701669483</stp>
         <tr r="C112" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4270611429</v>
+        <v>#N/A Requesting Data...3832202926</v>
         <stp/>
         <stp>BDP|14006145231309322495</stp>
         <tr r="C65" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4271543903</v>
+        <v>#N/A Requesting Data...4084281335</v>
         <stp/>
         <stp>BDP|14761213634019822741</stp>
         <tr r="G2" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4291679866</v>
+        <v>#N/A Requesting Data...3508138283</v>
         <stp/>
         <stp>BDP|15399231330039360601</stp>
         <tr r="E42" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4278067948</v>
+        <v>#N/A Requesting Data...3916031351</v>
         <stp/>
         <stp>BDP|11120752607359953480</stp>
         <tr r="G61" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4285189688</v>
+        <v>#N/A Requesting Data...4190646809</v>
         <stp/>
         <stp>BDP|15939978441203902037</stp>
         <tr r="C26" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4292634386</v>
+        <v>#N/A Requesting Data...3703052280</v>
         <stp/>
         <stp>BDP|18066043829836356791</stp>
         <tr r="G78" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4294789977</v>
+        <v>#N/A Requesting Data...3571080134</v>
         <stp/>
         <stp>BDP|14168806967588813989</stp>
         <tr r="F77" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4292318761</v>
+        <v>#N/A Requesting Data...3837378225</v>
         <stp/>
         <stp>BDP|18397803367339867766</stp>
         <tr r="F101" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4286674282</v>
+        <v>#N/A Requesting Data...3547763846</v>
         <stp/>
         <stp>BDP|15895803206017416271</stp>
         <tr r="C33" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4292689074</v>
+        <v>#N/A Requesting Data...3808307199</v>
         <stp/>
         <stp>BDP|14908732543227691836</stp>
         <tr r="E94" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4289650716</v>
+        <v>#N/A Requesting Data...3914438069</v>
         <stp/>
         <stp>BDP|12957817799052931996</stp>
         <tr r="E120" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4286903926</v>
+        <v>#N/A Requesting Data...3563550115</v>
         <stp/>
         <stp>BDP|16275205432289392600</stp>
         <tr r="E101" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4288341068</v>
+        <v>#N/A Requesting Data...3957570315</v>
         <stp/>
         <stp>BDP|10407655300028223605</stp>
         <tr r="F47" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4289182940</v>
+        <v>#N/A Requesting Data...4018001458</v>
         <stp/>
         <stp>BDP|14031612538318230186</stp>
         <tr r="C136" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4290663879</v>
+        <v>#N/A Requesting Data...3938613847</v>
         <stp/>
         <stp>BDP|13840587393604095357</stp>
         <tr r="G3" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4293572198</v>
+        <v>#N/A Requesting Data...4090495501</v>
         <stp/>
         <stp>BDP|18397555740376217727</stp>
         <tr r="F17" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4290767945</v>
+        <v>#N/A Requesting Data...4247008007</v>
         <stp/>
         <stp>BDP|15886108592084595196</stp>
         <tr r="F19" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4293067475</v>
+        <v>#N/A Requesting Data...3840167892</v>
         <stp/>
         <stp>BDP|12574943311804341655</stp>
         <tr r="C58" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4293994787</v>
+        <v>#N/A Requesting Data...3704508034</v>
         <stp/>
         <stp>BDP|15276164033266227932</stp>
         <tr r="C121" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4293002775</v>
+        <v>#N/A Requesting Data...3893337354</v>
         <stp/>
         <stp>BDP|11413915902765857449</stp>
         <tr r="C135" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4294791825</v>
+        <v>#N/A Requesting Data...3645419042</v>
         <stp/>
         <stp>BDP|10888161880627674738</stp>
         <tr r="G74" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2506562413</v>
+        <v>#N/A Requesting Data...3804521255</v>
         <stp/>
         <stp>BDP|18252264749434830399</stp>
         <tr r="E91" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3934356438</v>
+        <v>#N/A Requesting Data...4146949027</v>
         <stp/>
         <stp>BDP|16230814927561165496</stp>
         <tr r="C25" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2085942493</v>
+        <v>#N/A Requesting Data...3968324255</v>
         <stp/>
         <stp>BDP|11669407615485914850</stp>
         <tr r="E28" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2234996456</v>
+        <v>#N/A Requesting Data...3899551763</v>
         <stp/>
         <stp>BDP|15385895124225473341</stp>
         <tr r="F89" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2695312321</v>
+        <v>#N/A Requesting Data...4065719701</v>
         <stp/>
         <stp>BDP|16215575297831427265</stp>
         <tr r="G19" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3254501146</v>
+        <v>#N/A Requesting Data...3804110569</v>
         <stp/>
         <stp>BDP|15664489079057139842</stp>
         <tr r="C50" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1979052416</v>
+        <v>#N/A Requesting Data...3902262022</v>
         <stp/>
         <stp>BDP|13556466380534139208</stp>
         <tr r="C63" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...315028421</v>
+        <v>#N/A Requesting Data...4272177644</v>
         <stp/>
         <stp>BDP|12426034393664290636</stp>
         <tr r="G70" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3280205165</v>
+        <v>#N/A Requesting Data...4224208764</v>
         <stp/>
         <stp>BDP|11206974657257798316</stp>
         <tr r="G5" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4176285346</v>
+        <v>#N/A Requesting Data...3788346055</v>
         <stp/>
         <stp>BDP|15687672872765725835</stp>
         <tr r="G133" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...427713182</v>
+        <v>#N/A Requesting Data...4189056389</v>
         <stp/>
         <stp>BDP|10646340980557108540</stp>
         <tr r="G83" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1084929359</v>
+        <v>#N/A Requesting Data...4037353102</v>
         <stp/>
         <stp>BDP|13932387258969800286</stp>
         <tr r="G30" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3063882440</v>
+        <v>#N/A Requesting Data...3832355008</v>
         <stp/>
         <stp>BDP|14685689793557045247</stp>
         <tr r="G11" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1876683399</v>
+        <v>#N/A Requesting Data...4177542026</v>
         <stp/>
         <stp>BDP|11792528289940283264</stp>
         <tr r="G39" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...408436630</v>
+        <v>#N/A Requesting Data...3624115340</v>
         <stp/>
         <stp>BDP|14038814629908297802</stp>
         <tr r="E14" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2653094264</v>
+        <v>#N/A Requesting Data...3937205248</v>
         <stp/>
         <stp>BDP|17960836852555549100</stp>
         <tr r="F79" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...438682416</v>
+        <v>#N/A Requesting Data...3875437268</v>
         <stp/>
         <stp>BDP|12258786923690042954</stp>
         <tr r="G82" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...56462515</v>
+        <v>#N/A Requesting Data...4198141866</v>
         <stp/>
         <stp>BDP|11831892951331348329</stp>
         <tr r="C35" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3574043701</v>
+        <v>#N/A Requesting Data...4083569064</v>
         <stp/>
         <stp>BDP|12634554786653062247</stp>
         <tr r="F34" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4034418762</v>
+        <v>#N/A Requesting Data...3941311581</v>
         <stp/>
         <stp>BDP|10304787173197381988</stp>
         <tr r="G53" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4289880550</v>
+        <v>#N/A Requesting Data...4162557029</v>
         <stp/>
         <stp>BDP|15772343051115104818</stp>
         <tr r="C127" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...299324302</v>
+        <v>#N/A Requesting Data...3871916214</v>
         <stp/>
         <stp>BDP|13619322587163510542</stp>
         <tr r="C45" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2856067250</v>
+        <v>#N/A Requesting Data...4258461547</v>
         <stp/>
         <stp>BDP|13709828003397613269</stp>
         <tr r="C54" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2478454406</v>
+        <v>#N/A Requesting Data...3614397923</v>
         <stp/>
         <stp>BDP|11596891797659679653</stp>
         <tr r="C89" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1412898430</v>
+        <v>#N/A Requesting Data...3618276181</v>
         <stp/>
         <stp>BDP|18339290641951108002</stp>
         <tr r="E17" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...160163862</v>
+        <v>#N/A Requesting Data...3735870737</v>
         <stp/>
         <stp>BDP|10418265688390464525</stp>
         <tr r="E18" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1834675267</v>
+        <v>#N/A Requesting Data...4112855496</v>
         <stp/>
         <stp>BDP|14859691791600738447</stp>
         <tr r="F45" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3389868748</v>
+        <v>#N/A Requesting Data...4186411263</v>
         <stp/>
         <stp>BDP|18255708956124343152</stp>
         <tr r="E26" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1365767767</v>
+        <v>#N/A Requesting Data...3563368796</v>
         <stp/>
         <stp>BDP|16855823919014233436</stp>
         <tr r="F30" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...422104685</v>
+        <v>#N/A Requesting Data...3776757533</v>
         <stp/>
         <stp>BDP|12821872971201299383</stp>
         <tr r="G124" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2091465056</v>
+        <v>#N/A Requesting Data...3724247436</v>
         <stp/>
         <stp>BDP|11466185903217969815</stp>
         <tr r="F33" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3051475109</v>
+        <v>#N/A Requesting Data...3905258434</v>
         <stp/>
         <stp>BDP|13711300257260836914</stp>
         <tr r="C102" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...979650779</v>
+        <v>#N/A Requesting Data...4240444189</v>
         <stp/>
         <stp>BDP|11622318103537999967</stp>
         <tr r="F15" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1710015160</v>
+        <v>#N/A Requesting Data...4132276208</v>
         <stp/>
         <stp>BDP|10597445640754361898</stp>
         <tr r="F50" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2954260565</v>
+        <v>#N/A Requesting Data...4174148150</v>
         <stp/>
         <stp>BDP|13987588094432951117</stp>
         <tr r="E127" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2227858768</v>
+        <v>#N/A Requesting Data...4247251717</v>
         <stp/>
         <stp>BDP|11655961067423868102</stp>
         <tr r="G104" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...781535297</v>
+        <v>#N/A Requesting Data...3647565102</v>
         <stp/>
         <stp>BDP|12468839190466923900</stp>
         <tr r="C20" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2894154755</v>
+        <v>#N/A Requesting Data...4096956498</v>
         <stp/>
         <stp>BDP|18411047804853597705</stp>
         <tr r="C67" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3523597466</v>
+        <v>#N/A Requesting Data...3770824079</v>
         <stp/>
         <stp>BDP|18331339124097518219</stp>
         <tr r="F66" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1178573464</v>
+        <v>#N/A Requesting Data...3864923315</v>
         <stp/>
         <stp>BDP|14983531083496973331</stp>
         <tr r="G132" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3188584140</v>
+        <v>#N/A Requesting Data...4002369305</v>
         <stp/>
         <stp>BDP|14115869171127460078</stp>
         <tr r="G37" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2966647750</v>
+        <v>#N/A Requesting Data...3827515176</v>
         <stp/>
         <stp>BDP|16963038037211063893</stp>
         <tr r="C13" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4005866698</v>
+        <v>#N/A Requesting Data...3744809918</v>
         <stp/>
         <stp>BDP|13900268704084418991</stp>
         <tr r="E37" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1186578925</v>
+        <v>#N/A Requesting Data...4189266437</v>
         <stp/>
         <stp>BDP|16311230542528118454</stp>
         <tr r="E9" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4142762822</v>
+        <v>#N/A Requesting Data...3611571964</v>
         <stp/>
         <stp>BDP|12403550728001134908</stp>
         <tr r="G38" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...219719260</v>
+        <v>#N/A Requesting Data...3788303215</v>
         <stp/>
         <stp>BDP|10528694388950747396</stp>
         <tr r="F80" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2986645018</v>
+        <v>#N/A Requesting Data...4139324937</v>
         <stp/>
         <stp>BDP|17962073596443790028</stp>
         <tr r="F23" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3297457101</v>
+        <v>#N/A Requesting Data...3707920390</v>
         <stp/>
         <stp>BDP|11322749828038387103</stp>
         <tr r="E122" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2457242402</v>
+        <v>#N/A Requesting Data...4148992116</v>
         <stp/>
         <stp>BDP|14872467854648029062</stp>
         <tr r="C75" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...903977434</v>
+        <v>#N/A Requesting Data...3972705673</v>
         <stp/>
         <stp>BDP|14951668809329151689</stp>
         <tr r="E56" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1041824577</v>
+        <v>#N/A Requesting Data...4206311242</v>
         <stp/>
         <stp>BDP|14211231849266296941</stp>
         <tr r="G103" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2852519003</v>
+        <v>#N/A Requesting Data...4071619617</v>
         <stp/>
         <stp>BDP|15282935006718574931</stp>
         <tr r="E92" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2314127336</v>
+        <v>#N/A Requesting Data...4050616347</v>
         <stp/>
         <stp>BDP|16389940868391785591</stp>
         <tr r="C120" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1497348691</v>
+        <v>#N/A Requesting Data...3673247870</v>
         <stp/>
         <stp>BDP|10830300668358540045</stp>
         <tr r="C115" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3217463440</v>
+        <v>#N/A Requesting Data...3799205234</v>
         <stp/>
         <stp>BDP|15417892931237679498</stp>
         <tr r="F8" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4167175547</v>
+        <v>#N/A Requesting Data...3739168411</v>
         <stp/>
         <stp>BDP|13776760394691002167</stp>
         <tr r="C4" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...243359572</v>
+        <v>#N/A Requesting Data...4239561141</v>
         <stp/>
         <stp>BDP|12950924085148446689</stp>
         <tr r="E121" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1032303005</v>
+        <v>#N/A Requesting Data...4034935342</v>
         <stp/>
         <stp>BDP|11202744698684518690</stp>
         <tr r="G111" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2813291994</v>
+        <v>#N/A Requesting Data...3836361376</v>
         <stp/>
         <stp>BDP|11005719894013994183</stp>
         <tr r="C3" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3273660796</v>
+        <v>#N/A Requesting Data...3804331024</v>
         <stp/>
         <stp>BDP|17061881470574956177</stp>
         <tr r="C69" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3882177113</v>
+        <v>#N/A Requesting Data...3889179560</v>
         <stp/>
         <stp>BDP|10195299258766033392</stp>
         <tr r="E90" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4065688802</v>
+        <v>#N/A Requesting Data...3698180825</v>
         <stp/>
         <stp>BDP|17559180385128709479</stp>
         <tr r="E15" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3138392778</v>
+        <v>#N/A Requesting Data...3939296032</v>
         <stp/>
         <stp>BDP|10477087317801173223</stp>
         <tr r="F125" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1263795305</v>
+        <v>#N/A Requesting Data...3675860848</v>
         <stp/>
         <stp>BDP|10431478218456128129</stp>
         <tr r="G32" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3754327315</v>
+        <v>#N/A Requesting Data...4117433921</v>
         <stp/>
         <stp>BDP|12817533695869473568</stp>
         <tr r="C82" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...668955891</v>
+        <v>#N/A Requesting Data...3872054015</v>
         <stp/>
         <stp>BDP|16722436137983528090</stp>
         <tr r="F127" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2617440960</v>
+        <v>#N/A Requesting Data...3775796792</v>
         <stp/>
         <stp>BDP|14949322880769358496</stp>
         <tr r="G16" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1736864264</v>
+        <v>#N/A Requesting Data...3948730926</v>
         <stp/>
         <stp>BDP|12620594347341901004</stp>
         <tr r="C76" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...722782012</v>
+        <v>#N/A Requesting Data...3986309221</v>
         <stp/>
         <stp>BDP|12047021516217693612</stp>
         <tr r="E126" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3179508051</v>
+        <v>#N/A Requesting Data...4047766543</v>
         <stp/>
         <stp>BDP|13612225533853005354</stp>
         <tr r="F102" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...300716337</v>
+        <v>#N/A Requesting Data...4247482710</v>
         <stp/>
         <stp>BDP|11536436753390219250</stp>
         <tr r="F129" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3247968499</v>
+        <v>#N/A Requesting Data...4052593359</v>
         <stp/>
         <stp>BDP|12946334758336119017</stp>
         <tr r="E72" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2921657825</v>
+        <v>#N/A Requesting Data...3869031530</v>
         <stp/>
         <stp>BDP|17733998071078953332</stp>
         <tr r="C23" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4280063119</v>
+        <v>#N/A Requesting Data...4247133900</v>
         <stp/>
         <stp>BDP|16362559715466602618</stp>
         <tr r="F68" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2495972136</v>
+        <v>#N/A Requesting Data...4045388090</v>
         <stp/>
         <stp>BDP|16070475881909673177</stp>
         <tr r="E112" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...480593425</v>
+        <v>#N/A Requesting Data...3627288064</v>
         <stp/>
         <stp>BDP|17590878194950224438</stp>
         <tr r="G87" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1140799514</v>
+        <v>#N/A Requesting Data...4210270437</v>
         <stp/>
         <stp>BDP|12427007793358727164</stp>
         <tr r="F100" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...613996177</v>
+        <v>#N/A Requesting Data...3765301745</v>
         <stp/>
         <stp>BDP|15601293270144483737</stp>
         <tr r="G15" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2053219848</v>
+        <v>#N/A Requesting Data...4018879473</v>
         <stp/>
         <stp>BDP|13723200346810339697</stp>
         <tr r="C38" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...627913633</v>
+        <v>#N/A Requesting Data...3672930451</v>
         <stp/>
         <stp>BDP|18086118189074176643</stp>
         <tr r="E88" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3748970072</v>
+        <v>#N/A Requesting Data...3746500268</v>
         <stp/>
         <stp>BDP|15679917748483251829</stp>
         <tr r="E6" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1513483301</v>
+        <v>#N/A Requesting Data...3649919862</v>
         <stp/>
         <stp>BDP|13421293548936861023</stp>
         <tr r="G66" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2781785852</v>
+        <v>#N/A Requesting Data...4010479008</v>
         <stp/>
         <stp>BDP|10594946509929542325</stp>
         <tr r="F5" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2306473804</v>
+        <v>#N/A Requesting Data...3692317876</v>
         <stp/>
         <stp>BDP|10668212108445960480</stp>
         <tr r="G57" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2139949289</v>
+        <v>#N/A Requesting Data...4275728538</v>
         <stp/>
         <stp>BDP|10103273213286136651</stp>
         <tr r="C6" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2503901128</v>
+        <v>#N/A Requesting Data...4240592956</v>
         <stp/>
         <stp>BDP|11259721862376480554</stp>
         <tr r="G69" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1439001086</v>
+        <v>#N/A Requesting Data...3809236879</v>
         <stp/>
         <stp>BDP|14885566279524266176</stp>
         <tr r="E30" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3165351925</v>
+        <v>#N/A Requesting Data...4070203646</v>
         <stp/>
         <stp>BDP|14519079130534129014</stp>
         <tr r="C49" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...976798771</v>
+        <v>#N/A Requesting Data...4286858991</v>
         <stp/>
         <stp>BDP|14873136635550817546</stp>
         <tr r="G130" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3375761963</v>
+        <v>#N/A Requesting Data...4250123242</v>
         <stp/>
         <stp>BDP|16641457892301341972</stp>
         <tr r="F130" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...873422538</v>
+        <v>#N/A Requesting Data...4245355885</v>
         <stp/>
         <stp>BDP|13231746637163726724</stp>
         <tr r="E7" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...924236668</v>
+        <v>#N/A Requesting Data...4114403224</v>
         <stp/>
         <stp>BDP|12945735048800380256</stp>
         <tr r="G118" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2232869679</v>
+        <v>#N/A Requesting Data...3906496396</v>
         <stp/>
         <stp>BDP|11265248170961260631</stp>
         <tr r="E47" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...355767762</v>
+        <v>#N/A Requesting Data...4274472987</v>
         <stp/>
         <stp>BDP|16351851074029385080</stp>
         <tr r="G35" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1848109280</v>
+        <v>#N/A Requesting Data...4069296952</v>
         <stp/>
         <stp>BDP|11944358991052271970</stp>
         <tr r="C103" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3501155202</v>
+        <v>#N/A Requesting Data...3783093118</v>
         <stp/>
         <stp>BDP|18410981990650283866</stp>
         <tr r="C99" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...401828935</v>
+        <v>#N/A Requesting Data...3738731596</v>
         <stp/>
         <stp>BDP|14383773052580838655</stp>
         <tr r="F104" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2821974899</v>
+        <v>#N/A Requesting Data...3996140545</v>
         <stp/>
         <stp>BDP|10871340643964419300</stp>
         <tr r="F95" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3635348580</v>
+        <v>#N/A Requesting Data...3938129765</v>
         <stp/>
         <stp>BDP|14690280185656044816</stp>
         <tr r="C94" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3519296729</v>
+        <v>#N/A Requesting Data...4002303920</v>
         <stp/>
         <stp>BDP|18305693996456795112</stp>
         <tr r="G80" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2388517896</v>
+        <v>#N/A Requesting Data...4069729934</v>
         <stp/>
         <stp>BDP|16273225567973824127</stp>
         <tr r="C79" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4292377611</v>
+        <v>#N/A Requesting Data...4144126276</v>
         <stp/>
         <stp>BDP|13313129291618997350</stp>
         <tr r="C43" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2368042199</v>
+        <v>#N/A Requesting Data...3686563826</v>
         <stp/>
         <stp>BDP|15444947284180871401</stp>
         <tr r="G27" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1541831443</v>
+        <v>#N/A Requesting Data...4044205316</v>
         <stp/>
         <stp>BDP|12935317504846234704</stp>
         <tr r="F98" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1608344860</v>
+        <v>#N/A Requesting Data...4274595427</v>
         <stp/>
         <stp>BDP|13057895365605005829</stp>
         <tr r="C138" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2532978598</v>
+        <v>#N/A Requesting Data...3739040210</v>
         <stp/>
         <stp>BDP|16160321537943284588</stp>
         <tr r="E76" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2718903413</v>
+        <v>#N/A Requesting Data...4034413668</v>
         <stp/>
         <stp>BDP|10621599828921836610</stp>
         <tr r="C12" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1494994779</v>
+        <v>#N/A Requesting Data...3744218359</v>
         <stp/>
         <stp>BDP|14881076967673386157</stp>
         <tr r="F122" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2325848620</v>
+        <v>#N/A Requesting Data...4076325782</v>
         <stp/>
         <stp>BDP|17321553610055816607</stp>
         <tr r="F96" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4132732032</v>
+        <v>#N/A Requesting Data...4189002484</v>
         <stp/>
         <stp>BDP|12793555755147383546</stp>
         <tr r="F42" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...875791330</v>
+        <v>#N/A Requesting Data...4005512685</v>
         <stp/>
         <stp>BDP|10194327202093986081</stp>
         <tr r="F132" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3164846488</v>
+        <v>#N/A Requesting Data...4020107105</v>
         <stp/>
         <stp>BDP|12798194599768683232</stp>
         <tr r="C42" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1976797481</v>
+        <v>#N/A Requesting Data...4094144469</v>
         <stp/>
         <stp>BDP|15675203172551734114</stp>
         <tr r="F12" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...459810095</v>
+        <v>#N/A Requesting Data...3907866224</v>
         <stp/>
         <stp>BDP|17779010845097021465</stp>
         <tr r="G23" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3618408954</v>
+        <v>#N/A Requesting Data...4218806231</v>
         <stp/>
         <stp>BDP|14698661432127374654</stp>
         <tr r="E53" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2491506460</v>
+        <v>#N/A Requesting Data...3756654010</v>
         <stp/>
         <stp>BDP|16055018629402477686</stp>
         <tr r="F18" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2476945193</v>
+        <v>#N/A Requesting Data...3730340833</v>
         <stp/>
         <stp>BDP|14191015466523343124</stp>
         <tr r="G42" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3515706798</v>
+        <v>#N/A Requesting Data...4112375608</v>
         <stp/>
         <stp>BDP|16690545673604064064</stp>
         <tr r="G6" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...942368492</v>
+        <v>#N/A Requesting Data...3819857333</v>
         <stp/>
         <stp>BDP|11057556593645206836</stp>
         <tr r="E116" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1443171146</v>
+        <v>#N/A Requesting Data...3716252057</v>
         <stp/>
         <stp>BDP|14753168038796700174</stp>
         <tr r="E131" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3240183006</v>
+        <v>#N/A Requesting Data...3781691087</v>
         <stp/>
         <stp>BDP|18400936140157917378</stp>
         <tr r="G108" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...410904291</v>
+        <v>#N/A Requesting Data...3945450046</v>
         <stp/>
         <stp>BDP|11308062409311166143</stp>
         <tr r="F138" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2668032502</v>
+        <v>#N/A Requesting Data...3953479106</v>
         <stp/>
         <stp>BDP|14929251921187622207</stp>
         <tr r="G120" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2575722059</v>
+        <v>#N/A Requesting Data...4112792127</v>
         <stp/>
         <stp>BDP|13312546151322475095</stp>
         <tr r="C117" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2155279298</v>
+        <v>#N/A Requesting Data...4050030875</v>
         <stp/>
         <stp>BDP|10370784365528062849</stp>
         <tr r="G51" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1269219249</v>
+        <v>#N/A Requesting Data...4122459129</v>
         <stp/>
         <stp>BDP|17808503947101138629</stp>
         <tr r="F128" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1999760448</v>
+        <v>#N/A Requesting Data...3969156892</v>
         <stp/>
         <stp>BDP|17640270888515662931</stp>
         <tr r="E20" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2641231122</v>
+        <v>#N/A Requesting Data...3868715031</v>
         <stp/>
         <stp>BDP|17853766030844520642</stp>
         <tr r="F65" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2119696437</v>
+        <v>#N/A Requesting Data...4221020984</v>
         <stp/>
         <stp>BDP|17345319339237647129</stp>
         <tr r="C10" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3180933814</v>
+        <v>#N/A Requesting Data...4265064777</v>
         <stp/>
         <stp>BDP|18428163184190295050</stp>
         <tr r="C48" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1087564142</v>
+        <v>#N/A Requesting Data...3827185946</v>
         <stp/>
         <stp>BDP|11469771160883398201</stp>
         <tr r="G20" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1927762788</v>
+        <v>#N/A Requesting Data...4035164306</v>
         <stp/>
         <stp>BDP|12945229628891094206</stp>
         <tr r="F36" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3239947956</v>
+        <v>#N/A Requesting Data...4102131488</v>
         <stp/>
         <stp>BDP|13088969316699575369</stp>
         <tr r="G17" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...598327478</v>
+        <v>#N/A Requesting Data...3895712082</v>
         <stp/>
         <stp>BDP|14386928546318260068</stp>
         <tr r="C78" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...759352258</v>
+        <v>#N/A Requesting Data...3889918136</v>
         <stp/>
         <stp>BDP|16250000632946565269</stp>
         <tr r="F32" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2330606770</v>
+        <v>#N/A Requesting Data...4239879300</v>
         <stp/>
         <stp>BDP|10062445544650347114</stp>
         <tr r="E69" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2099397601</v>
+        <v>#N/A Requesting Data...3953188457</v>
         <stp/>
         <stp>BDP|16445974490524697317</stp>
         <tr r="F140" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2670499590</v>
+        <v>#N/A Requesting Data...4099177288</v>
         <stp/>
         <stp>BDP|18056984346180923430</stp>
         <tr r="F67" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1388029963</v>
+        <v>#N/A Requesting Data...4035030565</v>
         <stp/>
         <stp>BDP|13607419850307697457</stp>
         <tr r="G55" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3727837507</v>
+        <v>#N/A Requesting Data...4270674298</v>
         <stp/>
         <stp>BDP|17151526894293450943</stp>
         <tr r="E34" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4247745882</v>
+        <v>#N/A Requesting Data...3887337552</v>
         <stp/>
         <stp>BDP|14769233272840536059</stp>
         <tr r="F48" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1845222275</v>
+        <v>#N/A Requesting Data...3810176756</v>
         <stp/>
         <stp>BDP|16347078018142331376</stp>
         <tr r="E59" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3269256939</v>
+        <v>#N/A Requesting Data...4211547554</v>
         <stp/>
         <stp>BDP|12157937398585487157</stp>
         <tr r="F69" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2677249979</v>
+        <v>#N/A Requesting Data...4189389702</v>
         <stp/>
         <stp>BDP|10450024654077121490</stp>
         <tr r="G29" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1726899211</v>
+        <v>#N/A Requesting Data...4184766793</v>
         <stp/>
         <stp>BDP|12405274734177384298</stp>
         <tr r="G109" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1329921153</v>
+        <v>#N/A Requesting Data...3893229532</v>
         <stp/>
         <stp>BDP|11693290023110245727</stp>
         <tr r="F93" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...854339115</v>
+        <v>#N/A Requesting Data...4128699743</v>
         <stp/>
         <stp>BDP|16857915317939051104</stp>
         <tr r="E4" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2332188480</v>
+        <v>#N/A Requesting Data...4237617556</v>
         <stp/>
         <stp>BDP|13092630751014311204</stp>
         <tr r="C29" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...772345592</v>
+        <v>#N/A Requesting Data...3848779969</v>
         <stp/>
         <stp>BDP|16560165422091315234</stp>
         <tr r="E74" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1104159411</v>
+        <v>#N/A Requesting Data...3738883324</v>
         <stp/>
         <stp>BDP|15578620992514708823</stp>
         <tr r="C74" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3611707592</v>
+        <v>#N/A Requesting Data...4173744341</v>
         <stp/>
         <stp>BDP|16311826266949112751</stp>
         <tr r="E137" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1650928770</v>
+        <v>#N/A Requesting Data...4249846499</v>
         <stp/>
         <stp>BDP|12423551309476829732</stp>
         <tr r="E29" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2509466141</v>
+        <v>#N/A Requesting Data...4242242279</v>
         <stp/>
         <stp>BDP|15334425393507822980</stp>
         <tr r="C71" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4157593917</v>
+        <v>#N/A Requesting Data...4004927127</v>
         <stp/>
         <stp>BDP|14187404668490888034</stp>
         <tr r="E115" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2402065436</v>
+        <v>#N/A Requesting Data...3853091647</v>
         <stp/>
         <stp>BDP|14038301256494491076</stp>
         <tr r="E12" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3731901525</v>
+        <v>#N/A Requesting Data...3825811037</v>
         <stp/>
         <stp>BDP|12212063840830333025</stp>
         <tr r="E132" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2379508885</v>
+        <v>#N/A Requesting Data...4268402093</v>
         <stp/>
         <stp>BDP|12411228970299104833</stp>
         <tr r="E40" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...687610854</v>
+        <v>#N/A Requesting Data...4016091007</v>
         <stp/>
         <stp>BDP|11324255971734653659</stp>
         <tr r="G93" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2604241971</v>
+        <v>#N/A Requesting Data...3956111507</v>
         <stp/>
         <stp>BDP|15080702944965265524</stp>
         <tr r="E5" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2313720552</v>
+        <v>#N/A Requesting Data...3888545718</v>
         <stp/>
         <stp>BDP|12709330545317601409</stp>
         <tr r="F78" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2571946984</v>
+        <v>#N/A Requesting Data...3995320252</v>
         <stp/>
         <stp>BDP|17558583635766924170</stp>
         <tr r="C139" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2687247238</v>
+        <v>#N/A Requesting Data...4055848639</v>
         <stp/>
         <stp>BDP|14043797868641345244</stp>
         <tr r="G127" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...824601074</v>
+        <v>#N/A Requesting Data...4294776740</v>
         <stp/>
         <stp>BDP|11097146762171726091</stp>
         <tr r="C125" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3786840278</v>
+        <v>#N/A Requesting Data...3851547992</v>
         <stp/>
         <stp>BDP|10083242995488903402</stp>
         <tr r="E22" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...662024065</v>
+        <v>#N/A Requesting Data...3999713055</v>
         <stp/>
         <stp>BDP|14104003677163905777</stp>
         <tr r="G89" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1506135412</v>
+        <v>#N/A Requesting Data...3897804189</v>
         <stp/>
         <stp>BDP|10493155251505330684</stp>
         <tr r="F113" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3298459031</v>
+        <v>#N/A Requesting Data...4166503751</v>
         <stp/>
         <stp>BDP|17307159600861837050</stp>
         <tr r="C28" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1840326041</v>
+        <v>#N/A Requesting Data...4220456319</v>
         <stp/>
         <stp>BDP|11974207352247436657</stp>
         <tr r="G84" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...470652296</v>
+        <v>#N/A Requesting Data...4220175592</v>
         <stp/>
         <stp>BDP|12417029733397010193</stp>
         <tr r="G129" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3187696211</v>
+        <v>#N/A Requesting Data...3912444600</v>
         <stp/>
         <stp>BDP|13696428749777505366</stp>
         <tr r="C128" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2903772977</v>
+        <v>#N/A Requesting Data...3903960782</v>
         <stp/>
         <stp>BDP|10265435339313984301</stp>
         <tr r="F136" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2883870625</v>
+        <v>#N/A Requesting Data...4279036694</v>
         <stp/>
         <stp>BDP|16742662035804692035</stp>
         <tr r="E24" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2835485463</v>
+        <v>#N/A Requesting Data...3878109756</v>
         <stp/>
         <stp>BDP|13311072247345018521</stp>
         <tr r="E129" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1642508288</v>
+        <v>#N/A Requesting Data...3941616660</v>
         <stp/>
         <stp>BDP|14635385909938704819</stp>
         <tr r="E106" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2400914228</v>
+        <v>#N/A Requesting Data...3814284416</v>
         <stp/>
         <stp>BDP|17965266240553639582</stp>
         <tr r="E10" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2492408394</v>
+        <v>#N/A Requesting Data...3918196002</v>
         <stp/>
         <stp>BDP|14559650107303581628</stp>
         <tr r="C72" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3621123176</v>
+        <v>#N/A Requesting Data...4205271251</v>
         <stp/>
         <stp>BDP|12078771150016496119</stp>
         <tr r="G102" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1991409140</v>
+        <v>#N/A Requesting Data...4166709673</v>
         <stp/>
         <stp>BDP|13437131854538783812</stp>
         <tr r="G22" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4081142123</v>
+        <v>#N/A Requesting Data...4139592345</v>
         <stp/>
         <stp>BDP|11816803688615161347</stp>
         <tr r="E51" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4126194847</v>
+        <v>#N/A Requesting Data...3818072210</v>
         <stp/>
         <stp>BDP|11136233214231371414</stp>
         <tr r="G139" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2978940767</v>
+        <v>#N/A Requesting Data...4174564591</v>
         <stp/>
         <stp>BDP|16387121100332435221</stp>
         <tr r="G96" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3404127902</v>
+        <v>#N/A Requesting Data...4088673050</v>
         <stp/>
         <stp>BDP|10044993787394494110</stp>
         <tr r="C113" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2973637078</v>
+        <v>#N/A Requesting Data...4181640102</v>
         <stp/>
         <stp>BDP|16851432539276999316</stp>
         <tr r="E44" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...803621145</v>
+        <v>#N/A Requesting Data...3783515942</v>
         <stp/>
         <stp>BDP|17514330731974993734</stp>
         <tr r="E65" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2358648386</v>
+        <v>#N/A Requesting Data...3887271210</v>
         <stp/>
         <stp>BDP|13397290692205579908</stp>
         <tr r="G128" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3545675663</v>
+        <v>#N/A Requesting Data...3892825247</v>
         <stp/>
         <stp>BDP|11770519860203890508</stp>
         <tr r="F106" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3016117083</v>
+        <v>#N/A Requesting Data...3944243844</v>
         <stp/>
         <stp>BDP|11828615722360397168</stp>
         <tr r="E71" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4248024259</v>
+        <v>#N/A Requesting Data...3997265139</v>
         <stp/>
         <stp>BDP|12429929188915695292</stp>
         <tr r="F109" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2213616416</v>
+        <v>#N/A Requesting Data...4242216834</v>
         <stp/>
         <stp>BDP|14807781952773549162</stp>
         <tr r="G33" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4078705538</v>
+        <v>#N/A Requesting Data...3926091822</v>
         <stp/>
         <stp>BDP|14141528956866623622</stp>
         <tr r="C134" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3206755032</v>
+        <v>#N/A Requesting Data...3978216436</v>
         <stp/>
         <stp>BDP|11925450918217650729</stp>
         <tr r="F86" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1916871612</v>
+        <v>#N/A Requesting Data...3813271980</v>
         <stp/>
         <stp>BDP|10075353521710450506</stp>
         <tr r="C109" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3407952105</v>
+        <v>#N/A Requesting Data...4099685295</v>
         <stp/>
         <stp>BDP|14507687284196916837</stp>
         <tr r="F6" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1960356371</v>
+        <v>#N/A Requesting Data...4033000623</v>
         <stp/>
         <stp>BDP|17592946715913980887</stp>
         <tr r="F7" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...983071769</v>
+        <v>#N/A Requesting Data...4053137118</v>
         <stp/>
         <stp>BDP|12670343566891576248</stp>
         <tr r="G36" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2706611284</v>
+        <v>#N/A Requesting Data...3937368759</v>
         <stp/>
         <stp>BDP|16059776447550017157</stp>
         <tr r="F63" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1454986582</v>
+        <v>#N/A Requesting Data...4283822391</v>
         <stp/>
         <stp>BDP|13709786759646324310</stp>
         <tr r="F46" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...849074466</v>
+        <v>#N/A Requesting Data...4141590523</v>
         <stp/>
         <stp>BDP|17680007951225535344</stp>
         <tr r="C93" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3125202582</v>
+        <v>#N/A Requesting Data...4252554044</v>
         <stp/>
         <stp>BDP|14249466628496635139</stp>
         <tr r="F26" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2116278067</v>
+        <v>#N/A Requesting Data...4155748843</v>
         <stp/>
         <stp>BDP|12616286245214000526</stp>
         <tr r="C114" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1718762596</v>
+        <v>#N/A Requesting Data...4075932744</v>
         <stp/>
         <stp>BDP|13229487552560837780</stp>
         <tr r="E139" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...794669539</v>
+        <v>#N/A Requesting Data...4283567373</v>
         <stp/>
         <stp>BDP|18412208651713792994</stp>
         <tr r="F118" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2659019485</v>
+        <v>#N/A Requesting Data...4085795259</v>
         <stp/>
         <stp>BDP|16919456577607807790</stp>
         <tr r="G56" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1773924770</v>
+        <v>#N/A Requesting Data...3807507602</v>
         <stp/>
         <stp>BDP|14958917677776306912</stp>
         <tr r="E124" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3272172021</v>
+        <v>#N/A Requesting Data...3803095504</v>
         <stp/>
         <stp>BDP|16906362551851442479</stp>
         <tr r="F14" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1634360491</v>
+        <v>#N/A Requesting Data...3949147125</v>
         <stp/>
         <stp>BDP|13303498173634341154</stp>
         <tr r="G72" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4044351873</v>
+        <v>#N/A Requesting Data...4053607097</v>
         <stp/>
         <stp>BDP|11394026073756494578</stp>
         <tr r="F4" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2089610352</v>
+        <v>#N/A Requesting Data...3833140024</v>
         <stp/>
         <stp>BDP|12821707660430898618</stp>
         <tr r="C40" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...554502583</v>
+        <v>#N/A Requesting Data...4156647236</v>
         <stp/>
         <stp>BDP|12207042919767891145</stp>
         <tr r="G131" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3936254852</v>
+        <v>#N/A Requesting Data...3872237876</v>
         <stp/>
         <stp>BDP|17617562141366516571</stp>
         <tr r="F24" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1533541328</v>
+        <v>#N/A Requesting Data...4280894856</v>
         <stp/>
         <stp>BDP|13776066979946925741</stp>
         <tr r="C90" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4290292627</v>
+        <v>#N/A Requesting Data...4010902473</v>
         <stp/>
         <stp>BDP|15429465971742273156</stp>
         <tr r="E67" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3028729700</v>
+        <v>#N/A Requesting Data...3875965464</v>
         <stp/>
         <stp>BDP|13319017160191784122</stp>
         <tr r="E43" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3016118179</v>
+        <v>#N/A Requesting Data...3961416046</v>
         <stp/>
         <stp>BDP|17197570677470339052</stp>
         <tr r="E33" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...436032487</v>
+        <v>#N/A Requesting Data...4267493647</v>
         <stp/>
         <stp>BDP|18198100188843948773</stp>
         <tr r="G60" s="1"/>
@@ -2669,1801 +2670,1801 @@
     </main>
     <main first="bofaddin.rtdserver">
       <tp t="s">
-        <v>#N/A Requesting Data...518081408</v>
+        <v>#N/A Requesting Data...4022351124</v>
         <stp/>
         <stp>BDP|3930904544763426134</stp>
         <tr r="C55" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3312975017</v>
+        <v>#N/A Requesting Data...4069639197</v>
         <stp/>
         <stp>BDP|7103625188072362707</stp>
         <tr r="E98" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3721352243</v>
+        <v>#N/A Requesting Data...4031489003</v>
         <stp/>
         <stp>BDP|9365312653090978315</stp>
         <tr r="G136" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3296472822</v>
+        <v>#N/A Requesting Data...4166499361</v>
         <stp/>
         <stp>BDP|6412151529379694002</stp>
         <tr r="F110" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2918484837</v>
+        <v>#N/A Requesting Data...3884148691</v>
         <stp/>
         <stp>BDP|6245426297947871034</stp>
         <tr r="C80" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3213940049</v>
+        <v>#N/A Requesting Data...3907106350</v>
         <stp/>
         <stp>BDP|2350385774053258906</stp>
         <tr r="F72" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...723846039</v>
+        <v>#N/A Requesting Data...4122507858</v>
         <stp/>
         <stp>BDP|8530657130876609747</stp>
         <tr r="C44" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3755700195</v>
+        <v>#N/A Requesting Data...4027004288</v>
         <stp/>
         <stp>BDP|7198979431090342164</stp>
         <tr r="E50" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2572649853</v>
+        <v>#N/A Requesting Data...4241712380</v>
         <stp/>
         <stp>BDP|9075300299347332881</stp>
         <tr r="G79" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1752361126</v>
+        <v>#N/A Requesting Data...4017053548</v>
         <stp/>
         <stp>BDP|5029740995104753357</stp>
         <tr r="C111" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...612292400</v>
+        <v>#N/A Requesting Data...4089461803</v>
         <stp/>
         <stp>BDP|8128743572863334748</stp>
         <tr r="C47" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2381951656</v>
+        <v>#N/A Requesting Data...3925988534</v>
         <stp/>
         <stp>BDP|6339719327836450907</stp>
         <tr r="C98" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2993222217</v>
+        <v>#N/A Requesting Data...3868956148</v>
         <stp/>
         <stp>BDP|4200580269163222863</stp>
         <tr r="E25" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1478811038</v>
+        <v>#N/A Requesting Data...4160451860</v>
         <stp/>
         <stp>BDP|5989352249668473659</stp>
         <tr r="G50" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4168175214</v>
+        <v>#N/A Requesting Data...4142169224</v>
         <stp/>
         <stp>BDP|2484433252649720677</stp>
         <tr r="G68" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1754565155</v>
+        <v>#N/A Requesting Data...4257581727</v>
         <stp/>
         <stp>BDP|6249870436562567333</stp>
         <tr r="E49" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1621839680</v>
+        <v>#N/A Requesting Data...4218573975</v>
         <stp/>
         <stp>BDP|9572192910556051262</stp>
         <tr r="E134" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...974651891</v>
+        <v>#N/A Requesting Data...4257976992</v>
         <stp/>
         <stp>BDP|7540551159163224910</stp>
         <tr r="F51" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...733891678</v>
+        <v>#N/A Requesting Data...4092103061</v>
         <stp/>
         <stp>BDP|8451204331587951367</stp>
         <tr r="F52" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3031939181</v>
+        <v>#N/A Requesting Data...4286464242</v>
         <stp/>
         <stp>BDP|3109256470563958869</stp>
         <tr r="C52" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1527204154</v>
+        <v>#N/A Requesting Data...4259193257</v>
         <stp/>
         <stp>BDP|3590543194827878545</stp>
         <tr r="F59" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2357555056</v>
+        <v>#N/A Requesting Data...3875127144</v>
         <stp/>
         <stp>BDP|3009997314886390075</stp>
         <tr r="G100" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2642193557</v>
+        <v>#N/A Requesting Data...4267973180</v>
         <stp/>
         <stp>BDP|4777106988391072114</stp>
         <tr r="F103" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1197602393</v>
+        <v>#N/A Requesting Data...3850797905</v>
         <stp/>
         <stp>BDP|4303401897634933024</stp>
         <tr r="E93" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2603315318</v>
+        <v>#N/A Requesting Data...4016965538</v>
         <stp/>
         <stp>BDP|9055938583773500695</stp>
         <tr r="C34" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3999619995</v>
+        <v>#N/A Requesting Data...3991883534</v>
         <stp/>
         <stp>BDP|1573317174439842142</stp>
         <tr r="E133" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4064223356</v>
+        <v>#N/A Requesting Data...3999414203</v>
         <stp/>
         <stp>BDP|7180318607099335068</stp>
         <tr r="C9" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3206411133</v>
+        <v>#N/A Requesting Data...4102296837</v>
         <stp/>
         <stp>BDP|8371873502449565411</stp>
         <tr r="C62" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4213591357</v>
+        <v>#N/A Requesting Data...4011518437</v>
         <stp/>
         <stp>BDP|9300723062997279226</stp>
         <tr r="C124" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...585915646</v>
+        <v>#N/A Requesting Data...4126019052</v>
         <stp/>
         <stp>BDP|5492561896244379063</stp>
         <tr r="F70" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1002116051</v>
+        <v>#N/A Requesting Data...4274780625</v>
         <stp/>
         <stp>BDP|8460669760190400504</stp>
         <tr r="C27" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1819947569</v>
+        <v>#N/A Requesting Data...4027423853</v>
         <stp/>
         <stp>BDP|7634975275120208406</stp>
         <tr r="C31" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3087356478</v>
+        <v>#N/A Requesting Data...4231847093</v>
         <stp/>
         <stp>BDP|4040591290066838371</stp>
         <tr r="E13" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2242541524</v>
+        <v>#N/A Requesting Data...4204351425</v>
         <stp/>
         <stp>BDP|9247766641156585153</stp>
         <tr r="G94" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3238336452</v>
+        <v>#N/A Requesting Data...3991613694</v>
         <stp/>
         <stp>BDP|7940113982976758589</stp>
         <tr r="E95" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1709438463</v>
+        <v>#N/A Requesting Data...4205399448</v>
         <stp/>
         <stp>BDP|9093620553903200797</stp>
         <tr r="C105" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4135381288</v>
+        <v>#N/A Requesting Data...4059838198</v>
         <stp/>
         <stp>BDP|2405932012622401695</stp>
         <tr r="G77" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1030181717</v>
+        <v>#N/A Requesting Data...4259587909</v>
         <stp/>
         <stp>BDP|9175353808212225665</stp>
         <tr r="C66" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3984799757</v>
+        <v>#N/A Requesting Data...4008268491</v>
         <stp/>
         <stp>BDP|1414608591110891051</stp>
         <tr r="F9" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2658441348</v>
+        <v>#N/A Requesting Data...4290323636</v>
         <stp/>
         <stp>BDP|3649732806419915339</stp>
         <tr r="G14" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3779564969</v>
+        <v>#N/A Requesting Data...4247328065</v>
         <stp/>
         <stp>BDP|7006257261095505888</stp>
         <tr r="F54" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...553895234</v>
+        <v>#N/A Requesting Data...4253009087</v>
         <stp/>
         <stp>BDP|9781989741438009272</stp>
         <tr r="C39" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3323518437</v>
+        <v>#N/A Requesting Data...4234401735</v>
         <stp/>
         <stp>BDP|7532189862547338936</stp>
         <tr r="F58" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1761689657</v>
+        <v>#N/A Requesting Data...4130059556</v>
         <stp/>
         <stp>BDP|4286027170164748985</stp>
         <tr r="G113" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3452668293</v>
+        <v>#N/A Requesting Data...3902461362</v>
         <stp/>
         <stp>BDP|4691882821088256816</stp>
         <tr r="F126" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3641591917</v>
+        <v>#N/A Requesting Data...4142808161</v>
         <stp/>
         <stp>BDP|4974055815239706225</stp>
         <tr r="G110" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2719265765</v>
+        <v>#N/A Requesting Data...4098165729</v>
         <stp/>
         <stp>BDP|5916130291376545539</stp>
         <tr r="F73" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2002845267</v>
+        <v>#N/A Requesting Data...4045440471</v>
         <stp/>
         <stp>BDP|9535646277681935723</stp>
         <tr r="E60" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1704704250</v>
+        <v>#N/A Requesting Data...4234982744</v>
         <stp/>
         <stp>BDP|3472420329653378814</stp>
         <tr r="G4" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2897983389</v>
+        <v>#N/A Requesting Data...4250450725</v>
         <stp/>
         <stp>BDP|9676580711333862054</stp>
         <tr r="E135" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...504095762</v>
+        <v>#N/A Requesting Data...3976131179</v>
         <stp/>
         <stp>BDP|8651287802994649096</stp>
         <tr r="E77" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3560125160</v>
+        <v>#N/A Requesting Data...4047397314</v>
         <stp/>
         <stp>BDP|5552297197720045083</stp>
         <tr r="E118" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3994770493</v>
+        <v>#N/A Requesting Data...4112465068</v>
         <stp/>
         <stp>BDP|6195991527552839107</stp>
         <tr r="C61" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2908490669</v>
+        <v>#N/A Requesting Data...3980898582</v>
         <stp/>
         <stp>BDP|2785537291931900199</stp>
         <tr r="G91" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...751735664</v>
+        <v>#N/A Requesting Data...4089082904</v>
         <stp/>
         <stp>BDP|9875435960971965593</stp>
         <tr r="C11" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1889383436</v>
+        <v>#N/A Requesting Data...3975613910</v>
         <stp/>
         <stp>BDP|5969741853480600831</stp>
         <tr r="E140" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4247879507</v>
+        <v>#N/A Requesting Data...4152716252</v>
         <stp/>
         <stp>BDP|7662972721973338089</stp>
         <tr r="F107" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1085846442</v>
+        <v>#N/A Requesting Data...4185648429</v>
         <stp/>
         <stp>BDP|4282903616430488389</stp>
         <tr r="G9" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3261427135</v>
+        <v>#N/A Requesting Data...4219598074</v>
         <stp/>
         <stp>BDP|6606398548307737925</stp>
         <tr r="C70" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1889545589</v>
+        <v>#N/A Requesting Data...3944257376</v>
         <stp/>
         <stp>BDP|2310021551041423963</stp>
         <tr r="F123" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...476686701</v>
+        <v>#N/A Requesting Data...4259519431</v>
         <stp/>
         <stp>BDP|1666950877162018261</stp>
         <tr r="E87" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4069151528</v>
+        <v>#N/A Requesting Data...3973373957</v>
         <stp/>
         <stp>BDP|6280569068792932854</stp>
         <tr r="C46" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4023058504</v>
+        <v>#N/A Requesting Data...4207711789</v>
         <stp/>
         <stp>BDP|9635152443296662577</stp>
         <tr r="C16" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2816128063</v>
+        <v>#N/A Requesting Data...4230373620</v>
         <stp/>
         <stp>BDP|5935740968278021330</stp>
         <tr r="C96" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4215053680</v>
+        <v>#N/A Requesting Data...4037751711</v>
         <stp/>
         <stp>BDP|8225387168083679130</stp>
         <tr r="E57" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2385728029</v>
+        <v>#N/A Requesting Data...4216800362</v>
         <stp/>
         <stp>BDP|8741792397660502982</stp>
         <tr r="G24" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4004691321</v>
+        <v>#N/A Requesting Data...4159469353</v>
         <stp/>
         <stp>BDP|1988621838892198978</stp>
         <tr r="F82" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3987017588</v>
+        <v>#N/A Requesting Data...4043685399</v>
         <stp/>
         <stp>BDP|5160947801244572083</stp>
         <tr r="C97" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2911829596</v>
+        <v>#N/A Requesting Data...4226971988</v>
         <stp/>
         <stp>BDP|8781684350665372626</stp>
         <tr r="G64" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4087962396</v>
+        <v>#N/A Requesting Data...4099790013</v>
         <stp/>
         <stp>BDP|8866465832365619258</stp>
         <tr r="F120" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4275591433</v>
+        <v>#N/A Requesting Data...4114059929</v>
         <stp/>
         <stp>BDP|1231973558974048121</stp>
         <tr r="E123" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...786492112</v>
+        <v>#N/A Requesting Data...4135742962</v>
         <stp/>
         <stp>BDP|9011959145835954962</stp>
         <tr r="E102" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2471186271</v>
+        <v>#N/A Requesting Data...4068472183</v>
         <stp/>
         <stp>BDP|7048111723254898858</stp>
         <tr r="E70" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1629652438</v>
+        <v>#N/A Requesting Data...4122233878</v>
         <stp/>
         <stp>BDP|7514426398370500271</stp>
         <tr r="F84" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1073851964</v>
+        <v>#N/A Requesting Data...4038493809</v>
         <stp/>
         <stp>BDP|2286847884578687294</stp>
         <tr r="C64" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...991935531</v>
+        <v>#N/A Requesting Data...4222955680</v>
         <stp/>
         <stp>BDP|8581359335587083771</stp>
         <tr r="G40" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1748497322</v>
+        <v>#N/A Requesting Data...4113750653</v>
         <stp/>
         <stp>BDP|9176352611073152053</stp>
         <tr r="G52" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...820948897</v>
+        <v>#N/A Requesting Data...4168649039</v>
         <stp/>
         <stp>BDP|3761613276703138977</stp>
         <tr r="C22" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2470048004</v>
+        <v>#N/A Requesting Data...4117870925</v>
         <stp/>
         <stp>BDP|2402283480247992710</stp>
         <tr r="G65" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1368564087</v>
+        <v>#N/A Requesting Data...3936351462</v>
         <stp/>
         <stp>BDP|2496054182730824314</stp>
         <tr r="F108" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...984842409</v>
+        <v>#N/A Requesting Data...4161932851</v>
         <stp/>
         <stp>BDP|1156198294412416234</stp>
         <tr r="G48" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1724358332</v>
+        <v>#N/A Requesting Data...4005016502</v>
         <stp/>
         <stp>BDP|1935863512592400318</stp>
         <tr r="G99" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3120157438</v>
+        <v>#N/A Requesting Data...4073701666</v>
         <stp/>
         <stp>BDP|1182070188629538920</stp>
         <tr r="F85" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...550341735</v>
+        <v>#N/A Requesting Data...4017956314</v>
         <stp/>
         <stp>BDP|9924697901094165296</stp>
         <tr r="E38" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3279436840</v>
+        <v>#N/A Requesting Data...4132398516</v>
         <stp/>
         <stp>BDP|6412137247758825261</stp>
         <tr r="G10" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2522449051</v>
+        <v>#N/A Requesting Data...3977555051</v>
         <stp/>
         <stp>BDP|6277108296426856136</stp>
         <tr r="G122" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2565148026</v>
+        <v>#N/A Requesting Data...4188975718</v>
         <stp/>
         <stp>BDP|2351176324921816947</stp>
         <tr r="E117" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1373088927</v>
+        <v>#N/A Requesting Data...4039199421</v>
         <stp/>
         <stp>BDP|6406207188846485346</stp>
         <tr r="C37" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3373975656</v>
+        <v>#N/A Requesting Data...3929750383</v>
         <stp/>
         <stp>BDP|8112280367483097628</stp>
         <tr r="F16" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2416176471</v>
+        <v>#N/A Requesting Data...4151832073</v>
         <stp/>
         <stp>BDP|6484624822372932905</stp>
         <tr r="C108" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4232546691</v>
+        <v>#N/A Requesting Data...4016273961</v>
         <stp/>
         <stp>BDP|8605875253514357834</stp>
         <tr r="C116" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4100730872</v>
+        <v>#N/A Requesting Data...3945024096</v>
         <stp/>
         <stp>BDP|2842991807747556512</stp>
         <tr r="E110" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3261368088</v>
+        <v>#N/A Requesting Data...4099960042</v>
         <stp/>
         <stp>BDP|1377759003508711718</stp>
         <tr r="E55" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...595397678</v>
+        <v>#N/A Requesting Data...4027482634</v>
         <stp/>
         <stp>BDP|1711361391887412536</stp>
         <tr r="G47" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1532257708</v>
+        <v>#N/A Requesting Data...4018838460</v>
         <stp/>
         <stp>BDP|4564815655442574234</stp>
         <tr r="F114" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3375130925</v>
+        <v>#N/A Requesting Data...3983128728</v>
         <stp/>
         <stp>BDP|6557751567646791843</stp>
         <tr r="C85" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2553465493</v>
+        <v>#N/A Requesting Data...4176442635</v>
         <stp/>
         <stp>BDP|5018226780961297742</stp>
         <tr r="E138" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1123431736</v>
+        <v>#N/A Requesting Data...4009546707</v>
         <stp/>
         <stp>BDP|7190582290036507495</stp>
         <tr r="E48" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3465237305</v>
+        <v>#N/A Requesting Data...4231456640</v>
         <stp/>
         <stp>BDP|7268732641219205478</stp>
         <tr r="F111" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3017135004</v>
+        <v>#N/A Requesting Data...4029290847</v>
         <stp/>
         <stp>BDP|5085458293997400582</stp>
         <tr r="C30" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2092337772</v>
+        <v>#N/A Requesting Data...4077514757</v>
         <stp/>
         <stp>BDP|2916061605678582044</stp>
         <tr r="E27" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2641737701</v>
+        <v>#N/A Requesting Data...3950731348</v>
         <stp/>
         <stp>BDP|5645196194854205325</stp>
         <tr r="E19" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2731811761</v>
+        <v>#N/A Requesting Data...4078498832</v>
         <stp/>
         <stp>BDP|8929421222763426766</stp>
         <tr r="F112" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1718300892</v>
+        <v>#N/A Requesting Data...4026179511</v>
         <stp/>
         <stp>BDP|2815946348173965667</stp>
         <tr r="C137" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1439557279</v>
+        <v>#N/A Requesting Data...4288950564</v>
         <stp/>
         <stp>BDP|6645611732949919042</stp>
         <tr r="G95" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2104998059</v>
+        <v>#N/A Requesting Data...4005353022</v>
         <stp/>
         <stp>BDP|8744658502964028082</stp>
         <tr r="F139" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1747626743</v>
+        <v>#N/A Requesting Data...4226802722</v>
         <stp/>
         <stp>BDP|4077907452745230782</stp>
         <tr r="C130" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3879305424</v>
+        <v>#N/A Requesting Data...4084912509</v>
         <stp/>
         <stp>BDP|8975856381415089739</stp>
         <tr r="E75" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...796117279</v>
+        <v>#N/A Requesting Data...3981563839</v>
         <stp/>
         <stp>BDP|5738611839292209825</stp>
         <tr r="G107" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1545288890</v>
+        <v>#N/A Requesting Data...4231967173</v>
         <stp/>
         <stp>BDP|4996818111432201578</stp>
         <tr r="G134" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1581317174</v>
+        <v>#N/A Requesting Data...4160735711</v>
         <stp/>
         <stp>BDP|5458032582021895609</stp>
         <tr r="E89" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4256604020</v>
+        <v>#N/A Requesting Data...4267357478</v>
         <stp/>
         <stp>BDP|2612461303954522846</stp>
         <tr r="F21" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2798959077</v>
+        <v>#N/A Requesting Data...4277812208</v>
         <stp/>
         <stp>BDP|5852840000806674187</stp>
         <tr r="F75" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2116181778</v>
+        <v>#N/A Requesting Data...4281717648</v>
         <stp/>
         <stp>BDP|7947641811679527399</stp>
         <tr r="G13" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3293266350</v>
+        <v>#N/A Requesting Data...4119601687</v>
         <stp/>
         <stp>BDP|8407769428857900025</stp>
         <tr r="C132" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3190428866</v>
+        <v>#N/A Requesting Data...4258051371</v>
         <stp/>
         <stp>BDP|1313714864639868399</stp>
         <tr r="F87" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1171654374</v>
+        <v>#N/A Requesting Data...4250660311</v>
         <stp/>
         <stp>BDP|2531298252748844733</stp>
         <tr r="F115" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2618312757</v>
+        <v>#N/A Requesting Data...4197585095</v>
         <stp/>
         <stp>BDP|8965389266391509672</stp>
         <tr r="C41" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2937843852</v>
+        <v>#N/A Requesting Data...4244768423</v>
         <stp/>
         <stp>BDP|9146373380128430189</stp>
         <tr r="F60" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3726882109</v>
+        <v>#N/A Requesting Data...4156801656</v>
         <stp/>
         <stp>BDP|8769626454200391097</stp>
         <tr r="G85" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3690847788</v>
+        <v>#N/A Requesting Data...4117291157</v>
         <stp/>
         <stp>BDP|7701346097304455298</stp>
         <tr r="C73" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3881378377</v>
+        <v>#N/A Requesting Data...4032513933</v>
         <stp/>
         <stp>BDP|1201589979318261083</stp>
         <tr r="G123" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3905305442</v>
+        <v>#N/A Requesting Data...4180526603</v>
         <stp/>
         <stp>BDP|9994425762708075853</stp>
         <tr r="G88" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1680813820</v>
+        <v>#N/A Requesting Data...4166208937</v>
         <stp/>
         <stp>BDP|8238868892513701135</stp>
         <tr r="G137" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2422385173</v>
+        <v>#N/A Requesting Data...4286484058</v>
         <stp/>
         <stp>BDP|3321556007464177923</stp>
         <tr r="E109" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1662561277</v>
+        <v>#N/A Requesting Data...4194764974</v>
         <stp/>
         <stp>BDP|8367368187378355023</stp>
         <tr r="F64" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2708459257</v>
+        <v>#N/A Requesting Data...4075283475</v>
         <stp/>
         <stp>BDP|9054142235387080711</stp>
         <tr r="F11" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1876545857</v>
+        <v>#N/A Requesting Data...4003466960</v>
         <stp/>
         <stp>BDP|4797724273716399932</stp>
         <tr r="C5" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1089566942</v>
+        <v>#N/A Requesting Data...4273634741</v>
         <stp/>
         <stp>BDP|3084971212582403246</stp>
         <tr r="F121" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2993439464</v>
+        <v>#N/A Requesting Data...4037624894</v>
         <stp/>
         <stp>BDP|6948762204713990690</stp>
         <tr r="G90" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1879853452</v>
+        <v>#N/A Requesting Data...4166762068</v>
         <stp/>
         <stp>BDP|1832764578595986067</stp>
         <tr r="G119" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2713902386</v>
+        <v>#N/A Requesting Data...4176824685</v>
         <stp/>
         <stp>BDP|4156639623951685595</stp>
         <tr r="F13" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3045217043</v>
+        <v>#N/A Requesting Data...4229648138</v>
         <stp/>
         <stp>BDP|5919761437851372455</stp>
         <tr r="C2" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2042070077</v>
+        <v>#N/A Requesting Data...4272773423</v>
         <stp/>
         <stp>BDP|1551339666687413790</stp>
         <tr r="F40" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3020176732</v>
+        <v>#N/A Requesting Data...4246468765</v>
         <stp/>
         <stp>BDP|6420437202397070174</stp>
         <tr r="C8" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2307001691</v>
+        <v>#N/A Requesting Data...4209695139</v>
         <stp/>
         <stp>BDP|1708381902825815365</stp>
         <tr r="C101" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3739861855</v>
+        <v>#N/A Requesting Data...4267561128</v>
         <stp/>
         <stp>BDP|4945796250777738578</stp>
         <tr r="G21" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2737792707</v>
+        <v>#N/A Requesting Data...4254408025</v>
         <stp/>
         <stp>BDP|6746841414412327938</stp>
         <tr r="G75" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3452257742</v>
+        <v>#N/A Requesting Data...4273855170</v>
         <stp/>
         <stp>BDP|1709445403856801620</stp>
         <tr r="E85" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3175338502</v>
+        <v>#N/A Requesting Data...4202467817</v>
         <stp/>
         <stp>BDP|9398823419477440265</stp>
         <tr r="G125" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3653286519</v>
+        <v>#N/A Requesting Data...4137424540</v>
         <stp/>
         <stp>BDP|3430878723724827801</stp>
         <tr r="G41" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1933149826</v>
+        <v>#N/A Requesting Data...4257826889</v>
         <stp/>
         <stp>BDP|9698422803149077198</stp>
         <tr r="C100" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1153823662</v>
+        <v>#N/A Requesting Data...4206277587</v>
         <stp/>
         <stp>BDP|2887002514665714363</stp>
         <tr r="G59" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4135634195</v>
+        <v>#N/A Requesting Data...4157952819</v>
         <stp/>
         <stp>BDP|2668814054578766269</stp>
         <tr r="E31" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3520025410</v>
+        <v>#N/A Requesting Data...4112246269</v>
         <stp/>
         <stp>BDP|8894702939828266110</stp>
         <tr r="C7" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2988772910</v>
+        <v>#N/A Requesting Data...4203531456</v>
         <stp/>
         <stp>BDP|3410885660260666884</stp>
         <tr r="E64" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1568660127</v>
+        <v>#N/A Requesting Data...4267429708</v>
         <stp/>
         <stp>BDP|3658713905400418152</stp>
         <tr r="E35" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3230746206</v>
+        <v>#N/A Requesting Data...4119355036</v>
         <stp/>
         <stp>BDP|7570300716478486864</stp>
         <tr r="E32" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3645675523</v>
+        <v>#N/A Requesting Data...4244957836</v>
         <stp/>
         <stp>BDP|7851492951527237434</stp>
         <tr r="E52" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2586454802</v>
+        <v>#N/A Requesting Data...4155343763</v>
         <stp/>
         <stp>BDP|7352242467910007671</stp>
         <tr r="F124" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1720337171</v>
+        <v>#N/A Requesting Data...4068336164</v>
         <stp/>
         <stp>BDP|5657563513753480721</stp>
         <tr r="E80" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2876498037</v>
+        <v>#N/A Requesting Data...4248789743</v>
         <stp/>
         <stp>BDP|5976587264538865878</stp>
         <tr r="E62" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3573779692</v>
+        <v>#N/A Requesting Data...4200973640</v>
         <stp/>
         <stp>BDP|7151318027339523982</stp>
         <tr r="F91" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2271282359</v>
+        <v>#N/A Requesting Data...4119748761</v>
         <stp/>
         <stp>BDP|1896477110772260049</stp>
         <tr r="C91" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2711614910</v>
+        <v>#N/A Requesting Data...4104427476</v>
         <stp/>
         <stp>BDP|4252725967471187287</stp>
         <tr r="F44" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1663092124</v>
+        <v>#N/A Requesting Data...4058511648</v>
         <stp/>
         <stp>BDP|6943451920864586278</stp>
         <tr r="C118" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3384823905</v>
+        <v>#N/A Requesting Data...4176203767</v>
         <stp/>
         <stp>BDP|5838113265174067025</stp>
         <tr r="F39" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1151104038</v>
+        <v>#N/A Requesting Data...4141948926</v>
         <stp/>
         <stp>BDP|3456718228377624745</stp>
         <tr r="E111" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2871425608</v>
+        <v>#N/A Requesting Data...4200192575</v>
         <stp/>
         <stp>BDP|5917425194519245724</stp>
         <tr r="E79" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...905661700</v>
+        <v>#N/A Requesting Data...4208242432</v>
         <stp/>
         <stp>BDP|6787533358407016713</stp>
         <tr r="F135" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2005895380</v>
+        <v>#N/A Requesting Data...4189393266</v>
         <stp/>
         <stp>BDP|5576451913756991076</stp>
         <tr r="E16" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4019845859</v>
+        <v>#N/A Requesting Data...4112858134</v>
         <stp/>
         <stp>BDP|5284390591628042184</stp>
         <tr r="C24" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2086988448</v>
+        <v>#N/A Requesting Data...4239142132</v>
         <stp/>
         <stp>BDP|5412037028917536689</stp>
         <tr r="G115" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4133588642</v>
+        <v>#N/A Requesting Data...4275996232</v>
         <stp/>
         <stp>BDP|8966942938724477029</stp>
         <tr r="C15" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2017128733</v>
+        <v>#N/A Requesting Data...4252990884</v>
         <stp/>
         <stp>BDP|2938144706552859709</stp>
         <tr r="G81" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3595983902</v>
+        <v>#N/A Requesting Data...4259827222</v>
         <stp/>
         <stp>BDP|3632949480676633244</stp>
         <tr r="F31" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2876852706</v>
+        <v>#N/A Requesting Data...4193790864</v>
         <stp/>
         <stp>BDP|3513418606797579639</stp>
         <tr r="F90" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3154671867</v>
+        <v>#N/A Requesting Data...4203915265</v>
         <stp/>
         <stp>BDP|1733520919261908213</stp>
         <tr r="G73" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3740638374</v>
+        <v>#N/A Requesting Data...4170929934</v>
         <stp/>
         <stp>BDP|8368969127023380651</stp>
         <tr r="F28" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3452678272</v>
+        <v>#N/A Requesting Data...4237307020</v>
         <stp/>
         <stp>BDP|7172716621593553717</stp>
         <tr r="F53" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4113270740</v>
+        <v>#N/A Requesting Data...4291420951</v>
         <stp/>
         <stp>BDP|2954250373819174944</stp>
         <tr r="F119" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2174932365</v>
+        <v>#N/A Requesting Data...4063412987</v>
         <stp/>
         <stp>BDP|4728287753511799518</stp>
         <tr r="F3" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1991476781</v>
+        <v>#N/A Requesting Data...4291876220</v>
         <stp/>
         <stp>BDP|6348617969513327227</stp>
         <tr r="E104" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3129896262</v>
+        <v>#N/A Requesting Data...4125441381</v>
         <stp/>
         <stp>BDP|7694099704858685831</stp>
         <tr r="C107" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...711748480</v>
+        <v>#N/A Requesting Data...4231448465</v>
         <stp/>
         <stp>BDP|4106834752526835861</stp>
         <tr r="F55" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1915963077</v>
+        <v>#N/A Requesting Data...4157471011</v>
         <stp/>
         <stp>BDP|7951337561756108354</stp>
         <tr r="G112" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2534670081</v>
+        <v>#N/A Requesting Data...4171929583</v>
         <stp/>
         <stp>BDP|5468867501418549294</stp>
         <tr r="E86" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2198089130</v>
+        <v>#N/A Requesting Data...4172867652</v>
         <stp/>
         <stp>BDP|4546740053823447251</stp>
         <tr r="C32" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1731885443</v>
+        <v>#N/A Requesting Data...4180571637</v>
         <stp/>
         <stp>BDP|7484527599745538990</stp>
         <tr r="F76" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3497278369</v>
+        <v>#N/A Requesting Data...4189342241</v>
         <stp/>
         <stp>BDP|5578475423865159117</stp>
         <tr r="E61" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3301520664</v>
+        <v>#N/A Requesting Data...4219392672</v>
         <stp/>
         <stp>BDP|6158107237024797760</stp>
         <tr r="E45" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2507934999</v>
+        <v>#N/A Requesting Data...4127251643</v>
         <stp/>
         <stp>BDP|4143076943390197735</stp>
         <tr r="F97" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3774029430</v>
+        <v>#N/A Requesting Data...4185528837</v>
         <stp/>
         <stp>BDP|1762196091349932721</stp>
         <tr r="E82" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...760238303</v>
+        <v>#N/A Requesting Data...4127729697</v>
         <stp/>
         <stp>BDP|4189169184528349241</stp>
         <tr r="F137" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2711260551</v>
+        <v>#N/A Requesting Data...4079951074</v>
         <stp/>
         <stp>BDP|9103140635044368872</stp>
         <tr r="F29" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1188475633</v>
+        <v>#N/A Requesting Data...4282998495</v>
         <stp/>
         <stp>BDP|5519603296584718917</stp>
         <tr r="G54" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2923461068</v>
+        <v>#N/A Requesting Data...4214642279</v>
         <stp/>
         <stp>BDP|1156250824766982737</stp>
         <tr r="G44" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2782375172</v>
+        <v>#N/A Requesting Data...4137439241</v>
         <stp/>
         <stp>BDP|6031605254431729496</stp>
         <tr r="G86" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1562793937</v>
+        <v>#N/A Requesting Data...4264050646</v>
         <stp/>
         <stp>BDP|2649489454114394728</stp>
         <tr r="C14" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3678833377</v>
+        <v>#N/A Requesting Data...4087541293</v>
         <stp/>
         <stp>BDP|8999377595616850481</stp>
         <tr r="E108" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2251178461</v>
+        <v>#N/A Requesting Data...4223326231</v>
         <stp/>
         <stp>BDP|8988928209665280487</stp>
         <tr r="F71" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2187063806</v>
+        <v>#N/A Requesting Data...4176462673</v>
         <stp/>
         <stp>BDP|8368023487691952119</stp>
         <tr r="F88" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2814852972</v>
+        <v>#N/A Requesting Data...4139621457</v>
         <stp/>
         <stp>BDP|5199287207907438042</stp>
         <tr r="E66" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3792145531</v>
+        <v>#N/A Requesting Data...4112277110</v>
         <stp/>
         <stp>BDP|7460099446995728631</stp>
         <tr r="F134" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3829242541</v>
+        <v>#N/A Requesting Data...4114571125</v>
         <stp/>
         <stp>BDP|6160638673325976246</stp>
         <tr r="C104" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1431281087</v>
+        <v>#N/A Requesting Data...4224018423</v>
         <stp/>
         <stp>BDP|5660731962530222490</stp>
         <tr r="E128" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3961437347</v>
+        <v>#N/A Requesting Data...4201834557</v>
         <stp/>
         <stp>BDP|3355023726294311595</stp>
         <tr r="G114" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2270856093</v>
+        <v>#N/A Requesting Data...4294317189</v>
         <stp/>
         <stp>BDP|5604474461391860653</stp>
         <tr r="E130" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3875016615</v>
+        <v>#N/A Requesting Data...4086032759</v>
         <stp/>
         <stp>BDP|3542140114402066179</stp>
         <tr r="E78" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1435459493</v>
+        <v>#N/A Requesting Data...4119453122</v>
         <stp/>
         <stp>BDP|2942496252996870592</stp>
         <tr r="G121" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4156512207</v>
+        <v>#N/A Requesting Data...4232270523</v>
         <stp/>
         <stp>BDP|1823820926283534897</stp>
         <tr r="G18" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1044844626</v>
+        <v>#N/A Requesting Data...4119105927</v>
         <stp/>
         <stp>BDP|3716189405712826043</stp>
         <tr r="G92" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1833322969</v>
+        <v>#N/A Requesting Data...4278595054</v>
         <stp/>
         <stp>BDP|3228146609442097080</stp>
         <tr r="C140" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4086450329</v>
+        <v>#N/A Requesting Data...4258063997</v>
         <stp/>
         <stp>BDP|9344147089140006098</stp>
         <tr r="E83" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2427302753</v>
+        <v>#N/A Requesting Data...4217950400</v>
         <stp/>
         <stp>BDP|6993061706081965773</stp>
         <tr r="F81" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3238679746</v>
+        <v>#N/A Requesting Data...4142595503</v>
         <stp/>
         <stp>BDP|6176792116871092198</stp>
         <tr r="C68" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3780260838</v>
+        <v>#N/A Requesting Data...4265830559</v>
         <stp/>
         <stp>BDP|7185432584822399912</stp>
         <tr r="F131" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3945989859</v>
+        <v>#N/A Requesting Data...4265041281</v>
         <stp/>
         <stp>BDP|8280856169194643320</stp>
         <tr r="G49" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3896284611</v>
+        <v>#N/A Requesting Data...4283273113</v>
         <stp/>
         <stp>BDP|9399109618929306123</stp>
         <tr r="F37" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1268168318</v>
+        <v>#N/A Requesting Data...4254028476</v>
         <stp/>
         <stp>BDP|6669663699409638145</stp>
         <tr r="C123" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3962840489</v>
+        <v>#N/A Requesting Data...4168049353</v>
         <stp/>
         <stp>BDP|6175693122901836298</stp>
         <tr r="C36" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1208355585</v>
+        <v>#N/A Requesting Data...4129673272</v>
         <stp/>
         <stp>BDP|8135075327118072391</stp>
         <tr r="C17" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1005430097</v>
+        <v>#N/A Requesting Data...4119401115</v>
         <stp/>
         <stp>BDP|5726291712345411206</stp>
         <tr r="G28" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3425673010</v>
+        <v>#N/A Requesting Data...4239858019</v>
         <stp/>
         <stp>BDP|8698973352783506690</stp>
         <tr r="F25" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3844235823</v>
+        <v>#N/A Requesting Data...4206039715</v>
         <stp/>
         <stp>BDP|5493604681742158862</stp>
         <tr r="G63" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1732042222</v>
+        <v>#N/A Requesting Data...4167232645</v>
         <stp/>
         <stp>BDP|3239104742287612040</stp>
         <tr r="E39" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3393203262</v>
+        <v>#N/A Requesting Data...4120670895</v>
         <stp/>
         <stp>BDP|3381147726641663059</stp>
         <tr r="C122" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1011684232</v>
+        <v>#N/A Requesting Data...4109648394</v>
         <stp/>
         <stp>BDP|6625906764329795167</stp>
         <tr r="F56" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3929985876</v>
+        <v>#N/A Requesting Data...4120558413</v>
         <stp/>
         <stp>BDP|3325218238213801010</stp>
         <tr r="F57" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2856733874</v>
+        <v>#N/A Requesting Data...4123567683</v>
         <stp/>
         <stp>BDP|1313137390988032037</stp>
         <tr r="C83" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2350954742</v>
+        <v>#N/A Requesting Data...4253647360</v>
         <stp/>
         <stp>BDP|3702733300853619616</stp>
         <tr r="G34" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2975749398</v>
+        <v>#N/A Requesting Data...4120070895</v>
         <stp/>
         <stp>BDP|8558611930018338475</stp>
         <tr r="F35" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3437496015</v>
+        <v>#N/A Requesting Data...4209765721</v>
         <stp/>
         <stp>BDP|5387098906493173798</stp>
         <tr r="G62" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2816734399</v>
+        <v>#N/A Requesting Data...4267267836</v>
         <stp/>
         <stp>BDP|1951038018907673608</stp>
         <tr r="C126" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4026968796</v>
+        <v>#N/A Requesting Data...4255925101</v>
         <stp/>
         <stp>BDP|9253802402770546012</stp>
         <tr r="F74" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3943826564</v>
+        <v>#N/A Requesting Data...4227138159</v>
         <stp/>
         <stp>BDP|1884505914021260664</stp>
         <tr r="E96" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1812095089</v>
+        <v>#N/A Requesting Data...4241242553</v>
         <stp/>
         <stp>BDP|3540127028674193608</stp>
         <tr r="F94" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3079863195</v>
+        <v>#N/A Requesting Data...4125148106</v>
         <stp/>
         <stp>BDP|5372375359741187031</stp>
         <tr r="F27" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...989572123</v>
+        <v>#N/A Requesting Data...4267057905</v>
         <stp/>
         <stp>BDP|5121625602631825066</stp>
         <tr r="E81" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3130239438</v>
+        <v>#N/A Requesting Data...4279739791</v>
         <stp/>
         <stp>BDP|5282708515920897138</stp>
         <tr r="F43" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2271172753</v>
+        <v>#N/A Requesting Data...4285292740</v>
         <stp/>
         <stp>BDP|1250299291741371958</stp>
         <tr r="G31" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1755087098</v>
+        <v>#N/A Requesting Data...4131346967</v>
         <stp/>
         <stp>BDP|4253176148933327033</stp>
         <tr r="C133" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4049502931</v>
+        <v>#N/A Requesting Data...4148382658</v>
         <stp/>
         <stp>BDP|9704751602229087502</stp>
         <tr r="F49" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...854290810</v>
+        <v>#N/A Requesting Data...4162047546</v>
         <stp/>
         <stp>BDP|6775233901286469015</stp>
         <tr r="E125" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1120715169</v>
+        <v>#N/A Requesting Data...4287263017</v>
         <stp/>
         <stp>BDP|7918289416910309647</stp>
         <tr r="C56" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2441058251</v>
+        <v>#N/A Requesting Data...4252468696</v>
         <stp/>
         <stp>BDP|3731272815900600241</stp>
         <tr r="C53" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3534989116</v>
+        <v>#N/A Requesting Data...4277653275</v>
         <stp/>
         <stp>BDP|1685459166489439868</stp>
         <tr r="F133" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1142040634</v>
+        <v>#N/A Requesting Data...4150412870</v>
         <stp/>
         <stp>BDP|2506644172580171154</stp>
         <tr r="C119" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1374031940</v>
+        <v>#N/A Requesting Data...4198122017</v>
         <stp/>
         <stp>BDP|1995353227627490580</stp>
         <tr r="E119" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3205491158</v>
+        <v>#N/A Requesting Data...4281135447</v>
         <stp/>
         <stp>BDP|9173868178561206592</stp>
         <tr r="C77" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2917154479</v>
+        <v>#N/A Requesting Data...4223905585</v>
         <stp/>
         <stp>BDP|4008096672221657096</stp>
         <tr r="G43" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2574984111</v>
+        <v>#N/A Requesting Data...4248063273</v>
         <stp/>
         <stp>BDP|5434663182001395869</stp>
         <tr r="E107" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1499522446</v>
+        <v>#N/A Requesting Data...4139740414</v>
         <stp/>
         <stp>BDP|8686279502629263146</stp>
         <tr r="C129" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2107797109</v>
+        <v>#N/A Requesting Data...4253412452</v>
         <stp/>
         <stp>BDP|4576300957588172984</stp>
         <tr r="E63" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1729453523</v>
+        <v>#N/A Requesting Data...4148698769</v>
         <stp/>
         <stp>BDP|7469671678835895086</stp>
         <tr r="E2" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1838897942</v>
+        <v>#N/A Requesting Data...4238657401</v>
         <stp/>
         <stp>BDP|5444751401066968714</stp>
         <tr r="E73" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1086082105</v>
+        <v>#N/A Requesting Data...4287934330</v>
         <stp/>
         <stp>BDP|2824124077350027748</stp>
         <tr r="E136" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1391433013</v>
+        <v>#N/A Requesting Data...4163038912</v>
         <stp/>
         <stp>BDP|3708851985886704699</stp>
         <tr r="C19" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3634805172</v>
+        <v>#N/A Requesting Data...4264651497</v>
         <stp/>
         <stp>BDP|1006071828475585561</stp>
         <tr r="F116" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2062177258</v>
+        <v>#N/A Requesting Data...4162900400</v>
         <stp/>
         <stp>BDP|1086712249007771639</stp>
         <tr r="G26" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3985107186</v>
+        <v>#N/A Requesting Data...4248868117</v>
         <stp/>
         <stp>BDP|6634730869724168016</stp>
         <tr r="E103" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2415887883</v>
+        <v>#N/A Requesting Data...4254238134</v>
         <stp/>
         <stp>BDP|3520366017777816505</stp>
         <tr r="E97" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2087003033</v>
+        <v>#N/A Requesting Data...4156387327</v>
         <stp/>
         <stp>BDP|2995135217932647367</stp>
         <tr r="F105" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3347567706</v>
+        <v>#N/A Requesting Data...4223602821</v>
         <stp/>
         <stp>BDP|3565057922625094707</stp>
         <tr r="G45" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2506305386</v>
+        <v>#N/A Requesting Data...4231966456</v>
         <stp/>
         <stp>BDP|1485569542807651461</stp>
         <tr r="C86" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1274587287</v>
+        <v>#N/A Requesting Data...4241602911</v>
         <stp/>
         <stp>BDP|1159006460850353421</stp>
         <tr r="E46" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2654480716</v>
+        <v>#N/A Requesting Data...4247325885</v>
         <stp/>
         <stp>BDP|5113311422502283510</stp>
         <tr r="C84" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2171277543</v>
+        <v>#N/A Requesting Data...4209923271</v>
         <stp/>
         <stp>BDP|4420649803735408460</stp>
         <tr r="F117" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2051895516</v>
+        <v>#N/A Requesting Data...4212709728</v>
         <stp/>
         <stp>BDP|9873235984695079585</stp>
         <tr r="C60" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2154915284</v>
+        <v>#N/A Requesting Data...4288400313</v>
         <stp/>
         <stp>BDP|4726106605717010168</stp>
         <tr r="G46" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3258907437</v>
+        <v>#N/A Requesting Data...4290886109</v>
         <stp/>
         <stp>BDP|97453184744598227</stp>
         <tr r="G135" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1115661231</v>
+        <v>#N/A Requesting Data...4212183168</v>
         <stp/>
         <stp>BDP|71129432364790944</stp>
         <tr r="E105" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2301437588</v>
+        <v>#N/A Requesting Data...4245874779</v>
         <stp/>
         <stp>BDP|13870968378316918</stp>
         <tr r="F38" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1554907126</v>
+        <v>#N/A Requesting Data...4205410673</v>
         <stp/>
         <stp>BDP|545017254499479967</stp>
         <tr r="E23" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3686684491</v>
+        <v>#N/A Requesting Data...4255000964</v>
         <stp/>
         <stp>BDP|562457211792430265</stp>
         <tr r="G116" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2654882844</v>
+        <v>#N/A Requesting Data...4203658923</v>
         <stp/>
         <stp>BDP|752318736222262646</stp>
         <tr r="F83" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1898584463</v>
+        <v>#N/A Requesting Data...4284897895</v>
         <stp/>
         <stp>BDP|926433161397617222</stp>
         <tr r="F10" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2696222718</v>
+        <v>#N/A Requesting Data...4259669451</v>
         <stp/>
         <stp>BDP|455507803480864317</stp>
         <tr r="C51" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2161484984</v>
+        <v>#N/A Requesting Data...4213274624</v>
         <stp/>
         <stp>BDP|738430784972633891</stp>
         <tr r="F41" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3341530035</v>
+        <v>#N/A Requesting Data...4228508779</v>
         <stp/>
         <stp>BDP|226270545351892196</stp>
         <tr r="F61" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2051949616</v>
+        <v>#N/A Requesting Data...4224948932</v>
         <stp/>
         <stp>BDP|478534605105814154</stp>
         <tr r="G12" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1980328135</v>
+        <v>#N/A Requesting Data...4209863395</v>
         <stp/>
         <stp>BDP|292697057297288557</stp>
         <tr r="C106" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1021928372</v>
+        <v>#N/A Requesting Data...4287706742</v>
         <stp/>
         <stp>BDP|449489448517477649</stp>
         <tr r="E99" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2391817801</v>
+        <v>#N/A Requesting Data...4184689303</v>
         <stp/>
         <stp>BDP|477239144286521179</stp>
         <tr r="G138" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3534648721</v>
+        <v>#N/A Requesting Data...4265381459</v>
         <stp/>
         <stp>BDP|136361134742057301</stp>
         <tr r="C57" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1086730295</v>
+        <v>#N/A Requesting Data...4255131128</v>
         <stp/>
         <stp>BDP|282958180978155995</stp>
         <tr r="C59" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2903784918</v>
+        <v>#N/A Requesting Data...4293150151</v>
         <stp/>
         <stp>BDP|991366924295531418</stp>
         <tr r="F2" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1884815789</v>
+        <v>#N/A Requesting Data...4234564752</v>
         <stp/>
         <stp>BDP|934073235795196633</stp>
         <tr r="F62" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2563791705</v>
+        <v>#N/A Requesting Data...4235808200</v>
         <stp/>
         <stp>BDP|266608211912165570</stp>
         <tr r="E113" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3057108061</v>
+        <v>#N/A Requesting Data...4219185867</v>
         <stp/>
         <stp>BDP|910156400954699593</stp>
         <tr r="G8" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...949952724</v>
+        <v>#N/A Requesting Data...4202577906</v>
         <stp/>
         <stp>BDP|794293317440269040</stp>
         <tr r="E100" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3688105301</v>
+        <v>#N/A Requesting Data...4247404564</v>
         <stp/>
         <stp>BDP|206766873121157269</stp>
         <tr r="E41" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2368675557</v>
+        <v>#N/A Requesting Data...4208626049</v>
         <stp/>
         <stp>BDP|315261912951356153</stp>
         <tr r="E21" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3793664019</v>
+        <v>#N/A Requesting Data...4205044752</v>
         <stp/>
         <stp>BDP|169080827246056602</stp>
         <tr r="G126" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3089408073</v>
+        <v>#N/A Requesting Data...4222925825</v>
         <stp/>
         <stp>BDP|454779781439338455</stp>
         <tr r="E36" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1188566924</v>
+        <v>#N/A Requesting Data...4254096581</v>
         <stp/>
         <stp>BDP|198524097739196711</stp>
         <tr r="F92" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1173514560</v>
+        <v>#N/A Requesting Data...4229314266</v>
         <stp/>
         <stp>BDP|618726407191106421</stp>
         <tr r="C92" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...820464992</v>
+        <v>#N/A Requesting Data...4211825374</v>
         <stp/>
         <stp>BDP|442808307356626303</stp>
         <tr r="F20" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4256063393</v>
+        <v>#N/A Requesting Data...4249940261</v>
         <stp/>
         <stp>BDP|624014897144495064</stp>
         <tr r="G140" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1783031425</v>
+        <v>#N/A Requesting Data...4230282101</v>
         <stp/>
         <stp>BDP|304889655090792147</stp>
         <tr r="E58" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2527661743</v>
+        <v>#N/A Requesting Data...4228418610</v>
         <stp/>
         <stp>BDP|427627592191043219</stp>
         <tr r="C87" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1418598446</v>
+        <v>#N/A Requesting Data...4227339527</v>
         <stp/>
         <stp>BDP|768711067038142524</stp>
         <tr r="G25" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...3788159422</v>
+        <v>#N/A Requesting Data...4289727508</v>
         <stp/>
         <stp>BDP|447365482187669383</stp>
         <tr r="C95" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4140118475</v>
+        <v>#N/A Requesting Data...4219311770</v>
         <stp/>
         <stp>BDP|901925773788783965</stp>
         <tr r="G67" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...772544483</v>
+        <v>#N/A Requesting Data...4236109299</v>
         <stp/>
         <stp>BDP|511429594874391764</stp>
         <tr r="G117" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4182151723</v>
+        <v>#N/A Requesting Data...4267340704</v>
         <stp/>
         <stp>BDP|544620567958067604</stp>
         <tr r="C131" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1235115029</v>
+        <v>#N/A Requesting Data...4273310261</v>
         <stp/>
         <stp>BDP|945569483354328027</stp>
         <tr r="C21" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...4280471265</v>
+        <v>#N/A Requesting Data...4236175994</v>
         <stp/>
         <stp>BDP|691281527639744142</stp>
         <tr r="E8" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...1832172342</v>
+        <v>#N/A Requesting Data...4284109869</v>
         <stp/>
         <stp>BDP|968314719543295935</stp>
         <tr r="E68" s="1"/>
       </tp>
       <tp t="s">
-        <v>#N/A Requesting Data...2064194954</v>
+        <v>#N/A Requesting Data...4233396207</v>
         <stp/>
         <stp>BDP|760426044168153386</stp>
         <tr r="G7" s="1"/>
@@ -4769,7 +4770,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E140"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -4838,7 +4839,7 @@
         <v>305</v>
       </c>
       <c r="E4" t="s">
-        <v>305</v>
+        <v>286</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -4985,10 +4986,10 @@
         <v>227</v>
       </c>
       <c r="C13" t="s">
-        <v>301</v>
+        <v>315</v>
       </c>
       <c r="D13" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="E13" t="s">
         <v>316</v>
@@ -5036,7 +5037,7 @@
         <v>6</v>
       </c>
       <c r="C16" t="s">
-        <v>304</v>
+        <v>287</v>
       </c>
       <c r="D16" t="s">
         <v>305</v>
@@ -5603,7 +5604,7 @@
         <v>286</v>
       </c>
       <c r="E49" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
@@ -6045,7 +6046,7 @@
         <v>313</v>
       </c>
       <c r="E75" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.3">
@@ -6266,7 +6267,7 @@
         <v>305</v>
       </c>
       <c r="E88" t="s">
-        <v>288</v>
+        <v>327</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.3">
@@ -6365,7 +6366,7 @@
         <v>285</v>
       </c>
       <c r="D94" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
       <c r="E94" t="s">
         <v>298</v>
@@ -6722,7 +6723,7 @@
         <v>307</v>
       </c>
       <c r="D115" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="E115" t="s">
         <v>314</v>
@@ -7159,7 +7160,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G140"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7269,7 +7270,7 @@
       </c>
       <c r="G4" t="str">
         <f>_xll.BDP(D4,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
-        <v>CCC+u</v>
+        <v>B-u</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -7504,11 +7505,11 @@
       </c>
       <c r="E13" t="str">
         <f>_xll.BDP(D13,"RTG_MDY_FC_CURR_ISSUER_RATING")</f>
-        <v>Aa3</v>
+        <v>A1</v>
       </c>
       <c r="F13" t="str">
         <f>_xll.BDP(D13,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>AAu</v>
+        <v>AA-u</v>
       </c>
       <c r="G13" t="str">
         <f>_xll.BDP(D13,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
@@ -7585,7 +7586,7 @@
       </c>
       <c r="E16" t="str">
         <f>_xll.BDP(D16,"RTG_MDY_FC_CURR_ISSUER_RATING")</f>
-        <v>Ca</v>
+        <v>Caa3</v>
       </c>
       <c r="F16" t="str">
         <f>_xll.BDP(D16,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
@@ -8484,7 +8485,7 @@
       </c>
       <c r="G49" t="str">
         <f>_xll.BDP(D49,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
-        <v>B-</v>
+        <v>B</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
@@ -9186,7 +9187,7 @@
       </c>
       <c r="G75" t="str">
         <f>_xll.BDP(D75,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
-        <v>A</v>
+        <v>A+</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
@@ -9537,7 +9538,7 @@
       </c>
       <c r="G88" t="str">
         <f>_xll.BDP(D88,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
-        <v>CCCu</v>
+        <v>CCu</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.3">
@@ -9695,7 +9696,7 @@
       </c>
       <c r="F94" t="str">
         <f>_xll.BDP(D94,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>B-</v>
+        <v>B</v>
       </c>
       <c r="G94" t="str">
         <f>_xll.BDP(D94,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>
@@ -10262,7 +10263,7 @@
       </c>
       <c r="F115" t="str">
         <f>_xll.BDP(D115,"RTG_SP_LT_FC_ISSUER_CREDIT")</f>
-        <v>A+</v>
+        <v>A</v>
       </c>
       <c r="G115" t="str">
         <f>_xll.BDP(D115,"RTG_FITCH_LT_ISSUER_DEFAULT")</f>

</xml_diff>